<commit_message>
Remove unused rows in enums sheet
</commit_message>
<xml_diff>
--- a/data/mapping_config_files/NWSS-to-ODM-dictionary.xlsx
+++ b/data/mapping_config_files/NWSS-to-ODM-dictionary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-MapGenerator/PHES-ODM-MapGenerator/data/mapping_config_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F473A2CA-C820-0046-94BE-355E30642FD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A1816F2-5BAC-5D45-A7BD-F675F4EBA2A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="280" yWindow="500" windowWidth="39840" windowHeight="19600" activeTab="2" xr2:uid="{77810E24-F86B-BC44-A0D5-8790E6EC60B4}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2590" uniqueCount="769">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2507" uniqueCount="766">
   <si>
     <t>Reporter</t>
   </si>
@@ -2156,9 +2156,6 @@
     <t>customData</t>
   </si>
   <si>
-    <t>---</t>
-  </si>
-  <si>
     <t>collPer</t>
   </si>
   <si>
@@ -2208,12 +2205,6 @@
   </si>
   <si>
     <t>targetEnum</t>
-  </si>
-  <si>
-    <t>shedSet</t>
-  </si>
-  <si>
-    <t>other?</t>
   </si>
   <si>
     <t>Same targets: reporting_jurisdiction, wwtp_jurisdiction</t>
@@ -2478,7 +2469,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -2523,11 +2514,48 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thick">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thick">
+        <color auto="1"/>
+      </top>
+      <bottom style="thick">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thick">
+        <color auto="1"/>
+      </top>
+      <bottom style="thick">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color auto="1"/>
+      </right>
+      <top style="thick">
+        <color auto="1"/>
+      </top>
+      <bottom style="thick">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -2560,13 +2588,16 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -13838,8 +13869,8 @@
     <col min="12" max="12" width="47.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="20" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:12" s="24" customFormat="1" ht="20" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="24" t="s">
         <v>700</v>
       </c>
       <c r="B1" s="8" t="s">
@@ -13896,7 +13927,7 @@
         <v>121</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>741</v>
+        <v>738</v>
       </c>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
@@ -13904,7 +13935,7 @@
         <v>490</v>
       </c>
       <c r="L2" s="19" t="s">
-        <v>723</v>
+        <v>720</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
@@ -13930,7 +13961,7 @@
         <v>82</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>742</v>
+        <v>739</v>
       </c>
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
@@ -13959,7 +13990,7 @@
         <v>127</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>743</v>
+        <v>740</v>
       </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
@@ -13990,7 +14021,7 @@
         <v>84</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>744</v>
+        <v>741</v>
       </c>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
@@ -14019,7 +14050,7 @@
         <v>85</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>745</v>
+        <v>742</v>
       </c>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
@@ -14121,8 +14152,8 @@
       <c r="I10" s="6"/>
       <c r="J10" s="6"/>
       <c r="K10" s="2"/>
-      <c r="L10" s="23" t="s">
-        <v>757</v>
+      <c r="L10" s="22" t="s">
+        <v>754</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.2">
@@ -14136,7 +14167,7 @@
       <c r="I11" s="6"/>
       <c r="J11" s="6"/>
       <c r="K11" s="2"/>
-      <c r="L11" s="24"/>
+      <c r="L11" s="23"/>
     </row>
     <row r="12" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" t="b">
@@ -14643,7 +14674,7 @@
         <v>123</v>
       </c>
       <c r="L29" s="19" t="s">
-        <v>724</v>
+        <v>721</v>
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.2">
@@ -14696,7 +14727,7 @@
         <v>122</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>746</v>
+        <v>743</v>
       </c>
       <c r="I31" s="2"/>
       <c r="J31" s="2"/>
@@ -14723,7 +14754,7 @@
         <v>121</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>747</v>
+        <v>744</v>
       </c>
       <c r="I32" s="2"/>
       <c r="J32" s="2"/>
@@ -14739,19 +14770,17 @@
       <c r="C33" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="D33" s="2" t="s">
-        <v>703</v>
-      </c>
+      <c r="D33" s="2"/>
       <c r="E33" s="2"/>
       <c r="F33" s="2" t="s">
         <v>124</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="H33" s="6"/>
-      <c r="I33" s="21" t="s">
-        <v>739</v>
+      <c r="I33" s="20" t="s">
+        <v>736</v>
       </c>
       <c r="J33" s="2"/>
       <c r="K33" s="2"/>
@@ -14766,9 +14795,7 @@
       <c r="C34" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="D34" s="22" t="s">
-        <v>703</v>
-      </c>
+      <c r="D34" s="21"/>
       <c r="E34" s="3"/>
       <c r="F34" s="2" t="s">
         <v>124</v>
@@ -14777,8 +14804,8 @@
         <v>125</v>
       </c>
       <c r="H34" s="2"/>
-      <c r="I34" s="21" t="s">
-        <v>740</v>
+      <c r="I34" s="20" t="s">
+        <v>737</v>
       </c>
       <c r="J34" s="2"/>
       <c r="K34" s="2"/>
@@ -14806,7 +14833,7 @@
         <v>126</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>748</v>
+        <v>745</v>
       </c>
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
@@ -15089,13 +15116,13 @@
         <v>160</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>749</v>
+        <v>746</v>
       </c>
       <c r="I46" s="2"/>
       <c r="J46" s="2"/>
       <c r="K46" s="2"/>
       <c r="L46" s="19" t="s">
-        <v>758</v>
+        <v>755</v>
       </c>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.2">
@@ -15119,7 +15146,7 @@
         <v>160</v>
       </c>
       <c r="H47" s="2" t="s">
-        <v>750</v>
+        <v>747</v>
       </c>
       <c r="I47" s="2"/>
       <c r="J47" s="2"/>
@@ -15127,7 +15154,7 @@
         <v>596</v>
       </c>
       <c r="L47" s="19" t="s">
-        <v>760</v>
+        <v>757</v>
       </c>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.2">
@@ -15151,13 +15178,13 @@
         <v>160</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>751</v>
+        <v>748</v>
       </c>
       <c r="I48" s="2"/>
       <c r="J48" s="2"/>
       <c r="K48" s="2"/>
-      <c r="L48" s="23" t="s">
-        <v>759</v>
+      <c r="L48" s="22" t="s">
+        <v>756</v>
       </c>
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.2">
@@ -15171,7 +15198,7 @@
       <c r="I49" s="2"/>
       <c r="J49" s="2"/>
       <c r="K49" s="2"/>
-      <c r="L49" s="23"/>
+      <c r="L49" s="22"/>
     </row>
     <row r="50" spans="1:12" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" t="b">
@@ -15183,7 +15210,7 @@
       <c r="C50" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="D50" s="22" t="s">
+      <c r="D50" s="21" t="s">
         <v>49</v>
       </c>
       <c r="E50" s="2" t="s">
@@ -15295,7 +15322,7 @@
         <v>146</v>
       </c>
       <c r="H54" s="2" t="s">
-        <v>752</v>
+        <v>749</v>
       </c>
       <c r="I54" s="2"/>
       <c r="J54" s="2"/>
@@ -15324,7 +15351,7 @@
         <v>150</v>
       </c>
       <c r="H55" s="2" t="s">
-        <v>753</v>
+        <v>750</v>
       </c>
       <c r="I55" s="2"/>
       <c r="J55" s="2"/>
@@ -15373,7 +15400,7 @@
         <v>157</v>
       </c>
       <c r="L57" s="19" t="s">
-        <v>717</v>
+        <v>716</v>
       </c>
     </row>
     <row r="58" spans="1:12" x14ac:dyDescent="0.2">
@@ -15460,9 +15487,7 @@
       <c r="C61" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="D61" s="2" t="s">
-        <v>61</v>
-      </c>
+      <c r="D61" s="2"/>
       <c r="E61" s="2" t="s">
         <v>147</v>
       </c>
@@ -15474,7 +15499,7 @@
       </c>
       <c r="H61" s="2"/>
       <c r="I61" s="2" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="J61" s="2"/>
       <c r="K61" s="1" t="s">
@@ -15683,7 +15708,7 @@
         <v>169</v>
       </c>
       <c r="H69" s="2" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="I69" s="2"/>
       <c r="J69" s="2"/>
@@ -15905,7 +15930,7 @@
         <v>621</v>
       </c>
       <c r="L78" s="19" t="s">
-        <v>718</v>
+        <v>717</v>
       </c>
     </row>
     <row r="79" spans="1:12" x14ac:dyDescent="0.2">
@@ -16213,7 +16238,7 @@
         <v>486</v>
       </c>
       <c r="H90" s="2" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
       <c r="I90" s="2"/>
       <c r="J90" s="2"/>
@@ -16240,13 +16265,13 @@
         <v>488</v>
       </c>
       <c r="H91" s="2" t="s">
-        <v>756</v>
+        <v>753</v>
       </c>
       <c r="I91" s="2"/>
       <c r="J91" s="2"/>
       <c r="K91" s="2"/>
-      <c r="L91" s="23" t="s">
-        <v>762</v>
+      <c r="L91" s="22" t="s">
+        <v>759</v>
       </c>
     </row>
   </sheetData>
@@ -16275,11 +16300,11 @@
     <col min="14" max="14" width="27.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="20" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:14" s="24" customFormat="1" ht="20" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="24" t="s">
         <v>700</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="8" t="s">
         <v>695</v>
       </c>
       <c r="C1" s="9" t="s">
@@ -16288,14 +16313,14 @@
       <c r="D1" s="9" t="s">
         <v>697</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="E1" s="9" t="s">
         <v>698</v>
       </c>
       <c r="F1" s="9" t="s">
-        <v>705</v>
+        <v>704</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>725</v>
+        <v>722</v>
       </c>
       <c r="H1" s="11" t="s">
         <v>167</v>
@@ -16565,7 +16590,7 @@
         <v>665</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>726</v>
+        <v>723</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>177</v>
@@ -16632,7 +16657,7 @@
         <v>435</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="L10" s="2" t="s">
         <v>80</v>
@@ -16839,7 +16864,7 @@
         <v>440</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>707</v>
+        <v>706</v>
       </c>
       <c r="L16" s="2" t="s">
         <v>80</v>
@@ -17766,7 +17791,7 @@
         <v>459</v>
       </c>
       <c r="K41" s="2" t="s">
-        <v>708</v>
+        <v>707</v>
       </c>
       <c r="L41" s="2" t="s">
         <v>80</v>
@@ -19280,7 +19305,7 @@
         <v>498</v>
       </c>
       <c r="K82" s="2" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="L82" s="2" t="s">
         <v>80</v>
@@ -19905,7 +19930,7 @@
         <v>499</v>
       </c>
       <c r="K99" s="2" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="L99" s="2" t="s">
         <v>80</v>
@@ -20279,7 +20304,7 @@
         <v>481</v>
       </c>
       <c r="K110" s="2" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="L110" s="2" t="s">
         <v>80</v>
@@ -20558,7 +20583,7 @@
         <v>520</v>
       </c>
       <c r="K118" s="2" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="L118" s="2" t="s">
         <v>80</v>
@@ -20630,7 +20655,7 @@
         <v>665</v>
       </c>
       <c r="K120" s="1" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="L120" s="1"/>
       <c r="M120" s="1"/>
@@ -20664,7 +20689,7 @@
         <v>597</v>
       </c>
       <c r="K121" s="2" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="L121" s="2" t="s">
         <v>185</v>
@@ -20673,7 +20698,7 @@
         <v>171</v>
       </c>
       <c r="N121" s="2" t="s">
-        <v>715</v>
+        <v>714</v>
       </c>
     </row>
     <row r="122" spans="1:14" x14ac:dyDescent="0.2">
@@ -20922,7 +20947,7 @@
         <v>665</v>
       </c>
       <c r="G128" s="2" t="s">
-        <v>727</v>
+        <v>724</v>
       </c>
       <c r="H128" s="2" t="s">
         <v>177</v>
@@ -20943,7 +20968,7 @@
         <v>171</v>
       </c>
       <c r="N128" s="2" t="s">
-        <v>761</v>
+        <v>758</v>
       </c>
     </row>
     <row r="129" spans="1:14" x14ac:dyDescent="0.2">
@@ -21164,7 +21189,7 @@
         <v>665</v>
       </c>
       <c r="G134" s="2" t="s">
-        <v>731</v>
+        <v>728</v>
       </c>
       <c r="H134" s="2" t="s">
         <v>177</v>
@@ -21204,7 +21229,7 @@
         <v>665</v>
       </c>
       <c r="G135" s="2" t="s">
-        <v>733</v>
+        <v>730</v>
       </c>
       <c r="H135" s="2" t="s">
         <v>177</v>
@@ -21244,7 +21269,7 @@
         <v>665</v>
       </c>
       <c r="G136" s="2" t="s">
-        <v>735</v>
+        <v>732</v>
       </c>
       <c r="H136" s="2" t="s">
         <v>177</v>
@@ -21299,7 +21324,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BC10C3F-0C27-5546-8767-E60C7CACEA9D}">
-  <dimension ref="A1:J201"/>
+  <dimension ref="A1:J185"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="13.83203125" bestFit="1" customWidth="1"/>
@@ -21309,419 +21334,389 @@
     <col min="8" max="8" width="12.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="20" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="20" t="s">
+    <row r="1" spans="1:10" s="24" customFormat="1" ht="21" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="24" t="s">
         <v>700</v>
       </c>
-      <c r="B1" s="20" t="s">
+      <c r="B1" s="25" t="s">
         <v>649</v>
       </c>
-      <c r="C1" s="20" t="s">
+      <c r="C1" s="26" t="s">
         <v>651</v>
       </c>
-      <c r="D1" s="20" t="s">
+      <c r="D1" s="26" t="s">
+        <v>718</v>
+      </c>
+      <c r="E1" s="26" t="s">
+        <v>652</v>
+      </c>
+      <c r="F1" s="26" t="s">
+        <v>653</v>
+      </c>
+      <c r="G1" s="26" t="s">
+        <v>654</v>
+      </c>
+      <c r="H1" s="26" t="s">
         <v>719</v>
       </c>
-      <c r="E1" s="20" t="s">
-        <v>652</v>
-      </c>
-      <c r="F1" s="20" t="s">
-        <v>653</v>
-      </c>
-      <c r="G1" s="20" t="s">
-        <v>654</v>
-      </c>
-      <c r="H1" s="20" t="s">
-        <v>720</v>
-      </c>
-      <c r="I1" s="20" t="s">
+      <c r="I1" s="26" t="s">
         <v>655</v>
       </c>
-      <c r="J1" s="20" t="s">
+      <c r="J1" s="27" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2" t="s">
+        <v>725</v>
+      </c>
       <c r="E2" s="2" t="s">
-        <v>89</v>
+        <v>291</v>
       </c>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
-      <c r="H2" s="2" t="s">
-        <v>721</v>
-      </c>
+      <c r="H2" s="21"/>
       <c r="I2" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="J2" s="2"/>
+        <v>521</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>761</v>
+      </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2" t="s">
+        <v>725</v>
+      </c>
       <c r="E3" s="2" t="s">
-        <v>90</v>
+        <v>292</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
-      <c r="H3" s="2" t="s">
-        <v>721</v>
-      </c>
+      <c r="H3" s="2"/>
       <c r="I3" s="2" t="s">
-        <v>106</v>
+        <v>522</v>
       </c>
       <c r="J3" s="2"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2" t="s">
+        <v>725</v>
+      </c>
       <c r="E4" s="2" t="s">
-        <v>91</v>
+        <v>293</v>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
-      <c r="H4" s="2" t="s">
-        <v>721</v>
-      </c>
+      <c r="H4" s="2"/>
       <c r="I4" s="2" t="s">
-        <v>107</v>
+        <v>523</v>
       </c>
       <c r="J4" s="2"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2" t="s">
+        <v>725</v>
+      </c>
       <c r="E5" s="2" t="s">
-        <v>92</v>
+        <v>294</v>
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
-      <c r="H5" s="2" t="s">
-        <v>721</v>
-      </c>
+      <c r="H5" s="2"/>
       <c r="I5" s="2" t="s">
-        <v>108</v>
+        <v>525</v>
       </c>
       <c r="J5" s="2"/>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2" t="s">
+        <v>725</v>
+      </c>
       <c r="E6" s="2" t="s">
-        <v>93</v>
+        <v>295</v>
       </c>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
-      <c r="H6" s="2" t="s">
-        <v>721</v>
-      </c>
+      <c r="H6" s="2"/>
       <c r="I6" s="2" t="s">
-        <v>109</v>
+        <v>524</v>
       </c>
       <c r="J6" s="2"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2" t="s">
+        <v>725</v>
+      </c>
       <c r="E7" s="2" t="s">
-        <v>94</v>
+        <v>296</v>
       </c>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
-      <c r="H7" s="2" t="s">
-        <v>721</v>
-      </c>
+      <c r="H7" s="2"/>
       <c r="I7" s="2" t="s">
-        <v>118</v>
+        <v>528</v>
       </c>
       <c r="J7" s="2"/>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D8" s="2"/>
+      <c r="C8" s="2"/>
+      <c r="D8" s="2" t="s">
+        <v>725</v>
+      </c>
       <c r="E8" s="2" t="s">
-        <v>95</v>
+        <v>297</v>
       </c>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
-      <c r="H8" s="2" t="s">
-        <v>721</v>
-      </c>
+      <c r="H8" s="2"/>
       <c r="I8" s="2" t="s">
-        <v>117</v>
+        <v>529</v>
       </c>
       <c r="J8" s="2"/>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2" t="s">
+        <v>725</v>
+      </c>
       <c r="E9" s="2" t="s">
-        <v>96</v>
+        <v>298</v>
       </c>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
-      <c r="H9" s="2" t="s">
-        <v>721</v>
-      </c>
+      <c r="H9" s="2"/>
       <c r="I9" s="2" t="s">
-        <v>114</v>
+        <v>526</v>
       </c>
       <c r="J9" s="2"/>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D10" s="2"/>
+      <c r="C10" s="2"/>
+      <c r="D10" s="2" t="s">
+        <v>725</v>
+      </c>
       <c r="E10" s="2" t="s">
-        <v>97</v>
+        <v>299</v>
       </c>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
-      <c r="H10" s="2" t="s">
-        <v>721</v>
-      </c>
+      <c r="H10" s="2"/>
       <c r="I10" s="2" t="s">
-        <v>113</v>
+        <v>527</v>
       </c>
       <c r="J10" s="2"/>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2" t="s">
+        <v>725</v>
+      </c>
       <c r="E11" s="2" t="s">
-        <v>98</v>
+        <v>300</v>
       </c>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
-      <c r="H11" s="2" t="s">
-        <v>721</v>
-      </c>
+      <c r="H11" s="2"/>
       <c r="I11" s="2" t="s">
-        <v>112</v>
+        <v>530</v>
       </c>
       <c r="J11" s="2"/>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D12" s="2"/>
+      <c r="C12" s="2"/>
+      <c r="D12" s="2" t="s">
+        <v>725</v>
+      </c>
       <c r="E12" s="2" t="s">
-        <v>99</v>
+        <v>301</v>
       </c>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
-      <c r="H12" s="2" t="s">
-        <v>721</v>
-      </c>
+      <c r="H12" s="2"/>
       <c r="I12" s="2" t="s">
-        <v>111</v>
+        <v>531</v>
       </c>
       <c r="J12" s="2"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D13" s="2"/>
+      <c r="C13" s="2"/>
+      <c r="D13" s="2" t="s">
+        <v>725</v>
+      </c>
       <c r="E13" s="2" t="s">
-        <v>100</v>
+        <v>302</v>
       </c>
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
-      <c r="H13" s="2" t="s">
-        <v>721</v>
-      </c>
+      <c r="H13" s="2"/>
       <c r="I13" s="2" t="s">
-        <v>110</v>
+        <v>302</v>
       </c>
       <c r="J13" s="2"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D14" s="2"/>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2" t="s">
+        <v>725</v>
+      </c>
       <c r="E14" s="2" t="s">
-        <v>101</v>
+        <v>303</v>
       </c>
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
-      <c r="H14" s="2" t="s">
-        <v>721</v>
-      </c>
+      <c r="H14" s="2"/>
       <c r="I14" s="2" t="s">
-        <v>115</v>
+        <v>303</v>
       </c>
       <c r="J14" s="2"/>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="C15" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2" t="s">
+        <v>725</v>
+      </c>
       <c r="E15" s="2" t="s">
-        <v>102</v>
+        <v>304</v>
       </c>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
-      <c r="H15" s="2" t="s">
-        <v>721</v>
-      </c>
+      <c r="H15" s="2"/>
       <c r="I15" s="2" t="s">
-        <v>102</v>
+        <v>532</v>
       </c>
       <c r="J15" s="2"/>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2" t="s">
+        <v>725</v>
+      </c>
       <c r="E16" s="2" t="s">
-        <v>103</v>
+        <v>305</v>
       </c>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
-      <c r="H16" s="2" t="s">
-        <v>721</v>
-      </c>
+      <c r="H16" s="2"/>
       <c r="I16" s="2" t="s">
-        <v>116</v>
+        <v>305</v>
       </c>
       <c r="J16" s="2"/>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="C17" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2" t="s">
+        <v>725</v>
+      </c>
       <c r="E17" s="2" t="s">
-        <v>104</v>
+        <v>306</v>
       </c>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
-      <c r="H17" s="2" t="s">
-        <v>721</v>
-      </c>
+      <c r="H17" s="2"/>
       <c r="I17" s="2" t="s">
-        <v>722</v>
+        <v>533</v>
       </c>
       <c r="J17" s="2"/>
     </row>
@@ -21734,20 +21729,18 @@
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>291</v>
+        <v>307</v>
       </c>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
-      <c r="H18" s="22"/>
+      <c r="H18" s="2"/>
       <c r="I18" s="2" t="s">
-        <v>521</v>
-      </c>
-      <c r="J18" s="2" t="s">
-        <v>764</v>
-      </c>
+        <v>307</v>
+      </c>
+      <c r="J18" s="2"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" t="b">
@@ -21758,16 +21751,16 @@
       </c>
       <c r="C19" s="2"/>
       <c r="D19" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>292</v>
+        <v>308</v>
       </c>
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
       <c r="I19" s="2" t="s">
-        <v>522</v>
+        <v>534</v>
       </c>
       <c r="J19" s="2"/>
     </row>
@@ -21780,16 +21773,16 @@
       </c>
       <c r="C20" s="2"/>
       <c r="D20" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>293</v>
+        <v>309</v>
       </c>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
       <c r="I20" s="2" t="s">
-        <v>523</v>
+        <v>535</v>
       </c>
       <c r="J20" s="2"/>
     </row>
@@ -21802,16 +21795,16 @@
       </c>
       <c r="C21" s="2"/>
       <c r="D21" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>294</v>
+        <v>310</v>
       </c>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
       <c r="I21" s="2" t="s">
-        <v>525</v>
+        <v>536</v>
       </c>
       <c r="J21" s="2"/>
     </row>
@@ -21824,16 +21817,16 @@
       </c>
       <c r="C22" s="2"/>
       <c r="D22" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>295</v>
+        <v>311</v>
       </c>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
       <c r="I22" s="2" t="s">
-        <v>524</v>
+        <v>521</v>
       </c>
       <c r="J22" s="2"/>
     </row>
@@ -21846,16 +21839,16 @@
       </c>
       <c r="C23" s="2"/>
       <c r="D23" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>296</v>
+        <v>312</v>
       </c>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
       <c r="I23" s="2" t="s">
-        <v>528</v>
+        <v>522</v>
       </c>
       <c r="J23" s="2"/>
     </row>
@@ -21868,16 +21861,16 @@
       </c>
       <c r="C24" s="2"/>
       <c r="D24" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>297</v>
+        <v>313</v>
       </c>
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2" t="s">
-        <v>529</v>
+        <v>522</v>
       </c>
       <c r="J24" s="2"/>
     </row>
@@ -21890,16 +21883,16 @@
       </c>
       <c r="C25" s="2"/>
       <c r="D25" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>298</v>
+        <v>314</v>
       </c>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
       <c r="I25" s="2" t="s">
-        <v>526</v>
+        <v>535</v>
       </c>
       <c r="J25" s="2"/>
     </row>
@@ -21912,16 +21905,16 @@
       </c>
       <c r="C26" s="2"/>
       <c r="D26" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>299</v>
+        <v>315</v>
       </c>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
       <c r="I26" s="2" t="s">
-        <v>527</v>
+        <v>315</v>
       </c>
       <c r="J26" s="2"/>
     </row>
@@ -21934,16 +21927,16 @@
       </c>
       <c r="C27" s="2"/>
       <c r="D27" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>300</v>
+        <v>322</v>
       </c>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
       <c r="I27" s="2" t="s">
-        <v>530</v>
+        <v>322</v>
       </c>
       <c r="J27" s="2"/>
     </row>
@@ -21956,16 +21949,16 @@
       </c>
       <c r="C28" s="2"/>
       <c r="D28" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>301</v>
+        <v>339</v>
       </c>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
       <c r="I28" s="2" t="s">
-        <v>531</v>
+        <v>537</v>
       </c>
       <c r="J28" s="2"/>
     </row>
@@ -21978,16 +21971,16 @@
       </c>
       <c r="C29" s="2"/>
       <c r="D29" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>302</v>
+        <v>370</v>
       </c>
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
       <c r="I29" s="2" t="s">
-        <v>302</v>
+        <v>538</v>
       </c>
       <c r="J29" s="2"/>
     </row>
@@ -22000,16 +21993,16 @@
       </c>
       <c r="C30" s="2"/>
       <c r="D30" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>303</v>
+        <v>344</v>
       </c>
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
       <c r="I30" s="2" t="s">
-        <v>303</v>
+        <v>539</v>
       </c>
       <c r="J30" s="2"/>
     </row>
@@ -22022,16 +22015,16 @@
       </c>
       <c r="C31" s="2"/>
       <c r="D31" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>304</v>
+        <v>346</v>
       </c>
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
       <c r="I31" s="2" t="s">
-        <v>532</v>
+        <v>590</v>
       </c>
       <c r="J31" s="2"/>
     </row>
@@ -22044,16 +22037,16 @@
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>305</v>
+        <v>333</v>
       </c>
       <c r="F32" s="2"/>
       <c r="G32" s="2"/>
       <c r="H32" s="2"/>
       <c r="I32" s="2" t="s">
-        <v>305</v>
+        <v>333</v>
       </c>
       <c r="J32" s="2"/>
     </row>
@@ -22066,16 +22059,16 @@
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>306</v>
+        <v>368</v>
       </c>
       <c r="F33" s="2"/>
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
       <c r="I33" s="2" t="s">
-        <v>533</v>
+        <v>368</v>
       </c>
       <c r="J33" s="2"/>
     </row>
@@ -22088,16 +22081,16 @@
       </c>
       <c r="C34" s="2"/>
       <c r="D34" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>307</v>
+        <v>330</v>
       </c>
       <c r="F34" s="2"/>
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
       <c r="I34" s="2" t="s">
-        <v>307</v>
+        <v>330</v>
       </c>
       <c r="J34" s="2"/>
     </row>
@@ -22110,16 +22103,16 @@
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>308</v>
+        <v>362</v>
       </c>
       <c r="F35" s="2"/>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
       <c r="I35" s="2" t="s">
-        <v>534</v>
+        <v>362</v>
       </c>
       <c r="J35" s="2"/>
     </row>
@@ -22132,16 +22125,16 @@
       </c>
       <c r="C36" s="2"/>
       <c r="D36" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>309</v>
+        <v>328</v>
       </c>
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
       <c r="I36" s="2" t="s">
-        <v>535</v>
+        <v>328</v>
       </c>
       <c r="J36" s="2"/>
     </row>
@@ -22154,16 +22147,16 @@
       </c>
       <c r="C37" s="2"/>
       <c r="D37" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>310</v>
+        <v>325</v>
       </c>
       <c r="F37" s="2"/>
       <c r="G37" s="2"/>
       <c r="H37" s="2"/>
       <c r="I37" s="2" t="s">
-        <v>536</v>
+        <v>540</v>
       </c>
       <c r="J37" s="2"/>
     </row>
@@ -22176,16 +22169,16 @@
       </c>
       <c r="C38" s="2"/>
       <c r="D38" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>311</v>
+        <v>372</v>
       </c>
       <c r="F38" s="2"/>
       <c r="G38" s="2"/>
       <c r="H38" s="2"/>
       <c r="I38" s="2" t="s">
-        <v>521</v>
+        <v>567</v>
       </c>
       <c r="J38" s="2"/>
     </row>
@@ -22198,16 +22191,16 @@
       </c>
       <c r="C39" s="2"/>
       <c r="D39" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>312</v>
+        <v>347</v>
       </c>
       <c r="F39" s="2"/>
       <c r="G39" s="2"/>
       <c r="H39" s="2"/>
       <c r="I39" s="2" t="s">
-        <v>522</v>
+        <v>541</v>
       </c>
       <c r="J39" s="2"/>
     </row>
@@ -22220,16 +22213,16 @@
       </c>
       <c r="C40" s="2"/>
       <c r="D40" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>313</v>
+        <v>335</v>
       </c>
       <c r="F40" s="2"/>
       <c r="G40" s="2"/>
       <c r="H40" s="2"/>
       <c r="I40" s="2" t="s">
-        <v>522</v>
+        <v>568</v>
       </c>
       <c r="J40" s="2"/>
     </row>
@@ -22242,16 +22235,16 @@
       </c>
       <c r="C41" s="2"/>
       <c r="D41" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>314</v>
+        <v>338</v>
       </c>
       <c r="F41" s="2"/>
       <c r="G41" s="2"/>
       <c r="H41" s="2"/>
       <c r="I41" s="2" t="s">
-        <v>535</v>
+        <v>542</v>
       </c>
       <c r="J41" s="2"/>
     </row>
@@ -22264,16 +22257,16 @@
       </c>
       <c r="C42" s="2"/>
       <c r="D42" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>315</v>
+        <v>349</v>
       </c>
       <c r="F42" s="2"/>
       <c r="G42" s="2"/>
       <c r="H42" s="2"/>
       <c r="I42" s="2" t="s">
-        <v>315</v>
+        <v>543</v>
       </c>
       <c r="J42" s="2"/>
     </row>
@@ -22286,16 +22279,16 @@
       </c>
       <c r="C43" s="2"/>
       <c r="D43" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>322</v>
+        <v>373</v>
       </c>
       <c r="F43" s="2"/>
       <c r="G43" s="2"/>
       <c r="H43" s="2"/>
       <c r="I43" s="2" t="s">
-        <v>322</v>
+        <v>569</v>
       </c>
       <c r="J43" s="2"/>
     </row>
@@ -22308,16 +22301,16 @@
       </c>
       <c r="C44" s="2"/>
       <c r="D44" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="F44" s="2"/>
       <c r="G44" s="2"/>
       <c r="H44" s="2"/>
       <c r="I44" s="2" t="s">
-        <v>537</v>
+        <v>544</v>
       </c>
       <c r="J44" s="2"/>
     </row>
@@ -22330,16 +22323,16 @@
       </c>
       <c r="C45" s="2"/>
       <c r="D45" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>370</v>
+        <v>345</v>
       </c>
       <c r="F45" s="2"/>
       <c r="G45" s="2"/>
       <c r="H45" s="2"/>
       <c r="I45" s="2" t="s">
-        <v>538</v>
+        <v>545</v>
       </c>
       <c r="J45" s="2"/>
     </row>
@@ -22352,16 +22345,16 @@
       </c>
       <c r="C46" s="2"/>
       <c r="D46" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>344</v>
+        <v>324</v>
       </c>
       <c r="F46" s="2"/>
       <c r="G46" s="2"/>
       <c r="H46" s="2"/>
       <c r="I46" s="2" t="s">
-        <v>539</v>
+        <v>324</v>
       </c>
       <c r="J46" s="2"/>
     </row>
@@ -22374,16 +22367,16 @@
       </c>
       <c r="C47" s="2"/>
       <c r="D47" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>346</v>
+        <v>355</v>
       </c>
       <c r="F47" s="2"/>
       <c r="G47" s="2"/>
       <c r="H47" s="2"/>
       <c r="I47" s="2" t="s">
-        <v>590</v>
+        <v>355</v>
       </c>
       <c r="J47" s="2"/>
     </row>
@@ -22396,16 +22389,16 @@
       </c>
       <c r="C48" s="2"/>
       <c r="D48" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="F48" s="2"/>
       <c r="G48" s="2"/>
       <c r="H48" s="2"/>
       <c r="I48" s="2" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="J48" s="2"/>
     </row>
@@ -22418,16 +22411,16 @@
       </c>
       <c r="C49" s="2"/>
       <c r="D49" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>368</v>
+        <v>350</v>
       </c>
       <c r="F49" s="2"/>
       <c r="G49" s="2"/>
       <c r="H49" s="2"/>
       <c r="I49" s="2" t="s">
-        <v>368</v>
+        <v>350</v>
       </c>
       <c r="J49" s="2"/>
     </row>
@@ -22440,16 +22433,16 @@
       </c>
       <c r="C50" s="2"/>
       <c r="D50" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>330</v>
+        <v>357</v>
       </c>
       <c r="F50" s="2"/>
       <c r="G50" s="2"/>
       <c r="H50" s="2"/>
       <c r="I50" s="2" t="s">
-        <v>330</v>
+        <v>357</v>
       </c>
       <c r="J50" s="2"/>
     </row>
@@ -22462,16 +22455,16 @@
       </c>
       <c r="C51" s="2"/>
       <c r="D51" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>362</v>
+        <v>320</v>
       </c>
       <c r="F51" s="2"/>
       <c r="G51" s="2"/>
       <c r="H51" s="2"/>
       <c r="I51" s="2" t="s">
-        <v>362</v>
+        <v>320</v>
       </c>
       <c r="J51" s="2"/>
     </row>
@@ -22484,16 +22477,16 @@
       </c>
       <c r="C52" s="2"/>
       <c r="D52" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>328</v>
+        <v>343</v>
       </c>
       <c r="F52" s="2"/>
       <c r="G52" s="2"/>
       <c r="H52" s="2"/>
       <c r="I52" s="2" t="s">
-        <v>328</v>
+        <v>343</v>
       </c>
       <c r="J52" s="2"/>
     </row>
@@ -22506,16 +22499,16 @@
       </c>
       <c r="C53" s="2"/>
       <c r="D53" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>325</v>
+        <v>342</v>
       </c>
       <c r="F53" s="2"/>
       <c r="G53" s="2"/>
       <c r="H53" s="2"/>
       <c r="I53" s="2" t="s">
-        <v>540</v>
+        <v>342</v>
       </c>
       <c r="J53" s="2"/>
     </row>
@@ -22528,16 +22521,16 @@
       </c>
       <c r="C54" s="2"/>
       <c r="D54" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>372</v>
+        <v>329</v>
       </c>
       <c r="F54" s="2"/>
       <c r="G54" s="2"/>
       <c r="H54" s="2"/>
       <c r="I54" s="2" t="s">
-        <v>567</v>
+        <v>329</v>
       </c>
       <c r="J54" s="2"/>
     </row>
@@ -22550,16 +22543,16 @@
       </c>
       <c r="C55" s="2"/>
       <c r="D55" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>347</v>
+        <v>371</v>
       </c>
       <c r="F55" s="2"/>
       <c r="G55" s="2"/>
       <c r="H55" s="2"/>
       <c r="I55" s="2" t="s">
-        <v>541</v>
+        <v>371</v>
       </c>
       <c r="J55" s="2"/>
     </row>
@@ -22572,16 +22565,16 @@
       </c>
       <c r="C56" s="2"/>
       <c r="D56" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="F56" s="2"/>
       <c r="G56" s="2"/>
       <c r="H56" s="2"/>
       <c r="I56" s="2" t="s">
-        <v>568</v>
+        <v>336</v>
       </c>
       <c r="J56" s="2"/>
     </row>
@@ -22594,16 +22587,16 @@
       </c>
       <c r="C57" s="2"/>
       <c r="D57" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>338</v>
+        <v>374</v>
       </c>
       <c r="F57" s="2"/>
       <c r="G57" s="2"/>
       <c r="H57" s="2"/>
       <c r="I57" s="2" t="s">
-        <v>542</v>
+        <v>374</v>
       </c>
       <c r="J57" s="2"/>
     </row>
@@ -22616,16 +22609,16 @@
       </c>
       <c r="C58" s="2"/>
       <c r="D58" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>349</v>
+        <v>326</v>
       </c>
       <c r="F58" s="2"/>
       <c r="G58" s="2"/>
       <c r="H58" s="2"/>
       <c r="I58" s="2" t="s">
-        <v>543</v>
+        <v>326</v>
       </c>
       <c r="J58" s="2"/>
     </row>
@@ -22638,16 +22631,16 @@
       </c>
       <c r="C59" s="2"/>
       <c r="D59" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>373</v>
+        <v>366</v>
       </c>
       <c r="F59" s="2"/>
       <c r="G59" s="2"/>
       <c r="H59" s="2"/>
       <c r="I59" s="2" t="s">
-        <v>569</v>
+        <v>366</v>
       </c>
       <c r="J59" s="2"/>
     </row>
@@ -22660,16 +22653,16 @@
       </c>
       <c r="C60" s="2"/>
       <c r="D60" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>341</v>
+        <v>375</v>
       </c>
       <c r="F60" s="2"/>
       <c r="G60" s="2"/>
       <c r="H60" s="2"/>
       <c r="I60" s="2" t="s">
-        <v>544</v>
+        <v>375</v>
       </c>
       <c r="J60" s="2"/>
     </row>
@@ -22682,16 +22675,16 @@
       </c>
       <c r="C61" s="2"/>
       <c r="D61" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="F61" s="2"/>
       <c r="G61" s="2"/>
       <c r="H61" s="2"/>
       <c r="I61" s="2" t="s">
-        <v>545</v>
+        <v>348</v>
       </c>
       <c r="J61" s="2"/>
     </row>
@@ -22704,16 +22697,16 @@
       </c>
       <c r="C62" s="2"/>
       <c r="D62" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E62" s="2" t="s">
-        <v>324</v>
+        <v>361</v>
       </c>
       <c r="F62" s="2"/>
       <c r="G62" s="2"/>
       <c r="H62" s="2"/>
       <c r="I62" s="2" t="s">
-        <v>324</v>
+        <v>361</v>
       </c>
       <c r="J62" s="2"/>
     </row>
@@ -22726,16 +22719,16 @@
       </c>
       <c r="C63" s="2"/>
       <c r="D63" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E63" s="2" t="s">
-        <v>355</v>
+        <v>363</v>
       </c>
       <c r="F63" s="2"/>
       <c r="G63" s="2"/>
       <c r="H63" s="2"/>
       <c r="I63" s="2" t="s">
-        <v>355</v>
+        <v>363</v>
       </c>
       <c r="J63" s="2"/>
     </row>
@@ -22748,16 +22741,16 @@
       </c>
       <c r="C64" s="2"/>
       <c r="D64" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E64" s="2" t="s">
-        <v>332</v>
+        <v>365</v>
       </c>
       <c r="F64" s="2"/>
       <c r="G64" s="2"/>
       <c r="H64" s="2"/>
       <c r="I64" s="2" t="s">
-        <v>332</v>
+        <v>365</v>
       </c>
       <c r="J64" s="2"/>
     </row>
@@ -22770,16 +22763,16 @@
       </c>
       <c r="C65" s="2"/>
       <c r="D65" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>350</v>
+        <v>321</v>
       </c>
       <c r="F65" s="2"/>
       <c r="G65" s="2"/>
       <c r="H65" s="2"/>
       <c r="I65" s="2" t="s">
-        <v>350</v>
+        <v>321</v>
       </c>
       <c r="J65" s="2"/>
     </row>
@@ -22792,16 +22785,16 @@
       </c>
       <c r="C66" s="2"/>
       <c r="D66" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E66" s="2" t="s">
-        <v>357</v>
+        <v>376</v>
       </c>
       <c r="F66" s="2"/>
       <c r="G66" s="2"/>
       <c r="H66" s="2"/>
       <c r="I66" s="2" t="s">
-        <v>357</v>
+        <v>376</v>
       </c>
       <c r="J66" s="2"/>
     </row>
@@ -22814,16 +22807,16 @@
       </c>
       <c r="C67" s="2"/>
       <c r="D67" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E67" s="2" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="F67" s="2"/>
       <c r="G67" s="2"/>
       <c r="H67" s="2"/>
       <c r="I67" s="2" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="J67" s="2"/>
     </row>
@@ -22836,16 +22829,16 @@
       </c>
       <c r="C68" s="2"/>
       <c r="D68" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E68" s="2" t="s">
-        <v>343</v>
+        <v>317</v>
       </c>
       <c r="F68" s="2"/>
       <c r="G68" s="2"/>
       <c r="H68" s="2"/>
       <c r="I68" s="2" t="s">
-        <v>343</v>
+        <v>317</v>
       </c>
       <c r="J68" s="2"/>
     </row>
@@ -22858,16 +22851,16 @@
       </c>
       <c r="C69" s="2"/>
       <c r="D69" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="F69" s="2"/>
       <c r="G69" s="2"/>
       <c r="H69" s="2"/>
       <c r="I69" s="2" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="J69" s="2"/>
     </row>
@@ -22880,16 +22873,16 @@
       </c>
       <c r="C70" s="2"/>
       <c r="D70" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="F70" s="2"/>
       <c r="G70" s="2"/>
       <c r="H70" s="2"/>
       <c r="I70" s="2" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="J70" s="2"/>
     </row>
@@ -22902,16 +22895,16 @@
       </c>
       <c r="C71" s="2"/>
       <c r="D71" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="F71" s="2"/>
       <c r="G71" s="2"/>
       <c r="H71" s="2"/>
       <c r="I71" s="2" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="J71" s="2"/>
     </row>
@@ -22924,16 +22917,16 @@
       </c>
       <c r="C72" s="2"/>
       <c r="D72" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>336</v>
+        <v>356</v>
       </c>
       <c r="F72" s="2"/>
       <c r="G72" s="2"/>
       <c r="H72" s="2"/>
       <c r="I72" s="2" t="s">
-        <v>336</v>
+        <v>356</v>
       </c>
       <c r="J72" s="2"/>
     </row>
@@ -22946,16 +22939,16 @@
       </c>
       <c r="C73" s="2"/>
       <c r="D73" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>374</v>
+        <v>358</v>
       </c>
       <c r="F73" s="2"/>
       <c r="G73" s="2"/>
       <c r="H73" s="2"/>
       <c r="I73" s="2" t="s">
-        <v>374</v>
+        <v>358</v>
       </c>
       <c r="J73" s="2"/>
     </row>
@@ -22968,16 +22961,16 @@
       </c>
       <c r="C74" s="2"/>
       <c r="D74" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E74" s="2" t="s">
-        <v>326</v>
+        <v>364</v>
       </c>
       <c r="F74" s="2"/>
       <c r="G74" s="2"/>
       <c r="H74" s="2"/>
       <c r="I74" s="2" t="s">
-        <v>326</v>
+        <v>364</v>
       </c>
       <c r="J74" s="2"/>
     </row>
@@ -22990,16 +22983,16 @@
       </c>
       <c r="C75" s="2"/>
       <c r="D75" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>366</v>
+        <v>331</v>
       </c>
       <c r="F75" s="2"/>
       <c r="G75" s="2"/>
       <c r="H75" s="2"/>
       <c r="I75" s="2" t="s">
-        <v>366</v>
+        <v>331</v>
       </c>
       <c r="J75" s="2"/>
     </row>
@@ -23012,16 +23005,16 @@
       </c>
       <c r="C76" s="2"/>
       <c r="D76" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>375</v>
+        <v>337</v>
       </c>
       <c r="F76" s="2"/>
       <c r="G76" s="2"/>
       <c r="H76" s="2"/>
       <c r="I76" s="2" t="s">
-        <v>375</v>
+        <v>337</v>
       </c>
       <c r="J76" s="2"/>
     </row>
@@ -23034,16 +23027,16 @@
       </c>
       <c r="C77" s="2"/>
       <c r="D77" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="F77" s="2"/>
       <c r="G77" s="2"/>
       <c r="H77" s="2"/>
       <c r="I77" s="2" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="J77" s="2"/>
     </row>
@@ -23056,16 +23049,16 @@
       </c>
       <c r="C78" s="2"/>
       <c r="D78" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>361</v>
+        <v>352</v>
       </c>
       <c r="F78" s="2"/>
       <c r="G78" s="2"/>
       <c r="H78" s="2"/>
       <c r="I78" s="2" t="s">
-        <v>361</v>
+        <v>352</v>
       </c>
       <c r="J78" s="2"/>
     </row>
@@ -23078,16 +23071,16 @@
       </c>
       <c r="C79" s="2"/>
       <c r="D79" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>363</v>
+        <v>353</v>
       </c>
       <c r="F79" s="2"/>
       <c r="G79" s="2"/>
       <c r="H79" s="2"/>
       <c r="I79" s="2" t="s">
-        <v>363</v>
+        <v>353</v>
       </c>
       <c r="J79" s="2"/>
     </row>
@@ -23100,16 +23093,16 @@
       </c>
       <c r="C80" s="2"/>
       <c r="D80" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>365</v>
+        <v>354</v>
       </c>
       <c r="F80" s="2"/>
       <c r="G80" s="2"/>
       <c r="H80" s="2"/>
       <c r="I80" s="2" t="s">
-        <v>365</v>
+        <v>354</v>
       </c>
       <c r="J80" s="2"/>
     </row>
@@ -23122,16 +23115,16 @@
       </c>
       <c r="C81" s="2"/>
       <c r="D81" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E81" s="2" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="F81" s="2"/>
       <c r="G81" s="2"/>
       <c r="H81" s="2"/>
       <c r="I81" s="2" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="J81" s="2"/>
     </row>
@@ -23144,16 +23137,16 @@
       </c>
       <c r="C82" s="2"/>
       <c r="D82" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E82" s="2" t="s">
-        <v>376</v>
+        <v>318</v>
       </c>
       <c r="F82" s="2"/>
       <c r="G82" s="2"/>
       <c r="H82" s="2"/>
       <c r="I82" s="2" t="s">
-        <v>376</v>
+        <v>318</v>
       </c>
       <c r="J82" s="2"/>
     </row>
@@ -23166,16 +23159,16 @@
       </c>
       <c r="C83" s="2"/>
       <c r="D83" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>316</v>
+        <v>360</v>
       </c>
       <c r="F83" s="2"/>
       <c r="G83" s="2"/>
       <c r="H83" s="2"/>
       <c r="I83" s="2" t="s">
-        <v>316</v>
+        <v>360</v>
       </c>
       <c r="J83" s="2"/>
     </row>
@@ -23188,16 +23181,16 @@
       </c>
       <c r="C84" s="2"/>
       <c r="D84" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>317</v>
+        <v>367</v>
       </c>
       <c r="F84" s="2"/>
       <c r="G84" s="2"/>
       <c r="H84" s="2"/>
       <c r="I84" s="2" t="s">
-        <v>317</v>
+        <v>367</v>
       </c>
       <c r="J84" s="2"/>
     </row>
@@ -23210,16 +23203,16 @@
       </c>
       <c r="C85" s="2"/>
       <c r="D85" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>340</v>
+        <v>319</v>
       </c>
       <c r="F85" s="2"/>
       <c r="G85" s="2"/>
       <c r="H85" s="2"/>
       <c r="I85" s="2" t="s">
-        <v>340</v>
+        <v>319</v>
       </c>
       <c r="J85" s="2"/>
     </row>
@@ -23232,16 +23225,16 @@
       </c>
       <c r="C86" s="2"/>
       <c r="D86" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
       <c r="F86" s="2"/>
       <c r="G86" s="2"/>
       <c r="H86" s="2"/>
       <c r="I86" s="2" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
       <c r="J86" s="2"/>
     </row>
@@ -23254,16 +23247,16 @@
       </c>
       <c r="C87" s="2"/>
       <c r="D87" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E87" s="2" t="s">
-        <v>369</v>
+        <v>359</v>
       </c>
       <c r="F87" s="2"/>
       <c r="G87" s="2"/>
       <c r="H87" s="2"/>
       <c r="I87" s="2" t="s">
-        <v>369</v>
+        <v>359</v>
       </c>
       <c r="J87" s="2"/>
     </row>
@@ -23276,16 +23269,16 @@
       </c>
       <c r="C88" s="2"/>
       <c r="D88" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>356</v>
+        <v>377</v>
       </c>
       <c r="F88" s="2"/>
       <c r="G88" s="2"/>
       <c r="H88" s="2"/>
       <c r="I88" s="2" t="s">
-        <v>356</v>
+        <v>570</v>
       </c>
       <c r="J88" s="2"/>
     </row>
@@ -23298,16 +23291,16 @@
       </c>
       <c r="C89" s="2"/>
       <c r="D89" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>358</v>
+        <v>378</v>
       </c>
       <c r="F89" s="2"/>
       <c r="G89" s="2"/>
       <c r="H89" s="2"/>
       <c r="I89" s="2" t="s">
-        <v>358</v>
+        <v>571</v>
       </c>
       <c r="J89" s="2"/>
     </row>
@@ -23320,16 +23313,16 @@
       </c>
       <c r="C90" s="2"/>
       <c r="D90" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>364</v>
+        <v>379</v>
       </c>
       <c r="F90" s="2"/>
       <c r="G90" s="2"/>
       <c r="H90" s="2"/>
       <c r="I90" s="2" t="s">
-        <v>364</v>
+        <v>572</v>
       </c>
       <c r="J90" s="2"/>
     </row>
@@ -23342,16 +23335,16 @@
       </c>
       <c r="C91" s="2"/>
       <c r="D91" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>331</v>
+        <v>380</v>
       </c>
       <c r="F91" s="2"/>
       <c r="G91" s="2"/>
       <c r="H91" s="2"/>
       <c r="I91" s="2" t="s">
-        <v>331</v>
+        <v>573</v>
       </c>
       <c r="J91" s="2"/>
     </row>
@@ -23364,16 +23357,16 @@
       </c>
       <c r="C92" s="2"/>
       <c r="D92" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E92" s="2" t="s">
-        <v>337</v>
+        <v>381</v>
       </c>
       <c r="F92" s="2"/>
       <c r="G92" s="2"/>
       <c r="H92" s="2"/>
       <c r="I92" s="2" t="s">
-        <v>337</v>
+        <v>574</v>
       </c>
       <c r="J92" s="2"/>
     </row>
@@ -23386,16 +23379,16 @@
       </c>
       <c r="C93" s="2"/>
       <c r="D93" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E93" s="2" t="s">
-        <v>351</v>
+        <v>382</v>
       </c>
       <c r="F93" s="2"/>
       <c r="G93" s="2"/>
       <c r="H93" s="2"/>
       <c r="I93" s="2" t="s">
-        <v>351</v>
+        <v>575</v>
       </c>
       <c r="J93" s="2"/>
     </row>
@@ -23408,16 +23401,16 @@
       </c>
       <c r="C94" s="2"/>
       <c r="D94" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E94" s="2" t="s">
-        <v>352</v>
+        <v>383</v>
       </c>
       <c r="F94" s="2"/>
       <c r="G94" s="2"/>
       <c r="H94" s="2"/>
       <c r="I94" s="2" t="s">
-        <v>352</v>
+        <v>576</v>
       </c>
       <c r="J94" s="2"/>
     </row>
@@ -23430,16 +23423,16 @@
       </c>
       <c r="C95" s="2"/>
       <c r="D95" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>353</v>
+        <v>384</v>
       </c>
       <c r="F95" s="2"/>
       <c r="G95" s="2"/>
       <c r="H95" s="2"/>
       <c r="I95" s="2" t="s">
-        <v>353</v>
+        <v>577</v>
       </c>
       <c r="J95" s="2"/>
     </row>
@@ -23452,16 +23445,16 @@
       </c>
       <c r="C96" s="2"/>
       <c r="D96" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E96" s="2" t="s">
-        <v>354</v>
+        <v>385</v>
       </c>
       <c r="F96" s="2"/>
       <c r="G96" s="2"/>
       <c r="H96" s="2"/>
       <c r="I96" s="2" t="s">
-        <v>354</v>
+        <v>578</v>
       </c>
       <c r="J96" s="2"/>
     </row>
@@ -23474,16 +23467,16 @@
       </c>
       <c r="C97" s="2"/>
       <c r="D97" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E97" s="2" t="s">
-        <v>323</v>
+        <v>386</v>
       </c>
       <c r="F97" s="2"/>
       <c r="G97" s="2"/>
       <c r="H97" s="2"/>
       <c r="I97" s="2" t="s">
-        <v>323</v>
+        <v>386</v>
       </c>
       <c r="J97" s="2"/>
     </row>
@@ -23496,16 +23489,16 @@
       </c>
       <c r="C98" s="2"/>
       <c r="D98" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E98" s="2" t="s">
-        <v>318</v>
+        <v>387</v>
       </c>
       <c r="F98" s="2"/>
       <c r="G98" s="2"/>
       <c r="H98" s="2"/>
       <c r="I98" s="2" t="s">
-        <v>318</v>
+        <v>387</v>
       </c>
       <c r="J98" s="2"/>
     </row>
@@ -23518,16 +23511,16 @@
       </c>
       <c r="C99" s="2"/>
       <c r="D99" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>360</v>
+        <v>388</v>
       </c>
       <c r="F99" s="2"/>
       <c r="G99" s="2"/>
       <c r="H99" s="2"/>
       <c r="I99" s="2" t="s">
-        <v>360</v>
+        <v>580</v>
       </c>
       <c r="J99" s="2"/>
     </row>
@@ -23540,16 +23533,16 @@
       </c>
       <c r="C100" s="2"/>
       <c r="D100" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E100" s="2" t="s">
-        <v>367</v>
+        <v>389</v>
       </c>
       <c r="F100" s="2"/>
       <c r="G100" s="2"/>
       <c r="H100" s="2"/>
       <c r="I100" s="2" t="s">
-        <v>367</v>
+        <v>389</v>
       </c>
       <c r="J100" s="2"/>
     </row>
@@ -23562,16 +23555,16 @@
       </c>
       <c r="C101" s="2"/>
       <c r="D101" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E101" s="2" t="s">
-        <v>319</v>
+        <v>390</v>
       </c>
       <c r="F101" s="2"/>
       <c r="G101" s="2"/>
       <c r="H101" s="2"/>
       <c r="I101" s="2" t="s">
-        <v>319</v>
+        <v>579</v>
       </c>
       <c r="J101" s="2"/>
     </row>
@@ -23584,16 +23577,16 @@
       </c>
       <c r="C102" s="2"/>
       <c r="D102" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E102" s="2" t="s">
-        <v>334</v>
+        <v>391</v>
       </c>
       <c r="F102" s="2"/>
       <c r="G102" s="2"/>
       <c r="H102" s="2"/>
       <c r="I102" s="2" t="s">
-        <v>334</v>
+        <v>391</v>
       </c>
       <c r="J102" s="2"/>
     </row>
@@ -23606,16 +23599,16 @@
       </c>
       <c r="C103" s="2"/>
       <c r="D103" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E103" s="2" t="s">
-        <v>359</v>
+        <v>392</v>
       </c>
       <c r="F103" s="2"/>
       <c r="G103" s="2"/>
       <c r="H103" s="2"/>
       <c r="I103" s="2" t="s">
-        <v>359</v>
+        <v>392</v>
       </c>
       <c r="J103" s="2"/>
     </row>
@@ -23628,16 +23621,16 @@
       </c>
       <c r="C104" s="2"/>
       <c r="D104" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E104" s="2" t="s">
-        <v>377</v>
+        <v>393</v>
       </c>
       <c r="F104" s="2"/>
       <c r="G104" s="2"/>
       <c r="H104" s="2"/>
       <c r="I104" s="2" t="s">
-        <v>570</v>
+        <v>582</v>
       </c>
       <c r="J104" s="2"/>
     </row>
@@ -23650,16 +23643,16 @@
       </c>
       <c r="C105" s="2"/>
       <c r="D105" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E105" s="2" t="s">
-        <v>378</v>
+        <v>394</v>
       </c>
       <c r="F105" s="2"/>
       <c r="G105" s="2"/>
       <c r="H105" s="2"/>
       <c r="I105" s="2" t="s">
-        <v>571</v>
+        <v>394</v>
       </c>
       <c r="J105" s="2"/>
     </row>
@@ -23672,16 +23665,16 @@
       </c>
       <c r="C106" s="2"/>
       <c r="D106" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E106" s="2" t="s">
-        <v>379</v>
+        <v>395</v>
       </c>
       <c r="F106" s="2"/>
       <c r="G106" s="2"/>
       <c r="H106" s="2"/>
       <c r="I106" s="2" t="s">
-        <v>572</v>
+        <v>581</v>
       </c>
       <c r="J106" s="2"/>
     </row>
@@ -23694,16 +23687,16 @@
       </c>
       <c r="C107" s="2"/>
       <c r="D107" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E107" s="2" t="s">
-        <v>380</v>
+        <v>396</v>
       </c>
       <c r="F107" s="2"/>
       <c r="G107" s="2"/>
       <c r="H107" s="2"/>
       <c r="I107" s="2" t="s">
-        <v>573</v>
+        <v>396</v>
       </c>
       <c r="J107" s="2"/>
     </row>
@@ -23716,16 +23709,16 @@
       </c>
       <c r="C108" s="2"/>
       <c r="D108" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E108" s="2" t="s">
-        <v>381</v>
+        <v>277</v>
       </c>
       <c r="F108" s="2"/>
       <c r="G108" s="2"/>
       <c r="H108" s="2"/>
       <c r="I108" s="2" t="s">
-        <v>574</v>
+        <v>583</v>
       </c>
       <c r="J108" s="2"/>
     </row>
@@ -23738,16 +23731,16 @@
       </c>
       <c r="C109" s="2"/>
       <c r="D109" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E109" s="2" t="s">
-        <v>382</v>
+        <v>278</v>
       </c>
       <c r="F109" s="2"/>
       <c r="G109" s="2"/>
       <c r="H109" s="2"/>
       <c r="I109" s="2" t="s">
-        <v>575</v>
+        <v>584</v>
       </c>
       <c r="J109" s="2"/>
     </row>
@@ -23760,16 +23753,16 @@
       </c>
       <c r="C110" s="2"/>
       <c r="D110" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E110" s="2" t="s">
-        <v>383</v>
+        <v>279</v>
       </c>
       <c r="F110" s="2"/>
       <c r="G110" s="2"/>
       <c r="H110" s="2"/>
       <c r="I110" s="2" t="s">
-        <v>576</v>
+        <v>585</v>
       </c>
       <c r="J110" s="2"/>
     </row>
@@ -23782,16 +23775,16 @@
       </c>
       <c r="C111" s="2"/>
       <c r="D111" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E111" s="2" t="s">
-        <v>384</v>
+        <v>397</v>
       </c>
       <c r="F111" s="2"/>
       <c r="G111" s="2"/>
       <c r="H111" s="2"/>
       <c r="I111" s="2" t="s">
-        <v>577</v>
+        <v>586</v>
       </c>
       <c r="J111" s="2"/>
     </row>
@@ -23804,16 +23797,16 @@
       </c>
       <c r="C112" s="2"/>
       <c r="D112" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E112" s="2" t="s">
-        <v>385</v>
+        <v>398</v>
       </c>
       <c r="F112" s="2"/>
       <c r="G112" s="2"/>
       <c r="H112" s="2"/>
       <c r="I112" s="2" t="s">
-        <v>578</v>
+        <v>587</v>
       </c>
       <c r="J112" s="2"/>
     </row>
@@ -23826,16 +23819,16 @@
       </c>
       <c r="C113" s="2"/>
       <c r="D113" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E113" s="2" t="s">
-        <v>386</v>
+        <v>399</v>
       </c>
       <c r="F113" s="2"/>
       <c r="G113" s="2"/>
       <c r="H113" s="2"/>
       <c r="I113" s="2" t="s">
-        <v>386</v>
+        <v>589</v>
       </c>
       <c r="J113" s="2"/>
     </row>
@@ -23848,16 +23841,16 @@
       </c>
       <c r="C114" s="2"/>
       <c r="D114" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E114" s="2" t="s">
-        <v>387</v>
+        <v>400</v>
       </c>
       <c r="F114" s="2"/>
       <c r="G114" s="2"/>
       <c r="H114" s="2"/>
       <c r="I114" s="2" t="s">
-        <v>387</v>
+        <v>588</v>
       </c>
       <c r="J114" s="2"/>
     </row>
@@ -23870,16 +23863,16 @@
       </c>
       <c r="C115" s="2"/>
       <c r="D115" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E115" s="2" t="s">
-        <v>388</v>
+        <v>283</v>
       </c>
       <c r="F115" s="2"/>
       <c r="G115" s="2"/>
       <c r="H115" s="2"/>
       <c r="I115" s="2" t="s">
-        <v>580</v>
+        <v>592</v>
       </c>
       <c r="J115" s="2"/>
     </row>
@@ -23892,16 +23885,16 @@
       </c>
       <c r="C116" s="2"/>
       <c r="D116" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E116" s="2" t="s">
-        <v>389</v>
+        <v>284</v>
       </c>
       <c r="F116" s="2"/>
       <c r="G116" s="2"/>
       <c r="H116" s="2"/>
       <c r="I116" s="2" t="s">
-        <v>389</v>
+        <v>593</v>
       </c>
       <c r="J116" s="2"/>
     </row>
@@ -23914,16 +23907,16 @@
       </c>
       <c r="C117" s="2"/>
       <c r="D117" s="2" t="s">
-        <v>728</v>
+        <v>725</v>
       </c>
       <c r="E117" s="2" t="s">
-        <v>390</v>
+        <v>401</v>
       </c>
       <c r="F117" s="2"/>
       <c r="G117" s="2"/>
       <c r="H117" s="2"/>
       <c r="I117" s="2" t="s">
-        <v>579</v>
+        <v>591</v>
       </c>
       <c r="J117" s="2"/>
     </row>
@@ -23931,43 +23924,41 @@
       <c r="A118" t="b">
         <v>1</v>
       </c>
-      <c r="B118" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B118" s="2"/>
       <c r="C118" s="2"/>
       <c r="D118" s="2" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="E118" s="2" t="s">
-        <v>391</v>
+        <v>271</v>
       </c>
       <c r="F118" s="2"/>
       <c r="G118" s="2"/>
       <c r="H118" s="2"/>
       <c r="I118" s="2" t="s">
-        <v>391</v>
-      </c>
-      <c r="J118" s="2"/>
+        <v>547</v>
+      </c>
+      <c r="J118" s="2" t="s">
+        <v>760</v>
+      </c>
     </row>
     <row r="119" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A119" t="b">
         <v>1</v>
       </c>
-      <c r="B119" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B119" s="2"/>
       <c r="C119" s="2"/>
       <c r="D119" s="2" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="E119" s="2" t="s">
-        <v>392</v>
+        <v>272</v>
       </c>
       <c r="F119" s="2"/>
       <c r="G119" s="2"/>
       <c r="H119" s="2"/>
       <c r="I119" s="2" t="s">
-        <v>392</v>
+        <v>552</v>
       </c>
       <c r="J119" s="2"/>
     </row>
@@ -23975,21 +23966,19 @@
       <c r="A120" t="b">
         <v>1</v>
       </c>
-      <c r="B120" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B120" s="2"/>
       <c r="C120" s="2"/>
       <c r="D120" s="2" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="E120" s="2" t="s">
-        <v>393</v>
+        <v>273</v>
       </c>
       <c r="F120" s="2"/>
       <c r="G120" s="2"/>
       <c r="H120" s="2"/>
       <c r="I120" s="2" t="s">
-        <v>582</v>
+        <v>553</v>
       </c>
       <c r="J120" s="2"/>
     </row>
@@ -23997,21 +23986,19 @@
       <c r="A121" t="b">
         <v>1</v>
       </c>
-      <c r="B121" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B121" s="2"/>
       <c r="C121" s="2"/>
       <c r="D121" s="2" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="E121" s="2" t="s">
-        <v>394</v>
+        <v>274</v>
       </c>
       <c r="F121" s="2"/>
       <c r="G121" s="2"/>
       <c r="H121" s="2"/>
       <c r="I121" s="2" t="s">
-        <v>394</v>
+        <v>554</v>
       </c>
       <c r="J121" s="2"/>
     </row>
@@ -24019,21 +24006,19 @@
       <c r="A122" t="b">
         <v>1</v>
       </c>
-      <c r="B122" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B122" s="2"/>
       <c r="C122" s="2"/>
       <c r="D122" s="2" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="E122" s="2" t="s">
-        <v>395</v>
+        <v>275</v>
       </c>
       <c r="F122" s="2"/>
       <c r="G122" s="2"/>
       <c r="H122" s="2"/>
       <c r="I122" s="2" t="s">
-        <v>581</v>
+        <v>555</v>
       </c>
       <c r="J122" s="2"/>
     </row>
@@ -24041,21 +24026,19 @@
       <c r="A123" t="b">
         <v>1</v>
       </c>
-      <c r="B123" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B123" s="2"/>
       <c r="C123" s="2"/>
       <c r="D123" s="2" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="E123" s="2" t="s">
-        <v>396</v>
+        <v>276</v>
       </c>
       <c r="F123" s="2"/>
       <c r="G123" s="2"/>
       <c r="H123" s="2"/>
       <c r="I123" s="2" t="s">
-        <v>396</v>
+        <v>556</v>
       </c>
       <c r="J123" s="2"/>
     </row>
@@ -24063,12 +24046,10 @@
       <c r="A124" t="b">
         <v>1</v>
       </c>
-      <c r="B124" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B124" s="2"/>
       <c r="C124" s="2"/>
       <c r="D124" s="2" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="E124" s="2" t="s">
         <v>277</v>
@@ -24077,7 +24058,7 @@
       <c r="G124" s="2"/>
       <c r="H124" s="2"/>
       <c r="I124" s="2" t="s">
-        <v>583</v>
+        <v>557</v>
       </c>
       <c r="J124" s="2"/>
     </row>
@@ -24085,12 +24066,10 @@
       <c r="A125" t="b">
         <v>1</v>
       </c>
-      <c r="B125" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B125" s="2"/>
       <c r="C125" s="2"/>
       <c r="D125" s="2" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="E125" s="2" t="s">
         <v>278</v>
@@ -24099,7 +24078,7 @@
       <c r="G125" s="2"/>
       <c r="H125" s="2"/>
       <c r="I125" s="2" t="s">
-        <v>584</v>
+        <v>558</v>
       </c>
       <c r="J125" s="2"/>
     </row>
@@ -24107,12 +24086,10 @@
       <c r="A126" t="b">
         <v>1</v>
       </c>
-      <c r="B126" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B126" s="2"/>
       <c r="C126" s="2"/>
       <c r="D126" s="2" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="E126" s="2" t="s">
         <v>279</v>
@@ -24121,7 +24098,7 @@
       <c r="G126" s="2"/>
       <c r="H126" s="2"/>
       <c r="I126" s="2" t="s">
-        <v>585</v>
+        <v>559</v>
       </c>
       <c r="J126" s="2"/>
     </row>
@@ -24129,21 +24106,19 @@
       <c r="A127" t="b">
         <v>1</v>
       </c>
-      <c r="B127" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B127" s="2"/>
       <c r="C127" s="2"/>
       <c r="D127" s="2" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="E127" s="2" t="s">
-        <v>397</v>
+        <v>280</v>
       </c>
       <c r="F127" s="2"/>
       <c r="G127" s="2"/>
       <c r="H127" s="2"/>
       <c r="I127" s="2" t="s">
-        <v>586</v>
+        <v>549</v>
       </c>
       <c r="J127" s="2"/>
     </row>
@@ -24151,21 +24126,19 @@
       <c r="A128" t="b">
         <v>1</v>
       </c>
-      <c r="B128" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B128" s="2"/>
       <c r="C128" s="2"/>
       <c r="D128" s="2" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="E128" s="2" t="s">
-        <v>398</v>
+        <v>281</v>
       </c>
       <c r="F128" s="2"/>
       <c r="G128" s="2"/>
       <c r="H128" s="2"/>
       <c r="I128" s="2" t="s">
-        <v>587</v>
+        <v>550</v>
       </c>
       <c r="J128" s="2"/>
     </row>
@@ -24173,21 +24146,19 @@
       <c r="A129" t="b">
         <v>1</v>
       </c>
-      <c r="B129" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B129" s="2"/>
       <c r="C129" s="2"/>
       <c r="D129" s="2" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="E129" s="2" t="s">
-        <v>399</v>
+        <v>282</v>
       </c>
       <c r="F129" s="2"/>
       <c r="G129" s="2"/>
       <c r="H129" s="2"/>
       <c r="I129" s="2" t="s">
-        <v>589</v>
+        <v>566</v>
       </c>
       <c r="J129" s="2"/>
     </row>
@@ -24195,21 +24166,19 @@
       <c r="A130" t="b">
         <v>1</v>
       </c>
-      <c r="B130" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B130" s="2"/>
       <c r="C130" s="2"/>
       <c r="D130" s="2" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="E130" s="2" t="s">
-        <v>400</v>
+        <v>283</v>
       </c>
       <c r="F130" s="2"/>
       <c r="G130" s="2"/>
       <c r="H130" s="2"/>
       <c r="I130" s="2" t="s">
-        <v>588</v>
+        <v>560</v>
       </c>
       <c r="J130" s="2"/>
     </row>
@@ -24217,21 +24186,19 @@
       <c r="A131" t="b">
         <v>1</v>
       </c>
-      <c r="B131" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B131" s="2"/>
       <c r="C131" s="2"/>
       <c r="D131" s="2" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="E131" s="2" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="F131" s="2"/>
       <c r="G131" s="2"/>
       <c r="H131" s="2"/>
       <c r="I131" s="2" t="s">
-        <v>592</v>
+        <v>551</v>
       </c>
       <c r="J131" s="2"/>
     </row>
@@ -24239,21 +24206,19 @@
       <c r="A132" t="b">
         <v>1</v>
       </c>
-      <c r="B132" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B132" s="2"/>
       <c r="C132" s="2"/>
       <c r="D132" s="2" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="E132" s="2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="F132" s="2"/>
       <c r="G132" s="2"/>
       <c r="H132" s="2"/>
       <c r="I132" s="2" t="s">
-        <v>593</v>
+        <v>561</v>
       </c>
       <c r="J132" s="2"/>
     </row>
@@ -24261,21 +24226,19 @@
       <c r="A133" t="b">
         <v>1</v>
       </c>
-      <c r="B133" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B133" s="2"/>
       <c r="C133" s="2"/>
       <c r="D133" s="2" t="s">
-        <v>728</v>
+        <v>726</v>
       </c>
       <c r="E133" s="2" t="s">
-        <v>401</v>
+        <v>286</v>
       </c>
       <c r="F133" s="2"/>
       <c r="G133" s="2"/>
       <c r="H133" s="2"/>
       <c r="I133" s="2" t="s">
-        <v>591</v>
+        <v>562</v>
       </c>
       <c r="J133" s="2"/>
     </row>
@@ -24286,20 +24249,18 @@
       <c r="B134" s="2"/>
       <c r="C134" s="2"/>
       <c r="D134" s="2" t="s">
-        <v>729</v>
+        <v>726</v>
       </c>
       <c r="E134" s="2" t="s">
-        <v>271</v>
+        <v>287</v>
       </c>
       <c r="F134" s="2"/>
       <c r="G134" s="2"/>
       <c r="H134" s="2"/>
       <c r="I134" s="2" t="s">
-        <v>547</v>
-      </c>
-      <c r="J134" s="2" t="s">
-        <v>763</v>
-      </c>
+        <v>563</v>
+      </c>
+      <c r="J134" s="2"/>
     </row>
     <row r="135" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A135" t="b">
@@ -24308,16 +24269,16 @@
       <c r="B135" s="2"/>
       <c r="C135" s="2"/>
       <c r="D135" s="2" t="s">
-        <v>729</v>
+        <v>726</v>
       </c>
       <c r="E135" s="2" t="s">
-        <v>272</v>
+        <v>288</v>
       </c>
       <c r="F135" s="2"/>
       <c r="G135" s="2"/>
       <c r="H135" s="2"/>
       <c r="I135" s="2" t="s">
-        <v>552</v>
+        <v>564</v>
       </c>
       <c r="J135" s="2"/>
     </row>
@@ -24328,16 +24289,16 @@
       <c r="B136" s="2"/>
       <c r="C136" s="2"/>
       <c r="D136" s="2" t="s">
-        <v>729</v>
+        <v>726</v>
       </c>
       <c r="E136" s="2" t="s">
-        <v>273</v>
+        <v>289</v>
       </c>
       <c r="F136" s="2"/>
       <c r="G136" s="2"/>
       <c r="H136" s="2"/>
       <c r="I136" s="2" t="s">
-        <v>553</v>
+        <v>565</v>
       </c>
       <c r="J136" s="2"/>
     </row>
@@ -24348,16 +24309,16 @@
       <c r="B137" s="2"/>
       <c r="C137" s="2"/>
       <c r="D137" s="2" t="s">
-        <v>729</v>
+        <v>726</v>
       </c>
       <c r="E137" s="2" t="s">
-        <v>274</v>
+        <v>290</v>
       </c>
       <c r="F137" s="2"/>
       <c r="G137" s="2"/>
       <c r="H137" s="2"/>
       <c r="I137" s="2" t="s">
-        <v>554</v>
+        <v>548</v>
       </c>
       <c r="J137" s="2"/>
     </row>
@@ -24368,18 +24329,20 @@
       <c r="B138" s="2"/>
       <c r="C138" s="2"/>
       <c r="D138" s="2" t="s">
-        <v>729</v>
+        <v>727</v>
       </c>
       <c r="E138" s="2" t="s">
-        <v>275</v>
+        <v>409</v>
       </c>
       <c r="F138" s="2"/>
       <c r="G138" s="2"/>
       <c r="H138" s="2"/>
       <c r="I138" s="2" t="s">
-        <v>555</v>
-      </c>
-      <c r="J138" s="2"/>
+        <v>518</v>
+      </c>
+      <c r="J138" s="2" t="s">
+        <v>762</v>
+      </c>
     </row>
     <row r="139" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A139" t="b">
@@ -24388,16 +24351,16 @@
       <c r="B139" s="2"/>
       <c r="C139" s="2"/>
       <c r="D139" s="2" t="s">
-        <v>729</v>
+        <v>727</v>
       </c>
       <c r="E139" s="2" t="s">
-        <v>276</v>
+        <v>410</v>
       </c>
       <c r="F139" s="2"/>
       <c r="G139" s="2"/>
       <c r="H139" s="2"/>
       <c r="I139" s="2" t="s">
-        <v>556</v>
+        <v>519</v>
       </c>
       <c r="J139" s="2"/>
     </row>
@@ -24408,16 +24371,16 @@
       <c r="B140" s="2"/>
       <c r="C140" s="2"/>
       <c r="D140" s="2" t="s">
-        <v>729</v>
+        <v>727</v>
       </c>
       <c r="E140" s="2" t="s">
-        <v>277</v>
+        <v>411</v>
       </c>
       <c r="F140" s="2"/>
       <c r="G140" s="2"/>
       <c r="H140" s="2"/>
       <c r="I140" s="2" t="s">
-        <v>557</v>
+        <v>411</v>
       </c>
       <c r="J140" s="2"/>
     </row>
@@ -24428,16 +24391,16 @@
       <c r="B141" s="2"/>
       <c r="C141" s="2"/>
       <c r="D141" s="2" t="s">
-        <v>729</v>
+        <v>727</v>
       </c>
       <c r="E141" s="2" t="s">
-        <v>278</v>
+        <v>412</v>
       </c>
       <c r="F141" s="2"/>
       <c r="G141" s="2"/>
       <c r="H141" s="2"/>
       <c r="I141" s="2" t="s">
-        <v>558</v>
+        <v>622</v>
       </c>
       <c r="J141" s="2"/>
     </row>
@@ -24448,16 +24411,16 @@
       <c r="B142" s="2"/>
       <c r="C142" s="2"/>
       <c r="D142" s="2" t="s">
-        <v>729</v>
+        <v>727</v>
       </c>
       <c r="E142" s="2" t="s">
-        <v>279</v>
+        <v>413</v>
       </c>
       <c r="F142" s="2"/>
       <c r="G142" s="2"/>
       <c r="H142" s="2"/>
       <c r="I142" s="2" t="s">
-        <v>559</v>
+        <v>623</v>
       </c>
       <c r="J142" s="2"/>
     </row>
@@ -24468,16 +24431,16 @@
       <c r="B143" s="2"/>
       <c r="C143" s="2"/>
       <c r="D143" s="2" t="s">
-        <v>729</v>
+        <v>727</v>
       </c>
       <c r="E143" s="2" t="s">
-        <v>280</v>
+        <v>414</v>
       </c>
       <c r="F143" s="2"/>
       <c r="G143" s="2"/>
       <c r="H143" s="2"/>
       <c r="I143" s="2" t="s">
-        <v>549</v>
+        <v>518</v>
       </c>
       <c r="J143" s="2"/>
     </row>
@@ -24488,16 +24451,16 @@
       <c r="B144" s="2"/>
       <c r="C144" s="2"/>
       <c r="D144" s="2" t="s">
-        <v>729</v>
+        <v>727</v>
       </c>
       <c r="E144" s="2" t="s">
-        <v>281</v>
+        <v>149</v>
       </c>
       <c r="F144" s="2"/>
       <c r="G144" s="2"/>
       <c r="H144" s="2"/>
       <c r="I144" s="2" t="s">
-        <v>550</v>
+        <v>612</v>
       </c>
       <c r="J144" s="2"/>
     </row>
@@ -24511,15 +24474,17 @@
         <v>729</v>
       </c>
       <c r="E145" s="2" t="s">
-        <v>282</v>
+        <v>415</v>
       </c>
       <c r="F145" s="2"/>
       <c r="G145" s="2"/>
       <c r="H145" s="2"/>
       <c r="I145" s="2" t="s">
-        <v>566</v>
-      </c>
-      <c r="J145" s="2"/>
+        <v>624</v>
+      </c>
+      <c r="J145" s="2" t="s">
+        <v>763</v>
+      </c>
     </row>
     <row r="146" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A146" t="b">
@@ -24531,13 +24496,13 @@
         <v>729</v>
       </c>
       <c r="E146" s="2" t="s">
-        <v>283</v>
+        <v>416</v>
       </c>
       <c r="F146" s="2"/>
       <c r="G146" s="2"/>
       <c r="H146" s="2"/>
       <c r="I146" s="2" t="s">
-        <v>560</v>
+        <v>625</v>
       </c>
       <c r="J146" s="2"/>
     </row>
@@ -24551,13 +24516,13 @@
         <v>729</v>
       </c>
       <c r="E147" s="2" t="s">
-        <v>284</v>
+        <v>417</v>
       </c>
       <c r="F147" s="2"/>
       <c r="G147" s="2"/>
       <c r="H147" s="2"/>
       <c r="I147" s="2" t="s">
-        <v>551</v>
+        <v>626</v>
       </c>
       <c r="J147" s="2"/>
     </row>
@@ -24571,13 +24536,13 @@
         <v>729</v>
       </c>
       <c r="E148" s="2" t="s">
-        <v>285</v>
+        <v>418</v>
       </c>
       <c r="F148" s="2"/>
       <c r="G148" s="2"/>
       <c r="H148" s="2"/>
       <c r="I148" s="2" t="s">
-        <v>561</v>
+        <v>627</v>
       </c>
       <c r="J148" s="2"/>
     </row>
@@ -24591,13 +24556,13 @@
         <v>729</v>
       </c>
       <c r="E149" s="2" t="s">
-        <v>286</v>
+        <v>149</v>
       </c>
       <c r="F149" s="2"/>
       <c r="G149" s="2"/>
       <c r="H149" s="2"/>
       <c r="I149" s="2" t="s">
-        <v>562</v>
+        <v>612</v>
       </c>
       <c r="J149" s="2"/>
     </row>
@@ -24608,18 +24573,20 @@
       <c r="B150" s="2"/>
       <c r="C150" s="2"/>
       <c r="D150" s="2" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
       <c r="E150" s="2" t="s">
-        <v>287</v>
+        <v>409</v>
       </c>
       <c r="F150" s="2"/>
       <c r="G150" s="2"/>
       <c r="H150" s="2"/>
       <c r="I150" s="2" t="s">
-        <v>563</v>
-      </c>
-      <c r="J150" s="2"/>
+        <v>518</v>
+      </c>
+      <c r="J150" s="2" t="s">
+        <v>764</v>
+      </c>
     </row>
     <row r="151" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A151" t="b">
@@ -24628,16 +24595,16 @@
       <c r="B151" s="2"/>
       <c r="C151" s="2"/>
       <c r="D151" s="2" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
       <c r="E151" s="2" t="s">
-        <v>288</v>
+        <v>410</v>
       </c>
       <c r="F151" s="2"/>
       <c r="G151" s="2"/>
       <c r="H151" s="2"/>
       <c r="I151" s="2" t="s">
-        <v>564</v>
+        <v>519</v>
       </c>
       <c r="J151" s="2"/>
     </row>
@@ -24648,16 +24615,16 @@
       <c r="B152" s="2"/>
       <c r="C152" s="2"/>
       <c r="D152" s="2" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
       <c r="E152" s="2" t="s">
-        <v>289</v>
+        <v>411</v>
       </c>
       <c r="F152" s="2"/>
       <c r="G152" s="2"/>
       <c r="H152" s="2"/>
       <c r="I152" s="2" t="s">
-        <v>565</v>
+        <v>411</v>
       </c>
       <c r="J152" s="2"/>
     </row>
@@ -24668,16 +24635,16 @@
       <c r="B153" s="2"/>
       <c r="C153" s="2"/>
       <c r="D153" s="2" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
       <c r="E153" s="2" t="s">
-        <v>290</v>
+        <v>412</v>
       </c>
       <c r="F153" s="2"/>
       <c r="G153" s="2"/>
       <c r="H153" s="2"/>
       <c r="I153" s="2" t="s">
-        <v>548</v>
+        <v>622</v>
       </c>
       <c r="J153" s="2"/>
     </row>
@@ -24688,20 +24655,18 @@
       <c r="B154" s="2"/>
       <c r="C154" s="2"/>
       <c r="D154" s="2" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="E154" s="2" t="s">
-        <v>409</v>
+        <v>413</v>
       </c>
       <c r="F154" s="2"/>
       <c r="G154" s="2"/>
       <c r="H154" s="2"/>
       <c r="I154" s="2" t="s">
-        <v>518</v>
-      </c>
-      <c r="J154" s="2" t="s">
-        <v>765</v>
-      </c>
+        <v>623</v>
+      </c>
+      <c r="J154" s="2"/>
     </row>
     <row r="155" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A155" t="b">
@@ -24710,16 +24675,16 @@
       <c r="B155" s="2"/>
       <c r="C155" s="2"/>
       <c r="D155" s="2" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="E155" s="2" t="s">
-        <v>410</v>
+        <v>419</v>
       </c>
       <c r="F155" s="2"/>
       <c r="G155" s="2"/>
       <c r="H155" s="2"/>
       <c r="I155" s="2" t="s">
-        <v>519</v>
+        <v>624</v>
       </c>
       <c r="J155" s="2"/>
     </row>
@@ -24730,16 +24695,16 @@
       <c r="B156" s="2"/>
       <c r="C156" s="2"/>
       <c r="D156" s="2" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="E156" s="2" t="s">
-        <v>411</v>
+        <v>416</v>
       </c>
       <c r="F156" s="2"/>
       <c r="G156" s="2"/>
       <c r="H156" s="2"/>
       <c r="I156" s="2" t="s">
-        <v>411</v>
+        <v>625</v>
       </c>
       <c r="J156" s="2"/>
     </row>
@@ -24750,16 +24715,16 @@
       <c r="B157" s="2"/>
       <c r="C157" s="2"/>
       <c r="D157" s="2" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="E157" s="2" t="s">
-        <v>412</v>
+        <v>417</v>
       </c>
       <c r="F157" s="2"/>
       <c r="G157" s="2"/>
       <c r="H157" s="2"/>
       <c r="I157" s="2" t="s">
-        <v>622</v>
+        <v>626</v>
       </c>
       <c r="J157" s="2"/>
     </row>
@@ -24770,16 +24735,16 @@
       <c r="B158" s="2"/>
       <c r="C158" s="2"/>
       <c r="D158" s="2" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="E158" s="2" t="s">
-        <v>413</v>
+        <v>418</v>
       </c>
       <c r="F158" s="2"/>
       <c r="G158" s="2"/>
       <c r="H158" s="2"/>
       <c r="I158" s="2" t="s">
-        <v>623</v>
+        <v>627</v>
       </c>
       <c r="J158" s="2"/>
     </row>
@@ -24790,16 +24755,16 @@
       <c r="B159" s="2"/>
       <c r="C159" s="2"/>
       <c r="D159" s="2" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="E159" s="2" t="s">
-        <v>414</v>
+        <v>420</v>
       </c>
       <c r="F159" s="2"/>
       <c r="G159" s="2"/>
       <c r="H159" s="2"/>
       <c r="I159" s="2" t="s">
-        <v>518</v>
+        <v>628</v>
       </c>
       <c r="J159" s="2"/>
     </row>
@@ -24810,7 +24775,7 @@
       <c r="B160" s="2"/>
       <c r="C160" s="2"/>
       <c r="D160" s="2" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="E160" s="2" t="s">
         <v>149</v>
@@ -24830,19 +24795,19 @@
       <c r="B161" s="2"/>
       <c r="C161" s="2"/>
       <c r="D161" s="2" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="E161" s="2" t="s">
-        <v>415</v>
+        <v>423</v>
       </c>
       <c r="F161" s="2"/>
       <c r="G161" s="2"/>
       <c r="H161" s="2"/>
       <c r="I161" s="2" t="s">
-        <v>624</v>
+        <v>598</v>
       </c>
       <c r="J161" s="2" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
     </row>
     <row r="162" spans="1:10" x14ac:dyDescent="0.2">
@@ -24852,16 +24817,16 @@
       <c r="B162" s="2"/>
       <c r="C162" s="2"/>
       <c r="D162" s="2" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="E162" s="2" t="s">
-        <v>416</v>
+        <v>424</v>
       </c>
       <c r="F162" s="2"/>
       <c r="G162" s="2"/>
       <c r="H162" s="2"/>
       <c r="I162" s="2" t="s">
-        <v>625</v>
+        <v>602</v>
       </c>
       <c r="J162" s="2"/>
     </row>
@@ -24872,16 +24837,16 @@
       <c r="B163" s="2"/>
       <c r="C163" s="2"/>
       <c r="D163" s="2" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="E163" s="2" t="s">
-        <v>417</v>
+        <v>425</v>
       </c>
       <c r="F163" s="2"/>
       <c r="G163" s="2"/>
       <c r="H163" s="2"/>
       <c r="I163" s="2" t="s">
-        <v>626</v>
+        <v>599</v>
       </c>
       <c r="J163" s="2"/>
     </row>
@@ -24892,16 +24857,16 @@
       <c r="B164" s="2"/>
       <c r="C164" s="2"/>
       <c r="D164" s="2" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="E164" s="2" t="s">
-        <v>418</v>
+        <v>426</v>
       </c>
       <c r="F164" s="2"/>
       <c r="G164" s="2"/>
       <c r="H164" s="2"/>
       <c r="I164" s="2" t="s">
-        <v>627</v>
+        <v>603</v>
       </c>
       <c r="J164" s="2"/>
     </row>
@@ -24912,16 +24877,16 @@
       <c r="B165" s="2"/>
       <c r="C165" s="2"/>
       <c r="D165" s="2" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="E165" s="2" t="s">
-        <v>149</v>
+        <v>427</v>
       </c>
       <c r="F165" s="2"/>
       <c r="G165" s="2"/>
       <c r="H165" s="2"/>
       <c r="I165" s="2" t="s">
-        <v>612</v>
+        <v>599</v>
       </c>
       <c r="J165" s="2"/>
     </row>
@@ -24932,20 +24897,18 @@
       <c r="B166" s="2"/>
       <c r="C166" s="2"/>
       <c r="D166" s="2" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="E166" s="2" t="s">
-        <v>409</v>
+        <v>428</v>
       </c>
       <c r="F166" s="2"/>
       <c r="G166" s="2"/>
       <c r="H166" s="2"/>
       <c r="I166" s="2" t="s">
-        <v>518</v>
-      </c>
-      <c r="J166" s="2" t="s">
-        <v>767</v>
-      </c>
+        <v>603</v>
+      </c>
+      <c r="J166" s="2"/>
     </row>
     <row r="167" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A167" t="b">
@@ -24954,16 +24917,16 @@
       <c r="B167" s="2"/>
       <c r="C167" s="2"/>
       <c r="D167" s="2" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="E167" s="2" t="s">
-        <v>410</v>
+        <v>429</v>
       </c>
       <c r="F167" s="2"/>
       <c r="G167" s="2"/>
       <c r="H167" s="2"/>
       <c r="I167" s="2" t="s">
-        <v>519</v>
+        <v>600</v>
       </c>
       <c r="J167" s="2"/>
     </row>
@@ -24974,16 +24937,16 @@
       <c r="B168" s="2"/>
       <c r="C168" s="2"/>
       <c r="D168" s="2" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="E168" s="2" t="s">
-        <v>411</v>
+        <v>430</v>
       </c>
       <c r="F168" s="2"/>
       <c r="G168" s="2"/>
       <c r="H168" s="2"/>
       <c r="I168" s="2" t="s">
-        <v>411</v>
+        <v>604</v>
       </c>
       <c r="J168" s="2"/>
     </row>
@@ -24994,16 +24957,16 @@
       <c r="B169" s="2"/>
       <c r="C169" s="2"/>
       <c r="D169" s="2" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="E169" s="2" t="s">
-        <v>412</v>
+        <v>431</v>
       </c>
       <c r="F169" s="2"/>
       <c r="G169" s="2"/>
       <c r="H169" s="2"/>
       <c r="I169" s="2" t="s">
-        <v>622</v>
+        <v>601</v>
       </c>
       <c r="J169" s="2"/>
     </row>
@@ -25014,16 +24977,16 @@
       <c r="B170" s="2"/>
       <c r="C170" s="2"/>
       <c r="D170" s="2" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="E170" s="2" t="s">
-        <v>413</v>
+        <v>432</v>
       </c>
       <c r="F170" s="2"/>
       <c r="G170" s="2"/>
       <c r="H170" s="2"/>
       <c r="I170" s="2" t="s">
-        <v>623</v>
+        <v>605</v>
       </c>
       <c r="J170" s="2"/>
     </row>
@@ -25034,16 +24997,16 @@
       <c r="B171" s="2"/>
       <c r="C171" s="2"/>
       <c r="D171" s="2" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="E171" s="2" t="s">
-        <v>419</v>
+        <v>433</v>
       </c>
       <c r="F171" s="2"/>
       <c r="G171" s="2"/>
       <c r="H171" s="2"/>
       <c r="I171" s="2" t="s">
-        <v>624</v>
+        <v>601</v>
       </c>
       <c r="J171" s="2"/>
     </row>
@@ -25054,16 +25017,16 @@
       <c r="B172" s="2"/>
       <c r="C172" s="2"/>
       <c r="D172" s="2" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="E172" s="2" t="s">
-        <v>416</v>
+        <v>434</v>
       </c>
       <c r="F172" s="2"/>
       <c r="G172" s="2"/>
       <c r="H172" s="2"/>
       <c r="I172" s="2" t="s">
-        <v>625</v>
+        <v>605</v>
       </c>
       <c r="J172" s="2"/>
     </row>
@@ -25077,15 +25040,17 @@
         <v>734</v>
       </c>
       <c r="E173" s="2" t="s">
-        <v>417</v>
+        <v>423</v>
       </c>
       <c r="F173" s="2"/>
       <c r="G173" s="2"/>
       <c r="H173" s="2"/>
       <c r="I173" s="2" t="s">
-        <v>626</v>
-      </c>
-      <c r="J173" s="2"/>
+        <v>598</v>
+      </c>
+      <c r="J173" s="2" t="s">
+        <v>735</v>
+      </c>
     </row>
     <row r="174" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A174" t="b">
@@ -25097,13 +25062,13 @@
         <v>734</v>
       </c>
       <c r="E174" s="2" t="s">
-        <v>418</v>
+        <v>424</v>
       </c>
       <c r="F174" s="2"/>
       <c r="G174" s="2"/>
       <c r="H174" s="2"/>
       <c r="I174" s="2" t="s">
-        <v>627</v>
+        <v>602</v>
       </c>
       <c r="J174" s="2"/>
     </row>
@@ -25117,13 +25082,13 @@
         <v>734</v>
       </c>
       <c r="E175" s="2" t="s">
-        <v>420</v>
+        <v>425</v>
       </c>
       <c r="F175" s="2"/>
       <c r="G175" s="2"/>
       <c r="H175" s="2"/>
       <c r="I175" s="2" t="s">
-        <v>628</v>
+        <v>599</v>
       </c>
       <c r="J175" s="2"/>
     </row>
@@ -25137,13 +25102,13 @@
         <v>734</v>
       </c>
       <c r="E176" s="2" t="s">
-        <v>149</v>
+        <v>426</v>
       </c>
       <c r="F176" s="2"/>
       <c r="G176" s="2"/>
       <c r="H176" s="2"/>
       <c r="I176" s="2" t="s">
-        <v>612</v>
+        <v>603</v>
       </c>
       <c r="J176" s="2"/>
     </row>
@@ -25154,20 +25119,18 @@
       <c r="B177" s="2"/>
       <c r="C177" s="2"/>
       <c r="D177" s="2" t="s">
-        <v>736</v>
+        <v>734</v>
       </c>
       <c r="E177" s="2" t="s">
-        <v>423</v>
+        <v>427</v>
       </c>
       <c r="F177" s="2"/>
       <c r="G177" s="2"/>
       <c r="H177" s="2"/>
       <c r="I177" s="2" t="s">
-        <v>598</v>
-      </c>
-      <c r="J177" s="2" t="s">
-        <v>768</v>
-      </c>
+        <v>599</v>
+      </c>
+      <c r="J177" s="2"/>
     </row>
     <row r="178" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A178" t="b">
@@ -25176,16 +25139,16 @@
       <c r="B178" s="2"/>
       <c r="C178" s="2"/>
       <c r="D178" s="2" t="s">
-        <v>736</v>
+        <v>734</v>
       </c>
       <c r="E178" s="2" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="F178" s="2"/>
       <c r="G178" s="2"/>
       <c r="H178" s="2"/>
       <c r="I178" s="2" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="J178" s="2"/>
     </row>
@@ -25196,16 +25159,16 @@
       <c r="B179" s="2"/>
       <c r="C179" s="2"/>
       <c r="D179" s="2" t="s">
-        <v>736</v>
+        <v>734</v>
       </c>
       <c r="E179" s="2" t="s">
-        <v>425</v>
+        <v>429</v>
       </c>
       <c r="F179" s="2"/>
       <c r="G179" s="2"/>
       <c r="H179" s="2"/>
       <c r="I179" s="2" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="J179" s="2"/>
     </row>
@@ -25216,16 +25179,16 @@
       <c r="B180" s="2"/>
       <c r="C180" s="2"/>
       <c r="D180" s="2" t="s">
-        <v>736</v>
+        <v>734</v>
       </c>
       <c r="E180" s="2" t="s">
-        <v>426</v>
+        <v>430</v>
       </c>
       <c r="F180" s="2"/>
       <c r="G180" s="2"/>
       <c r="H180" s="2"/>
       <c r="I180" s="2" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="J180" s="2"/>
     </row>
@@ -25236,16 +25199,16 @@
       <c r="B181" s="2"/>
       <c r="C181" s="2"/>
       <c r="D181" s="2" t="s">
-        <v>736</v>
+        <v>734</v>
       </c>
       <c r="E181" s="2" t="s">
-        <v>427</v>
+        <v>431</v>
       </c>
       <c r="F181" s="2"/>
       <c r="G181" s="2"/>
       <c r="H181" s="2"/>
       <c r="I181" s="2" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
       <c r="J181" s="2"/>
     </row>
@@ -25256,16 +25219,16 @@
       <c r="B182" s="2"/>
       <c r="C182" s="2"/>
       <c r="D182" s="2" t="s">
-        <v>736</v>
+        <v>734</v>
       </c>
       <c r="E182" s="2" t="s">
-        <v>428</v>
+        <v>432</v>
       </c>
       <c r="F182" s="2"/>
       <c r="G182" s="2"/>
       <c r="H182" s="2"/>
       <c r="I182" s="2" t="s">
-        <v>603</v>
+        <v>605</v>
       </c>
       <c r="J182" s="2"/>
     </row>
@@ -25276,16 +25239,16 @@
       <c r="B183" s="2"/>
       <c r="C183" s="2"/>
       <c r="D183" s="2" t="s">
-        <v>736</v>
+        <v>734</v>
       </c>
       <c r="E183" s="2" t="s">
-        <v>429</v>
+        <v>433</v>
       </c>
       <c r="F183" s="2"/>
       <c r="G183" s="2"/>
       <c r="H183" s="2"/>
       <c r="I183" s="2" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="J183" s="2"/>
     </row>
@@ -25296,16 +25259,16 @@
       <c r="B184" s="2"/>
       <c r="C184" s="2"/>
       <c r="D184" s="2" t="s">
-        <v>736</v>
+        <v>734</v>
       </c>
       <c r="E184" s="2" t="s">
-        <v>430</v>
+        <v>434</v>
       </c>
       <c r="F184" s="2"/>
       <c r="G184" s="2"/>
       <c r="H184" s="2"/>
       <c r="I184" s="2" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="J184" s="2"/>
     </row>
@@ -25316,340 +25279,18 @@
       <c r="B185" s="2"/>
       <c r="C185" s="2"/>
       <c r="D185" s="2" t="s">
-        <v>736</v>
+        <v>734</v>
       </c>
       <c r="E185" s="2" t="s">
-        <v>431</v>
+        <v>149</v>
       </c>
       <c r="F185" s="2"/>
       <c r="G185" s="2"/>
       <c r="H185" s="2"/>
       <c r="I185" s="2" t="s">
-        <v>601</v>
+        <v>612</v>
       </c>
       <c r="J185" s="2"/>
-    </row>
-    <row r="186" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A186" t="b">
-        <v>1</v>
-      </c>
-      <c r="B186" s="2"/>
-      <c r="C186" s="2"/>
-      <c r="D186" s="2" t="s">
-        <v>736</v>
-      </c>
-      <c r="E186" s="2" t="s">
-        <v>432</v>
-      </c>
-      <c r="F186" s="2"/>
-      <c r="G186" s="2"/>
-      <c r="H186" s="2"/>
-      <c r="I186" s="2" t="s">
-        <v>605</v>
-      </c>
-      <c r="J186" s="2"/>
-    </row>
-    <row r="187" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A187" t="b">
-        <v>1</v>
-      </c>
-      <c r="B187" s="2"/>
-      <c r="C187" s="2"/>
-      <c r="D187" s="2" t="s">
-        <v>736</v>
-      </c>
-      <c r="E187" s="2" t="s">
-        <v>433</v>
-      </c>
-      <c r="F187" s="2"/>
-      <c r="G187" s="2"/>
-      <c r="H187" s="2"/>
-      <c r="I187" s="2" t="s">
-        <v>601</v>
-      </c>
-      <c r="J187" s="2"/>
-    </row>
-    <row r="188" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A188" t="b">
-        <v>1</v>
-      </c>
-      <c r="B188" s="2"/>
-      <c r="C188" s="2"/>
-      <c r="D188" s="2" t="s">
-        <v>736</v>
-      </c>
-      <c r="E188" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="F188" s="2"/>
-      <c r="G188" s="2"/>
-      <c r="H188" s="2"/>
-      <c r="I188" s="2" t="s">
-        <v>605</v>
-      </c>
-      <c r="J188" s="2"/>
-    </row>
-    <row r="189" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A189" t="b">
-        <v>1</v>
-      </c>
-      <c r="B189" s="2"/>
-      <c r="C189" s="2"/>
-      <c r="D189" s="2" t="s">
-        <v>737</v>
-      </c>
-      <c r="E189" s="2" t="s">
-        <v>423</v>
-      </c>
-      <c r="F189" s="2"/>
-      <c r="G189" s="2"/>
-      <c r="H189" s="2"/>
-      <c r="I189" s="2" t="s">
-        <v>598</v>
-      </c>
-      <c r="J189" s="2" t="s">
-        <v>738</v>
-      </c>
-    </row>
-    <row r="190" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A190" t="b">
-        <v>1</v>
-      </c>
-      <c r="B190" s="2"/>
-      <c r="C190" s="2"/>
-      <c r="D190" s="2" t="s">
-        <v>737</v>
-      </c>
-      <c r="E190" s="2" t="s">
-        <v>424</v>
-      </c>
-      <c r="F190" s="2"/>
-      <c r="G190" s="2"/>
-      <c r="H190" s="2"/>
-      <c r="I190" s="2" t="s">
-        <v>602</v>
-      </c>
-      <c r="J190" s="2"/>
-    </row>
-    <row r="191" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A191" t="b">
-        <v>1</v>
-      </c>
-      <c r="B191" s="2"/>
-      <c r="C191" s="2"/>
-      <c r="D191" s="2" t="s">
-        <v>737</v>
-      </c>
-      <c r="E191" s="2" t="s">
-        <v>425</v>
-      </c>
-      <c r="F191" s="2"/>
-      <c r="G191" s="2"/>
-      <c r="H191" s="2"/>
-      <c r="I191" s="2" t="s">
-        <v>599</v>
-      </c>
-      <c r="J191" s="2"/>
-    </row>
-    <row r="192" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A192" t="b">
-        <v>1</v>
-      </c>
-      <c r="B192" s="2"/>
-      <c r="C192" s="2"/>
-      <c r="D192" s="2" t="s">
-        <v>737</v>
-      </c>
-      <c r="E192" s="2" t="s">
-        <v>426</v>
-      </c>
-      <c r="F192" s="2"/>
-      <c r="G192" s="2"/>
-      <c r="H192" s="2"/>
-      <c r="I192" s="2" t="s">
-        <v>603</v>
-      </c>
-      <c r="J192" s="2"/>
-    </row>
-    <row r="193" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A193" t="b">
-        <v>1</v>
-      </c>
-      <c r="B193" s="2"/>
-      <c r="C193" s="2"/>
-      <c r="D193" s="2" t="s">
-        <v>737</v>
-      </c>
-      <c r="E193" s="2" t="s">
-        <v>427</v>
-      </c>
-      <c r="F193" s="2"/>
-      <c r="G193" s="2"/>
-      <c r="H193" s="2"/>
-      <c r="I193" s="2" t="s">
-        <v>599</v>
-      </c>
-      <c r="J193" s="2"/>
-    </row>
-    <row r="194" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A194" t="b">
-        <v>1</v>
-      </c>
-      <c r="B194" s="2"/>
-      <c r="C194" s="2"/>
-      <c r="D194" s="2" t="s">
-        <v>737</v>
-      </c>
-      <c r="E194" s="2" t="s">
-        <v>428</v>
-      </c>
-      <c r="F194" s="2"/>
-      <c r="G194" s="2"/>
-      <c r="H194" s="2"/>
-      <c r="I194" s="2" t="s">
-        <v>603</v>
-      </c>
-      <c r="J194" s="2"/>
-    </row>
-    <row r="195" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A195" t="b">
-        <v>1</v>
-      </c>
-      <c r="B195" s="2"/>
-      <c r="C195" s="2"/>
-      <c r="D195" s="2" t="s">
-        <v>737</v>
-      </c>
-      <c r="E195" s="2" t="s">
-        <v>429</v>
-      </c>
-      <c r="F195" s="2"/>
-      <c r="G195" s="2"/>
-      <c r="H195" s="2"/>
-      <c r="I195" s="2" t="s">
-        <v>600</v>
-      </c>
-      <c r="J195" s="2"/>
-    </row>
-    <row r="196" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A196" t="b">
-        <v>1</v>
-      </c>
-      <c r="B196" s="2"/>
-      <c r="C196" s="2"/>
-      <c r="D196" s="2" t="s">
-        <v>737</v>
-      </c>
-      <c r="E196" s="2" t="s">
-        <v>430</v>
-      </c>
-      <c r="F196" s="2"/>
-      <c r="G196" s="2"/>
-      <c r="H196" s="2"/>
-      <c r="I196" s="2" t="s">
-        <v>604</v>
-      </c>
-      <c r="J196" s="2"/>
-    </row>
-    <row r="197" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A197" t="b">
-        <v>1</v>
-      </c>
-      <c r="B197" s="2"/>
-      <c r="C197" s="2"/>
-      <c r="D197" s="2" t="s">
-        <v>737</v>
-      </c>
-      <c r="E197" s="2" t="s">
-        <v>431</v>
-      </c>
-      <c r="F197" s="2"/>
-      <c r="G197" s="2"/>
-      <c r="H197" s="2"/>
-      <c r="I197" s="2" t="s">
-        <v>601</v>
-      </c>
-      <c r="J197" s="2"/>
-    </row>
-    <row r="198" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A198" t="b">
-        <v>1</v>
-      </c>
-      <c r="B198" s="2"/>
-      <c r="C198" s="2"/>
-      <c r="D198" s="2" t="s">
-        <v>737</v>
-      </c>
-      <c r="E198" s="2" t="s">
-        <v>432</v>
-      </c>
-      <c r="F198" s="2"/>
-      <c r="G198" s="2"/>
-      <c r="H198" s="2"/>
-      <c r="I198" s="2" t="s">
-        <v>605</v>
-      </c>
-      <c r="J198" s="2"/>
-    </row>
-    <row r="199" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A199" t="b">
-        <v>1</v>
-      </c>
-      <c r="B199" s="2"/>
-      <c r="C199" s="2"/>
-      <c r="D199" s="2" t="s">
-        <v>737</v>
-      </c>
-      <c r="E199" s="2" t="s">
-        <v>433</v>
-      </c>
-      <c r="F199" s="2"/>
-      <c r="G199" s="2"/>
-      <c r="H199" s="2"/>
-      <c r="I199" s="2" t="s">
-        <v>601</v>
-      </c>
-      <c r="J199" s="2"/>
-    </row>
-    <row r="200" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A200" t="b">
-        <v>1</v>
-      </c>
-      <c r="B200" s="2"/>
-      <c r="C200" s="2"/>
-      <c r="D200" s="2" t="s">
-        <v>737</v>
-      </c>
-      <c r="E200" s="2" t="s">
-        <v>434</v>
-      </c>
-      <c r="F200" s="2"/>
-      <c r="G200" s="2"/>
-      <c r="H200" s="2"/>
-      <c r="I200" s="2" t="s">
-        <v>605</v>
-      </c>
-      <c r="J200" s="2"/>
-    </row>
-    <row r="201" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A201" t="b">
-        <v>1</v>
-      </c>
-      <c r="B201" s="2"/>
-      <c r="C201" s="2"/>
-      <c r="D201" s="2" t="s">
-        <v>737</v>
-      </c>
-      <c r="E201" s="2" t="s">
-        <v>149</v>
-      </c>
-      <c r="F201" s="2"/>
-      <c r="G201" s="2"/>
-      <c r="H201" s="2"/>
-      <c r="I201" s="2" t="s">
-        <v>612</v>
-      </c>
-      <c r="J201" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Fixed up epaid and epaid_registry_id
</commit_message>
<xml_diff>
--- a/data/mapping_config_files/NWSS-to-ODM-dictionary.xlsx
+++ b/data/mapping_config_files/NWSS-to-ODM-dictionary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-MapGenerator/PHES-ODM-MapGenerator/data/mapping_config_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A1816F2-5BAC-5D45-A7BD-F675F4EBA2A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AADC31C-A064-044E-A948-9802024BE138}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="280" yWindow="500" windowWidth="39840" windowHeight="19600" activeTab="2" xr2:uid="{77810E24-F86B-BC44-A0D5-8790E6EC60B4}"/>
+    <workbookView xWindow="280" yWindow="500" windowWidth="39840" windowHeight="19600" xr2:uid="{77810E24-F86B-BC44-A0D5-8790E6EC60B4}"/>
   </bookViews>
   <sheets>
     <sheet name="maps" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
     <externalReference r:id="rId4"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">maps!$B$1:$K$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">maps!$A$1:$L$6</definedName>
     <definedName name="partID">[1]parts!$A:$A</definedName>
     <definedName name="partLabel">[1]parts!$B:$B</definedName>
   </definedNames>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2507" uniqueCount="766">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2391" uniqueCount="768">
   <si>
     <t>Reporter</t>
   </si>
@@ -2208,9 +2208,6 @@
   </si>
   <si>
     <t>Same targets: reporting_jurisdiction, wwtp_jurisdiction</t>
-  </si>
-  <si>
-    <t>Same targets: epaid, epa_registry_id</t>
   </si>
   <si>
     <t>wideOtherSlots</t>
@@ -2364,6 +2361,15 @@
   </si>
   <si>
     <t>For source slot pcr_target_units</t>
+  </si>
+  <si>
+    <t>{{epaid}}</t>
+  </si>
+  <si>
+    <t>{{epa_registry_id}}</t>
+  </si>
+  <si>
+    <t>Same targets: epaid, epa_registry_id, epaid, epaid_registry_id</t>
   </si>
 </sst>
 </file>
@@ -13510,30 +13516,30 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
-      <sheetData sheetId="5" refreshError="1"/>
-      <sheetData sheetId="6" refreshError="1"/>
-      <sheetData sheetId="7" refreshError="1"/>
-      <sheetData sheetId="8" refreshError="1"/>
-      <sheetData sheetId="9" refreshError="1"/>
-      <sheetData sheetId="10" refreshError="1"/>
-      <sheetData sheetId="11" refreshError="1"/>
-      <sheetData sheetId="12" refreshError="1"/>
-      <sheetData sheetId="13" refreshError="1"/>
-      <sheetData sheetId="14" refreshError="1"/>
-      <sheetData sheetId="15" refreshError="1"/>
-      <sheetData sheetId="16" refreshError="1"/>
-      <sheetData sheetId="17" refreshError="1"/>
-      <sheetData sheetId="18" refreshError="1"/>
-      <sheetData sheetId="19" refreshError="1"/>
-      <sheetData sheetId="20" refreshError="1"/>
-      <sheetData sheetId="21" refreshError="1"/>
-      <sheetData sheetId="22" refreshError="1"/>
-      <sheetData sheetId="23" refreshError="1"/>
-      <sheetData sheetId="24" refreshError="1"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
+      <sheetData sheetId="8"/>
+      <sheetData sheetId="9"/>
+      <sheetData sheetId="10"/>
+      <sheetData sheetId="11"/>
+      <sheetData sheetId="12"/>
+      <sheetData sheetId="13"/>
+      <sheetData sheetId="14"/>
+      <sheetData sheetId="15"/>
+      <sheetData sheetId="16"/>
+      <sheetData sheetId="17"/>
+      <sheetData sheetId="18"/>
+      <sheetData sheetId="19"/>
+      <sheetData sheetId="20"/>
+      <sheetData sheetId="21"/>
+      <sheetData sheetId="22"/>
+      <sheetData sheetId="23"/>
+      <sheetData sheetId="24"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -13927,7 +13933,7 @@
         <v>121</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
@@ -13961,7 +13967,7 @@
         <v>82</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
@@ -13990,13 +13996,16 @@
         <v>127</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>740</v>
+        <v>739</v>
       </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
       <c r="K4" s="1" t="s">
         <v>629</v>
       </c>
+      <c r="L4" s="19" t="s">
+        <v>767</v>
+      </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" t="b">
@@ -14021,7 +14030,7 @@
         <v>84</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>741</v>
+        <v>740</v>
       </c>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
@@ -14050,7 +14059,7 @@
         <v>85</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>742</v>
+        <v>741</v>
       </c>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
@@ -14153,7 +14162,7 @@
       <c r="J10" s="6"/>
       <c r="K10" s="2"/>
       <c r="L10" s="22" t="s">
-        <v>754</v>
+        <v>753</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.2">
@@ -14314,7 +14323,7 @@
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A17" t="b">
         <v>1</v>
       </c>
@@ -14343,7 +14352,7 @@
       <c r="J17" s="2"/>
       <c r="K17" s="2"/>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A18" t="b">
         <v>1</v>
       </c>
@@ -14372,7 +14381,7 @@
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A19" t="b">
         <v>1</v>
       </c>
@@ -14401,7 +14410,7 @@
       <c r="J19" s="2"/>
       <c r="K19" s="2"/>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A20" t="b">
         <v>1</v>
       </c>
@@ -14430,7 +14439,7 @@
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A21" t="b">
         <v>1</v>
       </c>
@@ -14459,7 +14468,7 @@
       <c r="J21" s="2"/>
       <c r="K21" s="2"/>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A22" t="b">
         <v>1</v>
       </c>
@@ -14488,7 +14497,7 @@
       <c r="J22" s="2"/>
       <c r="K22" s="2"/>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A23" t="b">
         <v>1</v>
       </c>
@@ -14517,7 +14526,7 @@
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A24" t="b">
         <v>1</v>
       </c>
@@ -14546,7 +14555,7 @@
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A25" t="b">
         <v>1</v>
       </c>
@@ -14575,7 +14584,7 @@
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A26" t="b">
         <v>1</v>
       </c>
@@ -14604,7 +14613,7 @@
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A27" t="b">
         <v>1</v>
       </c>
@@ -14633,7 +14642,7 @@
       <c r="J27" s="6"/>
       <c r="K27" s="2"/>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B28" s="2"/>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
@@ -14645,9 +14654,9 @@
       <c r="J28" s="6"/>
       <c r="K28" s="2"/>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A29" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>2</v>
@@ -14663,21 +14672,18 @@
         <v>81</v>
       </c>
       <c r="G29" s="2" t="s">
-        <v>81</v>
+        <v>127</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>127</v>
+        <v>765</v>
       </c>
       <c r="I29" s="2"/>
       <c r="J29" s="2"/>
       <c r="K29" s="7" t="s">
         <v>123</v>
       </c>
-      <c r="L29" s="19" t="s">
-        <v>721</v>
-      </c>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" t="b">
         <v>0</v>
       </c>
@@ -14695,10 +14701,10 @@
         <v>81</v>
       </c>
       <c r="G30" s="2" t="s">
-        <v>81</v>
+        <v>127</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>127</v>
+        <v>766</v>
       </c>
       <c r="I30" s="2"/>
       <c r="J30" s="2"/>
@@ -14706,7 +14712,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A31" t="b">
         <v>1</v>
       </c>
@@ -14727,13 +14733,13 @@
         <v>122</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>743</v>
+        <v>742</v>
       </c>
       <c r="I31" s="2"/>
       <c r="J31" s="2"/>
       <c r="K31" s="2"/>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" t="b">
         <v>0</v>
       </c>
@@ -14754,7 +14760,7 @@
         <v>121</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>744</v>
+        <v>743</v>
       </c>
       <c r="I32" s="2"/>
       <c r="J32" s="2"/>
@@ -14780,7 +14786,7 @@
       </c>
       <c r="H33" s="6"/>
       <c r="I33" s="20" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="J33" s="2"/>
       <c r="K33" s="2"/>
@@ -14805,7 +14811,7 @@
       </c>
       <c r="H34" s="2"/>
       <c r="I34" s="20" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="J34" s="2"/>
       <c r="K34" s="2"/>
@@ -14833,7 +14839,7 @@
         <v>126</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>745</v>
+        <v>744</v>
       </c>
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
@@ -15116,13 +15122,13 @@
         <v>160</v>
       </c>
       <c r="H46" s="2" t="s">
-        <v>746</v>
+        <v>745</v>
       </c>
       <c r="I46" s="2"/>
       <c r="J46" s="2"/>
       <c r="K46" s="2"/>
       <c r="L46" s="19" t="s">
-        <v>755</v>
+        <v>754</v>
       </c>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.2">
@@ -15146,7 +15152,7 @@
         <v>160</v>
       </c>
       <c r="H47" s="2" t="s">
-        <v>747</v>
+        <v>746</v>
       </c>
       <c r="I47" s="2"/>
       <c r="J47" s="2"/>
@@ -15154,7 +15160,7 @@
         <v>596</v>
       </c>
       <c r="L47" s="19" t="s">
-        <v>757</v>
+        <v>756</v>
       </c>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.2">
@@ -15178,13 +15184,13 @@
         <v>160</v>
       </c>
       <c r="H48" s="2" t="s">
-        <v>748</v>
+        <v>747</v>
       </c>
       <c r="I48" s="2"/>
       <c r="J48" s="2"/>
       <c r="K48" s="2"/>
       <c r="L48" s="22" t="s">
-        <v>756</v>
+        <v>755</v>
       </c>
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.2">
@@ -15322,7 +15328,7 @@
         <v>146</v>
       </c>
       <c r="H54" s="2" t="s">
-        <v>749</v>
+        <v>748</v>
       </c>
       <c r="I54" s="2"/>
       <c r="J54" s="2"/>
@@ -15351,7 +15357,7 @@
         <v>150</v>
       </c>
       <c r="H55" s="2" t="s">
-        <v>750</v>
+        <v>749</v>
       </c>
       <c r="I55" s="2"/>
       <c r="J55" s="2"/>
@@ -15708,7 +15714,7 @@
         <v>169</v>
       </c>
       <c r="H69" s="2" t="s">
-        <v>751</v>
+        <v>750</v>
       </c>
       <c r="I69" s="2"/>
       <c r="J69" s="2"/>
@@ -16238,7 +16244,7 @@
         <v>486</v>
       </c>
       <c r="H90" s="2" t="s">
-        <v>752</v>
+        <v>751</v>
       </c>
       <c r="I90" s="2"/>
       <c r="J90" s="2"/>
@@ -16265,17 +16271,17 @@
         <v>488</v>
       </c>
       <c r="H91" s="2" t="s">
-        <v>753</v>
+        <v>752</v>
       </c>
       <c r="I91" s="2"/>
       <c r="J91" s="2"/>
       <c r="K91" s="2"/>
       <c r="L91" s="22" t="s">
-        <v>759</v>
+        <v>758</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B1:K1" xr:uid="{3154BFCE-06D9-9649-B340-B23DCF20DD83}"/>
+  <autoFilter ref="A1:L6" xr:uid="{3154BFCE-06D9-9649-B340-B23DCF20DD83}"/>
   <conditionalFormatting sqref="H37:J37">
     <cfRule type="duplicateValues" dxfId="8" priority="10"/>
   </conditionalFormatting>
@@ -16320,7 +16326,7 @@
         <v>704</v>
       </c>
       <c r="G1" s="9" t="s">
-        <v>722</v>
+        <v>721</v>
       </c>
       <c r="H1" s="11" t="s">
         <v>167</v>
@@ -16590,7 +16596,7 @@
         <v>665</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>723</v>
+        <v>722</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>177</v>
@@ -20947,7 +20953,7 @@
         <v>665</v>
       </c>
       <c r="G128" s="2" t="s">
-        <v>724</v>
+        <v>723</v>
       </c>
       <c r="H128" s="2" t="s">
         <v>177</v>
@@ -20968,7 +20974,7 @@
         <v>171</v>
       </c>
       <c r="N128" s="2" t="s">
-        <v>758</v>
+        <v>757</v>
       </c>
     </row>
     <row r="129" spans="1:14" x14ac:dyDescent="0.2">
@@ -21189,7 +21195,7 @@
         <v>665</v>
       </c>
       <c r="G134" s="2" t="s">
-        <v>728</v>
+        <v>727</v>
       </c>
       <c r="H134" s="2" t="s">
         <v>177</v>
@@ -21229,7 +21235,7 @@
         <v>665</v>
       </c>
       <c r="G135" s="2" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="H135" s="2" t="s">
         <v>177</v>
@@ -21269,7 +21275,7 @@
         <v>665</v>
       </c>
       <c r="G136" s="2" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="H136" s="2" t="s">
         <v>177</v>
@@ -21327,11 +21333,13 @@
   <dimension ref="A1:J185"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.83203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="22.5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="25.5" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="25.5" customWidth="1"/>
     <col min="8" max="8" width="12.5" customWidth="1"/>
+    <col min="9" max="9" width="14.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" s="24" customFormat="1" ht="21" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -21370,12 +21378,10 @@
       <c r="A2" t="b">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>291</v>
@@ -21387,19 +21393,17 @@
         <v>521</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>761</v>
+        <v>760</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="b">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>292</v>
@@ -21416,12 +21420,10 @@
       <c r="A4" t="b">
         <v>1</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B4" s="2"/>
       <c r="C4" s="2"/>
       <c r="D4" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>293</v>
@@ -21438,12 +21440,10 @@
       <c r="A5" t="b">
         <v>1</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>294</v>
@@ -21460,12 +21460,10 @@
       <c r="A6" t="b">
         <v>1</v>
       </c>
-      <c r="B6" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B6" s="2"/>
       <c r="C6" s="2"/>
       <c r="D6" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>295</v>
@@ -21482,12 +21480,10 @@
       <c r="A7" t="b">
         <v>1</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B7" s="2"/>
       <c r="C7" s="2"/>
       <c r="D7" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>296</v>
@@ -21504,12 +21500,10 @@
       <c r="A8" t="b">
         <v>1</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B8" s="2"/>
       <c r="C8" s="2"/>
       <c r="D8" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>297</v>
@@ -21526,12 +21520,10 @@
       <c r="A9" t="b">
         <v>1</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B9" s="2"/>
       <c r="C9" s="2"/>
       <c r="D9" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>298</v>
@@ -21548,12 +21540,10 @@
       <c r="A10" t="b">
         <v>1</v>
       </c>
-      <c r="B10" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B10" s="2"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>299</v>
@@ -21570,12 +21560,10 @@
       <c r="A11" t="b">
         <v>1</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B11" s="2"/>
       <c r="C11" s="2"/>
       <c r="D11" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>300</v>
@@ -21592,12 +21580,10 @@
       <c r="A12" t="b">
         <v>1</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B12" s="2"/>
       <c r="C12" s="2"/>
       <c r="D12" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>301</v>
@@ -21614,12 +21600,10 @@
       <c r="A13" t="b">
         <v>1</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B13" s="2"/>
       <c r="C13" s="2"/>
       <c r="D13" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>302</v>
@@ -21636,12 +21620,10 @@
       <c r="A14" t="b">
         <v>1</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B14" s="2"/>
       <c r="C14" s="2"/>
       <c r="D14" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>303</v>
@@ -21658,12 +21640,10 @@
       <c r="A15" t="b">
         <v>1</v>
       </c>
-      <c r="B15" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B15" s="2"/>
       <c r="C15" s="2"/>
       <c r="D15" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>304</v>
@@ -21680,12 +21660,10 @@
       <c r="A16" t="b">
         <v>1</v>
       </c>
-      <c r="B16" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B16" s="2"/>
       <c r="C16" s="2"/>
       <c r="D16" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>305</v>
@@ -21702,12 +21680,10 @@
       <c r="A17" t="b">
         <v>1</v>
       </c>
-      <c r="B17" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B17" s="2"/>
       <c r="C17" s="2"/>
       <c r="D17" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>306</v>
@@ -21724,12 +21700,10 @@
       <c r="A18" t="b">
         <v>1</v>
       </c>
-      <c r="B18" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>307</v>
@@ -21746,12 +21720,10 @@
       <c r="A19" t="b">
         <v>1</v>
       </c>
-      <c r="B19" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B19" s="2"/>
       <c r="C19" s="2"/>
       <c r="D19" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>308</v>
@@ -21768,12 +21740,10 @@
       <c r="A20" t="b">
         <v>1</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>309</v>
@@ -21790,12 +21760,10 @@
       <c r="A21" t="b">
         <v>1</v>
       </c>
-      <c r="B21" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B21" s="2"/>
       <c r="C21" s="2"/>
       <c r="D21" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>310</v>
@@ -21812,12 +21780,10 @@
       <c r="A22" t="b">
         <v>1</v>
       </c>
-      <c r="B22" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B22" s="2"/>
       <c r="C22" s="2"/>
       <c r="D22" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>311</v>
@@ -21834,12 +21800,10 @@
       <c r="A23" t="b">
         <v>1</v>
       </c>
-      <c r="B23" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B23" s="2"/>
       <c r="C23" s="2"/>
       <c r="D23" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>312</v>
@@ -21856,12 +21820,10 @@
       <c r="A24" t="b">
         <v>1</v>
       </c>
-      <c r="B24" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B24" s="2"/>
       <c r="C24" s="2"/>
       <c r="D24" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>313</v>
@@ -21878,12 +21840,10 @@
       <c r="A25" t="b">
         <v>1</v>
       </c>
-      <c r="B25" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B25" s="2"/>
       <c r="C25" s="2"/>
       <c r="D25" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>314</v>
@@ -21900,12 +21860,10 @@
       <c r="A26" t="b">
         <v>1</v>
       </c>
-      <c r="B26" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B26" s="2"/>
       <c r="C26" s="2"/>
       <c r="D26" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>315</v>
@@ -21922,12 +21880,10 @@
       <c r="A27" t="b">
         <v>1</v>
       </c>
-      <c r="B27" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B27" s="2"/>
       <c r="C27" s="2"/>
       <c r="D27" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>322</v>
@@ -21944,12 +21900,10 @@
       <c r="A28" t="b">
         <v>1</v>
       </c>
-      <c r="B28" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B28" s="2"/>
       <c r="C28" s="2"/>
       <c r="D28" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>339</v>
@@ -21966,12 +21920,10 @@
       <c r="A29" t="b">
         <v>1</v>
       </c>
-      <c r="B29" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B29" s="2"/>
       <c r="C29" s="2"/>
       <c r="D29" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>370</v>
@@ -21988,12 +21940,10 @@
       <c r="A30" t="b">
         <v>1</v>
       </c>
-      <c r="B30" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B30" s="2"/>
       <c r="C30" s="2"/>
       <c r="D30" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>344</v>
@@ -22010,12 +21960,10 @@
       <c r="A31" t="b">
         <v>1</v>
       </c>
-      <c r="B31" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B31" s="2"/>
       <c r="C31" s="2"/>
       <c r="D31" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>346</v>
@@ -22032,12 +21980,10 @@
       <c r="A32" t="b">
         <v>1</v>
       </c>
-      <c r="B32" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B32" s="2"/>
       <c r="C32" s="2"/>
       <c r="D32" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>333</v>
@@ -22054,12 +22000,10 @@
       <c r="A33" t="b">
         <v>1</v>
       </c>
-      <c r="B33" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B33" s="2"/>
       <c r="C33" s="2"/>
       <c r="D33" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>368</v>
@@ -22076,12 +22020,10 @@
       <c r="A34" t="b">
         <v>1</v>
       </c>
-      <c r="B34" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B34" s="2"/>
       <c r="C34" s="2"/>
       <c r="D34" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>330</v>
@@ -22098,12 +22040,10 @@
       <c r="A35" t="b">
         <v>1</v>
       </c>
-      <c r="B35" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B35" s="2"/>
       <c r="C35" s="2"/>
       <c r="D35" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>362</v>
@@ -22120,12 +22060,10 @@
       <c r="A36" t="b">
         <v>1</v>
       </c>
-      <c r="B36" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B36" s="2"/>
       <c r="C36" s="2"/>
       <c r="D36" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>328</v>
@@ -22142,12 +22080,10 @@
       <c r="A37" t="b">
         <v>1</v>
       </c>
-      <c r="B37" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B37" s="2"/>
       <c r="C37" s="2"/>
       <c r="D37" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>325</v>
@@ -22164,12 +22100,10 @@
       <c r="A38" t="b">
         <v>1</v>
       </c>
-      <c r="B38" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B38" s="2"/>
       <c r="C38" s="2"/>
       <c r="D38" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E38" s="2" t="s">
         <v>372</v>
@@ -22186,12 +22120,10 @@
       <c r="A39" t="b">
         <v>1</v>
       </c>
-      <c r="B39" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B39" s="2"/>
       <c r="C39" s="2"/>
       <c r="D39" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>347</v>
@@ -22208,12 +22140,10 @@
       <c r="A40" t="b">
         <v>1</v>
       </c>
-      <c r="B40" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B40" s="2"/>
       <c r="C40" s="2"/>
       <c r="D40" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>335</v>
@@ -22230,12 +22160,10 @@
       <c r="A41" t="b">
         <v>1</v>
       </c>
-      <c r="B41" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B41" s="2"/>
       <c r="C41" s="2"/>
       <c r="D41" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>338</v>
@@ -22252,12 +22180,10 @@
       <c r="A42" t="b">
         <v>1</v>
       </c>
-      <c r="B42" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B42" s="2"/>
       <c r="C42" s="2"/>
       <c r="D42" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E42" s="2" t="s">
         <v>349</v>
@@ -22274,12 +22200,10 @@
       <c r="A43" t="b">
         <v>1</v>
       </c>
-      <c r="B43" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B43" s="2"/>
       <c r="C43" s="2"/>
       <c r="D43" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E43" s="2" t="s">
         <v>373</v>
@@ -22296,12 +22220,10 @@
       <c r="A44" t="b">
         <v>1</v>
       </c>
-      <c r="B44" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B44" s="2"/>
       <c r="C44" s="2"/>
       <c r="D44" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>341</v>
@@ -22318,12 +22240,10 @@
       <c r="A45" t="b">
         <v>1</v>
       </c>
-      <c r="B45" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B45" s="2"/>
       <c r="C45" s="2"/>
       <c r="D45" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E45" s="2" t="s">
         <v>345</v>
@@ -22340,12 +22260,10 @@
       <c r="A46" t="b">
         <v>1</v>
       </c>
-      <c r="B46" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B46" s="2"/>
       <c r="C46" s="2"/>
       <c r="D46" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E46" s="2" t="s">
         <v>324</v>
@@ -22362,12 +22280,10 @@
       <c r="A47" t="b">
         <v>1</v>
       </c>
-      <c r="B47" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B47" s="2"/>
       <c r="C47" s="2"/>
       <c r="D47" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E47" s="2" t="s">
         <v>355</v>
@@ -22384,12 +22300,10 @@
       <c r="A48" t="b">
         <v>1</v>
       </c>
-      <c r="B48" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B48" s="2"/>
       <c r="C48" s="2"/>
       <c r="D48" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E48" s="2" t="s">
         <v>332</v>
@@ -22406,12 +22320,10 @@
       <c r="A49" t="b">
         <v>1</v>
       </c>
-      <c r="B49" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B49" s="2"/>
       <c r="C49" s="2"/>
       <c r="D49" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E49" s="2" t="s">
         <v>350</v>
@@ -22428,12 +22340,10 @@
       <c r="A50" t="b">
         <v>1</v>
       </c>
-      <c r="B50" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B50" s="2"/>
       <c r="C50" s="2"/>
       <c r="D50" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E50" s="2" t="s">
         <v>357</v>
@@ -22450,12 +22360,10 @@
       <c r="A51" t="b">
         <v>1</v>
       </c>
-      <c r="B51" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B51" s="2"/>
       <c r="C51" s="2"/>
       <c r="D51" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E51" s="2" t="s">
         <v>320</v>
@@ -22472,12 +22380,10 @@
       <c r="A52" t="b">
         <v>1</v>
       </c>
-      <c r="B52" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B52" s="2"/>
       <c r="C52" s="2"/>
       <c r="D52" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E52" s="2" t="s">
         <v>343</v>
@@ -22494,12 +22400,10 @@
       <c r="A53" t="b">
         <v>1</v>
       </c>
-      <c r="B53" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B53" s="2"/>
       <c r="C53" s="2"/>
       <c r="D53" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E53" s="2" t="s">
         <v>342</v>
@@ -22516,12 +22420,10 @@
       <c r="A54" t="b">
         <v>1</v>
       </c>
-      <c r="B54" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B54" s="2"/>
       <c r="C54" s="2"/>
       <c r="D54" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>329</v>
@@ -22538,12 +22440,10 @@
       <c r="A55" t="b">
         <v>1</v>
       </c>
-      <c r="B55" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B55" s="2"/>
       <c r="C55" s="2"/>
       <c r="D55" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E55" s="2" t="s">
         <v>371</v>
@@ -22560,12 +22460,10 @@
       <c r="A56" t="b">
         <v>1</v>
       </c>
-      <c r="B56" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B56" s="2"/>
       <c r="C56" s="2"/>
       <c r="D56" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E56" s="2" t="s">
         <v>336</v>
@@ -22582,12 +22480,10 @@
       <c r="A57" t="b">
         <v>1</v>
       </c>
-      <c r="B57" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B57" s="2"/>
       <c r="C57" s="2"/>
       <c r="D57" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E57" s="2" t="s">
         <v>374</v>
@@ -22604,12 +22500,10 @@
       <c r="A58" t="b">
         <v>1</v>
       </c>
-      <c r="B58" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B58" s="2"/>
       <c r="C58" s="2"/>
       <c r="D58" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>326</v>
@@ -22626,12 +22520,10 @@
       <c r="A59" t="b">
         <v>1</v>
       </c>
-      <c r="B59" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B59" s="2"/>
       <c r="C59" s="2"/>
       <c r="D59" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E59" s="2" t="s">
         <v>366</v>
@@ -22648,12 +22540,10 @@
       <c r="A60" t="b">
         <v>1</v>
       </c>
-      <c r="B60" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B60" s="2"/>
       <c r="C60" s="2"/>
       <c r="D60" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E60" s="2" t="s">
         <v>375</v>
@@ -22670,12 +22560,10 @@
       <c r="A61" t="b">
         <v>1</v>
       </c>
-      <c r="B61" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B61" s="2"/>
       <c r="C61" s="2"/>
       <c r="D61" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E61" s="2" t="s">
         <v>348</v>
@@ -22692,12 +22580,10 @@
       <c r="A62" t="b">
         <v>1</v>
       </c>
-      <c r="B62" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B62" s="2"/>
       <c r="C62" s="2"/>
       <c r="D62" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E62" s="2" t="s">
         <v>361</v>
@@ -22714,12 +22600,10 @@
       <c r="A63" t="b">
         <v>1</v>
       </c>
-      <c r="B63" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B63" s="2"/>
       <c r="C63" s="2"/>
       <c r="D63" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E63" s="2" t="s">
         <v>363</v>
@@ -22736,12 +22620,10 @@
       <c r="A64" t="b">
         <v>1</v>
       </c>
-      <c r="B64" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B64" s="2"/>
       <c r="C64" s="2"/>
       <c r="D64" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E64" s="2" t="s">
         <v>365</v>
@@ -22758,12 +22640,10 @@
       <c r="A65" t="b">
         <v>1</v>
       </c>
-      <c r="B65" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B65" s="2"/>
       <c r="C65" s="2"/>
       <c r="D65" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E65" s="2" t="s">
         <v>321</v>
@@ -22780,12 +22660,10 @@
       <c r="A66" t="b">
         <v>1</v>
       </c>
-      <c r="B66" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B66" s="2"/>
       <c r="C66" s="2"/>
       <c r="D66" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E66" s="2" t="s">
         <v>376</v>
@@ -22802,12 +22680,10 @@
       <c r="A67" t="b">
         <v>1</v>
       </c>
-      <c r="B67" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B67" s="2"/>
       <c r="C67" s="2"/>
       <c r="D67" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E67" s="2" t="s">
         <v>316</v>
@@ -22824,12 +22700,10 @@
       <c r="A68" t="b">
         <v>1</v>
       </c>
-      <c r="B68" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B68" s="2"/>
       <c r="C68" s="2"/>
       <c r="D68" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E68" s="2" t="s">
         <v>317</v>
@@ -22846,12 +22720,10 @@
       <c r="A69" t="b">
         <v>1</v>
       </c>
-      <c r="B69" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B69" s="2"/>
       <c r="C69" s="2"/>
       <c r="D69" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E69" s="2" t="s">
         <v>340</v>
@@ -22868,12 +22740,10 @@
       <c r="A70" t="b">
         <v>1</v>
       </c>
-      <c r="B70" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B70" s="2"/>
       <c r="C70" s="2"/>
       <c r="D70" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E70" s="2" t="s">
         <v>327</v>
@@ -22890,12 +22760,10 @@
       <c r="A71" t="b">
         <v>1</v>
       </c>
-      <c r="B71" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B71" s="2"/>
       <c r="C71" s="2"/>
       <c r="D71" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E71" s="2" t="s">
         <v>369</v>
@@ -22912,12 +22780,10 @@
       <c r="A72" t="b">
         <v>1</v>
       </c>
-      <c r="B72" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B72" s="2"/>
       <c r="C72" s="2"/>
       <c r="D72" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E72" s="2" t="s">
         <v>356</v>
@@ -22934,12 +22800,10 @@
       <c r="A73" t="b">
         <v>1</v>
       </c>
-      <c r="B73" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B73" s="2"/>
       <c r="C73" s="2"/>
       <c r="D73" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E73" s="2" t="s">
         <v>358</v>
@@ -22956,12 +22820,10 @@
       <c r="A74" t="b">
         <v>1</v>
       </c>
-      <c r="B74" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B74" s="2"/>
       <c r="C74" s="2"/>
       <c r="D74" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E74" s="2" t="s">
         <v>364</v>
@@ -22978,12 +22840,10 @@
       <c r="A75" t="b">
         <v>1</v>
       </c>
-      <c r="B75" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B75" s="2"/>
       <c r="C75" s="2"/>
       <c r="D75" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E75" s="2" t="s">
         <v>331</v>
@@ -23000,12 +22860,10 @@
       <c r="A76" t="b">
         <v>1</v>
       </c>
-      <c r="B76" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B76" s="2"/>
       <c r="C76" s="2"/>
       <c r="D76" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E76" s="2" t="s">
         <v>337</v>
@@ -23022,12 +22880,10 @@
       <c r="A77" t="b">
         <v>1</v>
       </c>
-      <c r="B77" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B77" s="2"/>
       <c r="C77" s="2"/>
       <c r="D77" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E77" s="2" t="s">
         <v>351</v>
@@ -23044,12 +22900,10 @@
       <c r="A78" t="b">
         <v>1</v>
       </c>
-      <c r="B78" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B78" s="2"/>
       <c r="C78" s="2"/>
       <c r="D78" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E78" s="2" t="s">
         <v>352</v>
@@ -23066,12 +22920,10 @@
       <c r="A79" t="b">
         <v>1</v>
       </c>
-      <c r="B79" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B79" s="2"/>
       <c r="C79" s="2"/>
       <c r="D79" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E79" s="2" t="s">
         <v>353</v>
@@ -23088,12 +22940,10 @@
       <c r="A80" t="b">
         <v>1</v>
       </c>
-      <c r="B80" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B80" s="2"/>
       <c r="C80" s="2"/>
       <c r="D80" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E80" s="2" t="s">
         <v>354</v>
@@ -23110,12 +22960,10 @@
       <c r="A81" t="b">
         <v>1</v>
       </c>
-      <c r="B81" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B81" s="2"/>
       <c r="C81" s="2"/>
       <c r="D81" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E81" s="2" t="s">
         <v>323</v>
@@ -23132,12 +22980,10 @@
       <c r="A82" t="b">
         <v>1</v>
       </c>
-      <c r="B82" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B82" s="2"/>
       <c r="C82" s="2"/>
       <c r="D82" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E82" s="2" t="s">
         <v>318</v>
@@ -23154,12 +23000,10 @@
       <c r="A83" t="b">
         <v>1</v>
       </c>
-      <c r="B83" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B83" s="2"/>
       <c r="C83" s="2"/>
       <c r="D83" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E83" s="2" t="s">
         <v>360</v>
@@ -23176,12 +23020,10 @@
       <c r="A84" t="b">
         <v>1</v>
       </c>
-      <c r="B84" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B84" s="2"/>
       <c r="C84" s="2"/>
       <c r="D84" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E84" s="2" t="s">
         <v>367</v>
@@ -23198,12 +23040,10 @@
       <c r="A85" t="b">
         <v>1</v>
       </c>
-      <c r="B85" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B85" s="2"/>
       <c r="C85" s="2"/>
       <c r="D85" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E85" s="2" t="s">
         <v>319</v>
@@ -23220,12 +23060,10 @@
       <c r="A86" t="b">
         <v>1</v>
       </c>
-      <c r="B86" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B86" s="2"/>
       <c r="C86" s="2"/>
       <c r="D86" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E86" s="2" t="s">
         <v>334</v>
@@ -23242,12 +23080,10 @@
       <c r="A87" t="b">
         <v>1</v>
       </c>
-      <c r="B87" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B87" s="2"/>
       <c r="C87" s="2"/>
       <c r="D87" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E87" s="2" t="s">
         <v>359</v>
@@ -23264,12 +23100,10 @@
       <c r="A88" t="b">
         <v>1</v>
       </c>
-      <c r="B88" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B88" s="2"/>
       <c r="C88" s="2"/>
       <c r="D88" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E88" s="2" t="s">
         <v>377</v>
@@ -23286,12 +23120,10 @@
       <c r="A89" t="b">
         <v>1</v>
       </c>
-      <c r="B89" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B89" s="2"/>
       <c r="C89" s="2"/>
       <c r="D89" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E89" s="2" t="s">
         <v>378</v>
@@ -23308,12 +23140,10 @@
       <c r="A90" t="b">
         <v>1</v>
       </c>
-      <c r="B90" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B90" s="2"/>
       <c r="C90" s="2"/>
       <c r="D90" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E90" s="2" t="s">
         <v>379</v>
@@ -23330,12 +23160,10 @@
       <c r="A91" t="b">
         <v>1</v>
       </c>
-      <c r="B91" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B91" s="2"/>
       <c r="C91" s="2"/>
       <c r="D91" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E91" s="2" t="s">
         <v>380</v>
@@ -23352,12 +23180,10 @@
       <c r="A92" t="b">
         <v>1</v>
       </c>
-      <c r="B92" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B92" s="2"/>
       <c r="C92" s="2"/>
       <c r="D92" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E92" s="2" t="s">
         <v>381</v>
@@ -23374,12 +23200,10 @@
       <c r="A93" t="b">
         <v>1</v>
       </c>
-      <c r="B93" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B93" s="2"/>
       <c r="C93" s="2"/>
       <c r="D93" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E93" s="2" t="s">
         <v>382</v>
@@ -23396,12 +23220,10 @@
       <c r="A94" t="b">
         <v>1</v>
       </c>
-      <c r="B94" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B94" s="2"/>
       <c r="C94" s="2"/>
       <c r="D94" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E94" s="2" t="s">
         <v>383</v>
@@ -23418,12 +23240,10 @@
       <c r="A95" t="b">
         <v>1</v>
       </c>
-      <c r="B95" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B95" s="2"/>
       <c r="C95" s="2"/>
       <c r="D95" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E95" s="2" t="s">
         <v>384</v>
@@ -23440,12 +23260,10 @@
       <c r="A96" t="b">
         <v>1</v>
       </c>
-      <c r="B96" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B96" s="2"/>
       <c r="C96" s="2"/>
       <c r="D96" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E96" s="2" t="s">
         <v>385</v>
@@ -23462,12 +23280,10 @@
       <c r="A97" t="b">
         <v>1</v>
       </c>
-      <c r="B97" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B97" s="2"/>
       <c r="C97" s="2"/>
       <c r="D97" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E97" s="2" t="s">
         <v>386</v>
@@ -23484,12 +23300,10 @@
       <c r="A98" t="b">
         <v>1</v>
       </c>
-      <c r="B98" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B98" s="2"/>
       <c r="C98" s="2"/>
       <c r="D98" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E98" s="2" t="s">
         <v>387</v>
@@ -23506,12 +23320,10 @@
       <c r="A99" t="b">
         <v>1</v>
       </c>
-      <c r="B99" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B99" s="2"/>
       <c r="C99" s="2"/>
       <c r="D99" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E99" s="2" t="s">
         <v>388</v>
@@ -23528,12 +23340,10 @@
       <c r="A100" t="b">
         <v>1</v>
       </c>
-      <c r="B100" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B100" s="2"/>
       <c r="C100" s="2"/>
       <c r="D100" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E100" s="2" t="s">
         <v>389</v>
@@ -23550,12 +23360,10 @@
       <c r="A101" t="b">
         <v>1</v>
       </c>
-      <c r="B101" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B101" s="2"/>
       <c r="C101" s="2"/>
       <c r="D101" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E101" s="2" t="s">
         <v>390</v>
@@ -23572,12 +23380,10 @@
       <c r="A102" t="b">
         <v>1</v>
       </c>
-      <c r="B102" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B102" s="2"/>
       <c r="C102" s="2"/>
       <c r="D102" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E102" s="2" t="s">
         <v>391</v>
@@ -23594,12 +23400,10 @@
       <c r="A103" t="b">
         <v>1</v>
       </c>
-      <c r="B103" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B103" s="2"/>
       <c r="C103" s="2"/>
       <c r="D103" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E103" s="2" t="s">
         <v>392</v>
@@ -23616,12 +23420,10 @@
       <c r="A104" t="b">
         <v>1</v>
       </c>
-      <c r="B104" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B104" s="2"/>
       <c r="C104" s="2"/>
       <c r="D104" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E104" s="2" t="s">
         <v>393</v>
@@ -23638,12 +23440,10 @@
       <c r="A105" t="b">
         <v>1</v>
       </c>
-      <c r="B105" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B105" s="2"/>
       <c r="C105" s="2"/>
       <c r="D105" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E105" s="2" t="s">
         <v>394</v>
@@ -23660,12 +23460,10 @@
       <c r="A106" t="b">
         <v>1</v>
       </c>
-      <c r="B106" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B106" s="2"/>
       <c r="C106" s="2"/>
       <c r="D106" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E106" s="2" t="s">
         <v>395</v>
@@ -23682,12 +23480,10 @@
       <c r="A107" t="b">
         <v>1</v>
       </c>
-      <c r="B107" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B107" s="2"/>
       <c r="C107" s="2"/>
       <c r="D107" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E107" s="2" t="s">
         <v>396</v>
@@ -23704,12 +23500,10 @@
       <c r="A108" t="b">
         <v>1</v>
       </c>
-      <c r="B108" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B108" s="2"/>
       <c r="C108" s="2"/>
       <c r="D108" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E108" s="2" t="s">
         <v>277</v>
@@ -23726,12 +23520,10 @@
       <c r="A109" t="b">
         <v>1</v>
       </c>
-      <c r="B109" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B109" s="2"/>
       <c r="C109" s="2"/>
       <c r="D109" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E109" s="2" t="s">
         <v>278</v>
@@ -23748,12 +23540,10 @@
       <c r="A110" t="b">
         <v>1</v>
       </c>
-      <c r="B110" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B110" s="2"/>
       <c r="C110" s="2"/>
       <c r="D110" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E110" s="2" t="s">
         <v>279</v>
@@ -23770,12 +23560,10 @@
       <c r="A111" t="b">
         <v>1</v>
       </c>
-      <c r="B111" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B111" s="2"/>
       <c r="C111" s="2"/>
       <c r="D111" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E111" s="2" t="s">
         <v>397</v>
@@ -23792,12 +23580,10 @@
       <c r="A112" t="b">
         <v>1</v>
       </c>
-      <c r="B112" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B112" s="2"/>
       <c r="C112" s="2"/>
       <c r="D112" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E112" s="2" t="s">
         <v>398</v>
@@ -23814,12 +23600,10 @@
       <c r="A113" t="b">
         <v>1</v>
       </c>
-      <c r="B113" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B113" s="2"/>
       <c r="C113" s="2"/>
       <c r="D113" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E113" s="2" t="s">
         <v>399</v>
@@ -23836,12 +23620,10 @@
       <c r="A114" t="b">
         <v>1</v>
       </c>
-      <c r="B114" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B114" s="2"/>
       <c r="C114" s="2"/>
       <c r="D114" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E114" s="2" t="s">
         <v>400</v>
@@ -23858,12 +23640,10 @@
       <c r="A115" t="b">
         <v>1</v>
       </c>
-      <c r="B115" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B115" s="2"/>
       <c r="C115" s="2"/>
       <c r="D115" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E115" s="2" t="s">
         <v>283</v>
@@ -23880,12 +23660,10 @@
       <c r="A116" t="b">
         <v>1</v>
       </c>
-      <c r="B116" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B116" s="2"/>
       <c r="C116" s="2"/>
       <c r="D116" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E116" s="2" t="s">
         <v>284</v>
@@ -23902,12 +23680,10 @@
       <c r="A117" t="b">
         <v>1</v>
       </c>
-      <c r="B117" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B117" s="2"/>
       <c r="C117" s="2"/>
       <c r="D117" s="2" t="s">
-        <v>725</v>
+        <v>724</v>
       </c>
       <c r="E117" s="2" t="s">
         <v>401</v>
@@ -23927,7 +23703,7 @@
       <c r="B118" s="2"/>
       <c r="C118" s="2"/>
       <c r="D118" s="2" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="E118" s="2" t="s">
         <v>271</v>
@@ -23939,7 +23715,7 @@
         <v>547</v>
       </c>
       <c r="J118" s="2" t="s">
-        <v>760</v>
+        <v>759</v>
       </c>
     </row>
     <row r="119" spans="1:10" x14ac:dyDescent="0.2">
@@ -23949,7 +23725,7 @@
       <c r="B119" s="2"/>
       <c r="C119" s="2"/>
       <c r="D119" s="2" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="E119" s="2" t="s">
         <v>272</v>
@@ -23969,7 +23745,7 @@
       <c r="B120" s="2"/>
       <c r="C120" s="2"/>
       <c r="D120" s="2" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="E120" s="2" t="s">
         <v>273</v>
@@ -23989,7 +23765,7 @@
       <c r="B121" s="2"/>
       <c r="C121" s="2"/>
       <c r="D121" s="2" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="E121" s="2" t="s">
         <v>274</v>
@@ -24009,7 +23785,7 @@
       <c r="B122" s="2"/>
       <c r="C122" s="2"/>
       <c r="D122" s="2" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="E122" s="2" t="s">
         <v>275</v>
@@ -24029,7 +23805,7 @@
       <c r="B123" s="2"/>
       <c r="C123" s="2"/>
       <c r="D123" s="2" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="E123" s="2" t="s">
         <v>276</v>
@@ -24049,7 +23825,7 @@
       <c r="B124" s="2"/>
       <c r="C124" s="2"/>
       <c r="D124" s="2" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="E124" s="2" t="s">
         <v>277</v>
@@ -24069,7 +23845,7 @@
       <c r="B125" s="2"/>
       <c r="C125" s="2"/>
       <c r="D125" s="2" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="E125" s="2" t="s">
         <v>278</v>
@@ -24089,7 +23865,7 @@
       <c r="B126" s="2"/>
       <c r="C126" s="2"/>
       <c r="D126" s="2" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="E126" s="2" t="s">
         <v>279</v>
@@ -24109,7 +23885,7 @@
       <c r="B127" s="2"/>
       <c r="C127" s="2"/>
       <c r="D127" s="2" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="E127" s="2" t="s">
         <v>280</v>
@@ -24129,7 +23905,7 @@
       <c r="B128" s="2"/>
       <c r="C128" s="2"/>
       <c r="D128" s="2" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="E128" s="2" t="s">
         <v>281</v>
@@ -24149,7 +23925,7 @@
       <c r="B129" s="2"/>
       <c r="C129" s="2"/>
       <c r="D129" s="2" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="E129" s="2" t="s">
         <v>282</v>
@@ -24169,7 +23945,7 @@
       <c r="B130" s="2"/>
       <c r="C130" s="2"/>
       <c r="D130" s="2" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="E130" s="2" t="s">
         <v>283</v>
@@ -24189,7 +23965,7 @@
       <c r="B131" s="2"/>
       <c r="C131" s="2"/>
       <c r="D131" s="2" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="E131" s="2" t="s">
         <v>284</v>
@@ -24209,7 +23985,7 @@
       <c r="B132" s="2"/>
       <c r="C132" s="2"/>
       <c r="D132" s="2" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="E132" s="2" t="s">
         <v>285</v>
@@ -24229,7 +24005,7 @@
       <c r="B133" s="2"/>
       <c r="C133" s="2"/>
       <c r="D133" s="2" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="E133" s="2" t="s">
         <v>286</v>
@@ -24249,7 +24025,7 @@
       <c r="B134" s="2"/>
       <c r="C134" s="2"/>
       <c r="D134" s="2" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="E134" s="2" t="s">
         <v>287</v>
@@ -24269,7 +24045,7 @@
       <c r="B135" s="2"/>
       <c r="C135" s="2"/>
       <c r="D135" s="2" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="E135" s="2" t="s">
         <v>288</v>
@@ -24289,7 +24065,7 @@
       <c r="B136" s="2"/>
       <c r="C136" s="2"/>
       <c r="D136" s="2" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="E136" s="2" t="s">
         <v>289</v>
@@ -24309,7 +24085,7 @@
       <c r="B137" s="2"/>
       <c r="C137" s="2"/>
       <c r="D137" s="2" t="s">
-        <v>726</v>
+        <v>725</v>
       </c>
       <c r="E137" s="2" t="s">
         <v>290</v>
@@ -24329,7 +24105,7 @@
       <c r="B138" s="2"/>
       <c r="C138" s="2"/>
       <c r="D138" s="2" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="E138" s="2" t="s">
         <v>409</v>
@@ -24341,7 +24117,7 @@
         <v>518</v>
       </c>
       <c r="J138" s="2" t="s">
-        <v>762</v>
+        <v>761</v>
       </c>
     </row>
     <row r="139" spans="1:10" x14ac:dyDescent="0.2">
@@ -24351,7 +24127,7 @@
       <c r="B139" s="2"/>
       <c r="C139" s="2"/>
       <c r="D139" s="2" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="E139" s="2" t="s">
         <v>410</v>
@@ -24371,7 +24147,7 @@
       <c r="B140" s="2"/>
       <c r="C140" s="2"/>
       <c r="D140" s="2" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="E140" s="2" t="s">
         <v>411</v>
@@ -24391,7 +24167,7 @@
       <c r="B141" s="2"/>
       <c r="C141" s="2"/>
       <c r="D141" s="2" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="E141" s="2" t="s">
         <v>412</v>
@@ -24411,7 +24187,7 @@
       <c r="B142" s="2"/>
       <c r="C142" s="2"/>
       <c r="D142" s="2" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="E142" s="2" t="s">
         <v>413</v>
@@ -24431,7 +24207,7 @@
       <c r="B143" s="2"/>
       <c r="C143" s="2"/>
       <c r="D143" s="2" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="E143" s="2" t="s">
         <v>414</v>
@@ -24451,7 +24227,7 @@
       <c r="B144" s="2"/>
       <c r="C144" s="2"/>
       <c r="D144" s="2" t="s">
-        <v>727</v>
+        <v>726</v>
       </c>
       <c r="E144" s="2" t="s">
         <v>149</v>
@@ -24471,7 +24247,7 @@
       <c r="B145" s="2"/>
       <c r="C145" s="2"/>
       <c r="D145" s="2" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="E145" s="2" t="s">
         <v>415</v>
@@ -24483,7 +24259,7 @@
         <v>624</v>
       </c>
       <c r="J145" s="2" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
     </row>
     <row r="146" spans="1:10" x14ac:dyDescent="0.2">
@@ -24493,7 +24269,7 @@
       <c r="B146" s="2"/>
       <c r="C146" s="2"/>
       <c r="D146" s="2" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="E146" s="2" t="s">
         <v>416</v>
@@ -24513,7 +24289,7 @@
       <c r="B147" s="2"/>
       <c r="C147" s="2"/>
       <c r="D147" s="2" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="E147" s="2" t="s">
         <v>417</v>
@@ -24533,7 +24309,7 @@
       <c r="B148" s="2"/>
       <c r="C148" s="2"/>
       <c r="D148" s="2" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="E148" s="2" t="s">
         <v>418</v>
@@ -24553,7 +24329,7 @@
       <c r="B149" s="2"/>
       <c r="C149" s="2"/>
       <c r="D149" s="2" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="E149" s="2" t="s">
         <v>149</v>
@@ -24573,7 +24349,7 @@
       <c r="B150" s="2"/>
       <c r="C150" s="2"/>
       <c r="D150" s="2" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="E150" s="2" t="s">
         <v>409</v>
@@ -24585,7 +24361,7 @@
         <v>518</v>
       </c>
       <c r="J150" s="2" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
     </row>
     <row r="151" spans="1:10" x14ac:dyDescent="0.2">
@@ -24595,7 +24371,7 @@
       <c r="B151" s="2"/>
       <c r="C151" s="2"/>
       <c r="D151" s="2" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="E151" s="2" t="s">
         <v>410</v>
@@ -24615,7 +24391,7 @@
       <c r="B152" s="2"/>
       <c r="C152" s="2"/>
       <c r="D152" s="2" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="E152" s="2" t="s">
         <v>411</v>
@@ -24635,7 +24411,7 @@
       <c r="B153" s="2"/>
       <c r="C153" s="2"/>
       <c r="D153" s="2" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="E153" s="2" t="s">
         <v>412</v>
@@ -24655,7 +24431,7 @@
       <c r="B154" s="2"/>
       <c r="C154" s="2"/>
       <c r="D154" s="2" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="E154" s="2" t="s">
         <v>413</v>
@@ -24675,7 +24451,7 @@
       <c r="B155" s="2"/>
       <c r="C155" s="2"/>
       <c r="D155" s="2" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="E155" s="2" t="s">
         <v>419</v>
@@ -24695,7 +24471,7 @@
       <c r="B156" s="2"/>
       <c r="C156" s="2"/>
       <c r="D156" s="2" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="E156" s="2" t="s">
         <v>416</v>
@@ -24715,7 +24491,7 @@
       <c r="B157" s="2"/>
       <c r="C157" s="2"/>
       <c r="D157" s="2" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="E157" s="2" t="s">
         <v>417</v>
@@ -24735,7 +24511,7 @@
       <c r="B158" s="2"/>
       <c r="C158" s="2"/>
       <c r="D158" s="2" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="E158" s="2" t="s">
         <v>418</v>
@@ -24755,7 +24531,7 @@
       <c r="B159" s="2"/>
       <c r="C159" s="2"/>
       <c r="D159" s="2" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="E159" s="2" t="s">
         <v>420</v>
@@ -24775,7 +24551,7 @@
       <c r="B160" s="2"/>
       <c r="C160" s="2"/>
       <c r="D160" s="2" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="E160" s="2" t="s">
         <v>149</v>
@@ -24795,7 +24571,7 @@
       <c r="B161" s="2"/>
       <c r="C161" s="2"/>
       <c r="D161" s="2" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="E161" s="2" t="s">
         <v>423</v>
@@ -24807,7 +24583,7 @@
         <v>598</v>
       </c>
       <c r="J161" s="2" t="s">
-        <v>765</v>
+        <v>764</v>
       </c>
     </row>
     <row r="162" spans="1:10" x14ac:dyDescent="0.2">
@@ -24817,7 +24593,7 @@
       <c r="B162" s="2"/>
       <c r="C162" s="2"/>
       <c r="D162" s="2" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="E162" s="2" t="s">
         <v>424</v>
@@ -24837,7 +24613,7 @@
       <c r="B163" s="2"/>
       <c r="C163" s="2"/>
       <c r="D163" s="2" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="E163" s="2" t="s">
         <v>425</v>
@@ -24857,7 +24633,7 @@
       <c r="B164" s="2"/>
       <c r="C164" s="2"/>
       <c r="D164" s="2" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="E164" s="2" t="s">
         <v>426</v>
@@ -24877,7 +24653,7 @@
       <c r="B165" s="2"/>
       <c r="C165" s="2"/>
       <c r="D165" s="2" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="E165" s="2" t="s">
         <v>427</v>
@@ -24897,7 +24673,7 @@
       <c r="B166" s="2"/>
       <c r="C166" s="2"/>
       <c r="D166" s="2" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="E166" s="2" t="s">
         <v>428</v>
@@ -24917,7 +24693,7 @@
       <c r="B167" s="2"/>
       <c r="C167" s="2"/>
       <c r="D167" s="2" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="E167" s="2" t="s">
         <v>429</v>
@@ -24937,7 +24713,7 @@
       <c r="B168" s="2"/>
       <c r="C168" s="2"/>
       <c r="D168" s="2" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="E168" s="2" t="s">
         <v>430</v>
@@ -24957,7 +24733,7 @@
       <c r="B169" s="2"/>
       <c r="C169" s="2"/>
       <c r="D169" s="2" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="E169" s="2" t="s">
         <v>431</v>
@@ -24977,7 +24753,7 @@
       <c r="B170" s="2"/>
       <c r="C170" s="2"/>
       <c r="D170" s="2" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="E170" s="2" t="s">
         <v>432</v>
@@ -24997,7 +24773,7 @@
       <c r="B171" s="2"/>
       <c r="C171" s="2"/>
       <c r="D171" s="2" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="E171" s="2" t="s">
         <v>433</v>
@@ -25017,7 +24793,7 @@
       <c r="B172" s="2"/>
       <c r="C172" s="2"/>
       <c r="D172" s="2" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="E172" s="2" t="s">
         <v>434</v>
@@ -25037,7 +24813,7 @@
       <c r="B173" s="2"/>
       <c r="C173" s="2"/>
       <c r="D173" s="2" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="E173" s="2" t="s">
         <v>423</v>
@@ -25049,7 +24825,7 @@
         <v>598</v>
       </c>
       <c r="J173" s="2" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
     </row>
     <row r="174" spans="1:10" x14ac:dyDescent="0.2">
@@ -25059,7 +24835,7 @@
       <c r="B174" s="2"/>
       <c r="C174" s="2"/>
       <c r="D174" s="2" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="E174" s="2" t="s">
         <v>424</v>
@@ -25079,7 +24855,7 @@
       <c r="B175" s="2"/>
       <c r="C175" s="2"/>
       <c r="D175" s="2" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="E175" s="2" t="s">
         <v>425</v>
@@ -25099,7 +24875,7 @@
       <c r="B176" s="2"/>
       <c r="C176" s="2"/>
       <c r="D176" s="2" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="E176" s="2" t="s">
         <v>426</v>
@@ -25119,7 +24895,7 @@
       <c r="B177" s="2"/>
       <c r="C177" s="2"/>
       <c r="D177" s="2" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="E177" s="2" t="s">
         <v>427</v>
@@ -25139,7 +24915,7 @@
       <c r="B178" s="2"/>
       <c r="C178" s="2"/>
       <c r="D178" s="2" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="E178" s="2" t="s">
         <v>428</v>
@@ -25159,7 +24935,7 @@
       <c r="B179" s="2"/>
       <c r="C179" s="2"/>
       <c r="D179" s="2" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="E179" s="2" t="s">
         <v>429</v>
@@ -25179,7 +24955,7 @@
       <c r="B180" s="2"/>
       <c r="C180" s="2"/>
       <c r="D180" s="2" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="E180" s="2" t="s">
         <v>430</v>
@@ -25199,7 +24975,7 @@
       <c r="B181" s="2"/>
       <c r="C181" s="2"/>
       <c r="D181" s="2" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="E181" s="2" t="s">
         <v>431</v>
@@ -25219,7 +24995,7 @@
       <c r="B182" s="2"/>
       <c r="C182" s="2"/>
       <c r="D182" s="2" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="E182" s="2" t="s">
         <v>432</v>
@@ -25239,7 +25015,7 @@
       <c r="B183" s="2"/>
       <c r="C183" s="2"/>
       <c r="D183" s="2" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="E183" s="2" t="s">
         <v>433</v>
@@ -25259,7 +25035,7 @@
       <c r="B184" s="2"/>
       <c r="C184" s="2"/>
       <c r="D184" s="2" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="E184" s="2" t="s">
         <v>434</v>
@@ -25279,7 +25055,7 @@
       <c r="B185" s="2"/>
       <c r="C185" s="2"/>
       <c r="D185" s="2" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="E185" s="2" t="s">
         <v>149</v>

</xml_diff>

<commit_message>
Removed sourceValue for dashboard_ignore row (not an enum mapping)
</commit_message>
<xml_diff>
--- a/data/mapping_config_files/NWSS-to-ODM-dictionary.xlsx
+++ b/data/mapping_config_files/NWSS-to-ODM-dictionary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-MapGenerator/PHES-ODM-MapGenerator/data/mapping_config_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AADC31C-A064-044E-A948-9802024BE138}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7342C3BD-CDA0-914D-BE9F-959B5DED16CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="280" yWindow="500" windowWidth="39840" windowHeight="19600" xr2:uid="{77810E24-F86B-BC44-A0D5-8790E6EC60B4}"/>
   </bookViews>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2391" uniqueCount="768">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2390" uniqueCount="768">
   <si>
     <t>Reporter</t>
   </si>
@@ -15494,9 +15494,7 @@
         <v>650</v>
       </c>
       <c r="D61" s="2"/>
-      <c r="E61" s="2" t="s">
-        <v>147</v>
-      </c>
+      <c r="E61" s="2"/>
       <c r="F61" s="2" t="s">
         <v>124</v>
       </c>

</xml_diff>

<commit_message>
Updates to more complex derivations
</commit_message>
<xml_diff>
--- a/data/mapping_config_files/NWSS-to-ODM-dictionary.xlsx
+++ b/data/mapping_config_files/NWSS-to-ODM-dictionary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-MapGenerator/PHES-ODM-MapGenerator/data/mapping_config_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69609E77-4339-CA48-B7EC-B56850147210}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5F613E1-6D96-B64B-9A2F-54244DCC1AFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="220" yWindow="500" windowWidth="39840" windowHeight="19600" xr2:uid="{77810E24-F86B-BC44-A0D5-8790E6EC60B4}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15880" xr2:uid="{77810E24-F86B-BC44-A0D5-8790E6EC60B4}"/>
   </bookViews>
   <sheets>
     <sheet name="maps" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,9 @@
     <externalReference r:id="rId4"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">maps!$A$1:$L$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">enums!$A$1:$J$185</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">maps!$A$1:$L$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">wide!$A$1:$N$136</definedName>
     <definedName name="partID">[1]parts!$A:$A</definedName>
     <definedName name="partLabel">[1]parts!$B:$B</definedName>
   </definedNames>
@@ -45,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2374" uniqueCount="761">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2373" uniqueCount="761">
   <si>
     <t>Reporter</t>
   </si>
@@ -2252,9 +2254,6 @@
     <t>{{site_id}}</t>
   </si>
   <si>
-    <t>{{county_names}}</t>
-  </si>
-  <si>
     <t>{{zipcode}}</t>
   </si>
   <si>
@@ -2288,9 +2287,6 @@
     <t>See row 67 in original maps sheet</t>
   </si>
   <si>
-    <t>major_lab_method_desc is not in NWSS LinkML schema</t>
-  </si>
-  <si>
     <t>For source slot pcr_target</t>
   </si>
   <si>
@@ -2321,9 +2317,6 @@
     <t>contactID</t>
   </si>
   <si>
-    <t>Same targets: Concatenate: "EPA_id: value, EPA_registry_id: epaid_registry_id"</t>
-  </si>
-  <si>
     <t>{{sample_location_specify}}</t>
   </si>
   <si>
@@ -2349,6 +2342,15 @@
   </si>
   <si>
     <t>What about for other combinations of inhibition_adjust and inhibition_detect? All other cases: empty</t>
+  </si>
+  <si>
+    <t>"County names=" + county_names + "; EPA_id=" + epaid + "; EPA_registry_id=" + epa_registry_id</t>
+  </si>
+  <si>
+    <t>Good! Same targets: Concatenate: "EPA_id: value, EPA_registry_id: epaid_registry_id"</t>
+  </si>
+  <si>
+    <t>Fixed! major_lab_method_desc is not in NWSS LinkML schema: Is in data dictionary, rerun schema generator</t>
   </si>
 </sst>
 </file>
@@ -13909,7 +13911,7 @@
         <v>115</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>750</v>
+        <v>748</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>726</v>
@@ -13920,7 +13922,7 @@
         <v>483</v>
       </c>
       <c r="L2" s="19" t="s">
-        <v>755</v>
+        <v>752</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
@@ -13965,25 +13967,23 @@
       <c r="D4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="E4" s="2"/>
       <c r="F4" s="6" t="s">
         <v>77</v>
       </c>
       <c r="G4" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="H4" s="2" t="s">
-        <v>728</v>
-      </c>
-      <c r="I4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="21" t="s">
+        <v>758</v>
+      </c>
       <c r="J4" s="2"/>
       <c r="K4" s="1" t="s">
         <v>621</v>
       </c>
       <c r="L4" s="19" t="s">
-        <v>751</v>
+        <v>759</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
@@ -14009,7 +14009,7 @@
         <v>80</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>729</v>
+        <v>728</v>
       </c>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
@@ -14038,7 +14038,7 @@
         <v>81</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
@@ -14135,13 +14135,13 @@
         <v>121</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>752</v>
+        <v>749</v>
       </c>
       <c r="I10" s="6"/>
       <c r="J10" s="6"/>
       <c r="K10" s="2"/>
       <c r="L10" s="22" t="s">
-        <v>756</v>
+        <v>753</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.2">
@@ -14654,7 +14654,7 @@
         <v>121</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>747</v>
+        <v>745</v>
       </c>
       <c r="I29" s="2"/>
       <c r="J29" s="2"/>
@@ -14683,7 +14683,7 @@
         <v>121</v>
       </c>
       <c r="H30" s="2" t="s">
-        <v>748</v>
+        <v>746</v>
       </c>
       <c r="I30" s="2"/>
       <c r="J30" s="2"/>
@@ -14712,7 +14712,7 @@
         <v>116</v>
       </c>
       <c r="H31" s="2" t="s">
-        <v>731</v>
+        <v>730</v>
       </c>
       <c r="I31" s="2"/>
       <c r="J31" s="2"/>
@@ -14720,7 +14720,7 @@
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A32" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>2</v>
@@ -14736,10 +14736,10 @@
         <v>77</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>749</v>
+        <v>747</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>732</v>
+        <v>731</v>
       </c>
       <c r="I32" s="2"/>
       <c r="J32" s="2"/>
@@ -14818,7 +14818,7 @@
         <v>120</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>733</v>
+        <v>732</v>
       </c>
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
@@ -15202,7 +15202,7 @@
         <v>140</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>734</v>
+        <v>733</v>
       </c>
       <c r="I50" s="2"/>
       <c r="J50" s="2"/>
@@ -15231,7 +15231,7 @@
         <v>144</v>
       </c>
       <c r="H51" s="2" t="s">
-        <v>735</v>
+        <v>734</v>
       </c>
       <c r="I51" s="2"/>
       <c r="J51" s="2"/>
@@ -15588,7 +15588,7 @@
         <v>162</v>
       </c>
       <c r="H65" s="2" t="s">
-        <v>736</v>
+        <v>735</v>
       </c>
       <c r="I65" s="2"/>
       <c r="J65" s="2"/>
@@ -15807,10 +15807,10 @@
       <c r="I74" s="2"/>
       <c r="J74" s="2"/>
       <c r="K74" s="1" t="s">
-        <v>759</v>
+        <v>756</v>
       </c>
       <c r="L74" s="19" t="s">
-        <v>760</v>
+        <v>757</v>
       </c>
     </row>
     <row r="75" spans="1:12" x14ac:dyDescent="0.2">
@@ -16118,7 +16118,7 @@
         <v>479</v>
       </c>
       <c r="H86" s="2" t="s">
-        <v>737</v>
+        <v>736</v>
       </c>
       <c r="I86" s="2"/>
       <c r="J86" s="2"/>
@@ -16145,17 +16145,17 @@
         <v>481</v>
       </c>
       <c r="H87" s="2" t="s">
-        <v>738</v>
+        <v>737</v>
       </c>
       <c r="I87" s="2"/>
       <c r="J87" s="2"/>
       <c r="K87" s="2"/>
       <c r="L87" s="22" t="s">
-        <v>740</v>
+        <v>760</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L6" xr:uid="{3154BFCE-06D9-9649-B340-B23DCF20DD83}"/>
+  <autoFilter ref="A1:L87" xr:uid="{3154BFCE-06D9-9649-B340-B23DCF20DD83}"/>
   <conditionalFormatting sqref="H37:J37">
     <cfRule type="duplicateValues" dxfId="8" priority="10"/>
   </conditionalFormatting>
@@ -20453,7 +20453,7 @@
         <v>414</v>
       </c>
       <c r="G118" s="2" t="s">
-        <v>757</v>
+        <v>754</v>
       </c>
       <c r="H118" s="2" t="s">
         <v>76</v>
@@ -20829,7 +20829,7 @@
         <v>657</v>
       </c>
       <c r="G128" s="2" t="s">
-        <v>754</v>
+        <v>751</v>
       </c>
       <c r="H128" s="2" t="s">
         <v>170</v>
@@ -20850,7 +20850,7 @@
         <v>164</v>
       </c>
       <c r="N128" s="2" t="s">
-        <v>739</v>
+        <v>738</v>
       </c>
     </row>
     <row r="129" spans="1:14" x14ac:dyDescent="0.2">
@@ -20871,7 +20871,7 @@
         <v>657</v>
       </c>
       <c r="G129" s="2" t="s">
-        <v>753</v>
+        <v>750</v>
       </c>
       <c r="H129" s="2" t="s">
         <v>170</v>
@@ -20913,7 +20913,7 @@
         <v>657</v>
       </c>
       <c r="G130" s="2" t="s">
-        <v>753</v>
+        <v>750</v>
       </c>
       <c r="H130" s="2" t="s">
         <v>170</v>
@@ -20955,7 +20955,7 @@
         <v>657</v>
       </c>
       <c r="G131" s="2" t="s">
-        <v>753</v>
+        <v>750</v>
       </c>
       <c r="H131" s="2" t="s">
         <v>170</v>
@@ -20997,7 +20997,7 @@
         <v>657</v>
       </c>
       <c r="G132" s="2" t="s">
-        <v>758</v>
+        <v>755</v>
       </c>
       <c r="H132" s="2" t="s">
         <v>170</v>
@@ -21182,6 +21182,7 @@
       <c r="N136" s="2"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:N136" xr:uid="{B39AC7DD-3F73-2C47-925D-21E5B4EBE6FC}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="D99:D105">
     <sortCondition ref="D99:D105"/>
   </sortState>
@@ -21277,7 +21278,7 @@
         <v>514</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>742</v>
+        <v>740</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.2">
@@ -23599,7 +23600,7 @@
         <v>540</v>
       </c>
       <c r="J118" s="2" t="s">
-        <v>741</v>
+        <v>739</v>
       </c>
     </row>
     <row r="119" spans="1:10" x14ac:dyDescent="0.2">
@@ -24001,7 +24002,7 @@
         <v>511</v>
       </c>
       <c r="J138" s="2" t="s">
-        <v>743</v>
+        <v>741</v>
       </c>
     </row>
     <row r="139" spans="1:10" x14ac:dyDescent="0.2">
@@ -24143,7 +24144,7 @@
         <v>616</v>
       </c>
       <c r="J145" s="2" t="s">
-        <v>744</v>
+        <v>742</v>
       </c>
     </row>
     <row r="146" spans="1:10" x14ac:dyDescent="0.2">
@@ -24245,7 +24246,7 @@
         <v>511</v>
       </c>
       <c r="J150" s="2" t="s">
-        <v>745</v>
+        <v>743</v>
       </c>
     </row>
     <row r="151" spans="1:10" x14ac:dyDescent="0.2">
@@ -24467,7 +24468,7 @@
         <v>590</v>
       </c>
       <c r="J161" s="2" t="s">
-        <v>746</v>
+        <v>744</v>
       </c>
     </row>
     <row r="162" spans="1:10" x14ac:dyDescent="0.2">
@@ -24953,6 +24954,7 @@
       <c r="J185" s="2"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:J185" xr:uid="{1BC10C3F-0C27-5546-8767-E60C7CACEA9D}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>

</xml_diff>

<commit_message>
Readed 'not institution specific' for institution_type enum
</commit_message>
<xml_diff>
--- a/data/mapping_config_files/NWSS-to-ODM-dictionary.xlsx
+++ b/data/mapping_config_files/NWSS-to-ODM-dictionary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-MapGenerator/PHES-ODM-MapGenerator/data/mapping_config_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C6A2996-92A5-AE4A-9D50-E75DBBB41723}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C6C5052-DB9B-1142-8E50-8770330E035B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2020" yWindow="500" windowWidth="38940" windowHeight="20920" xr2:uid="{77810E24-F86B-BC44-A0D5-8790E6EC60B4}"/>
   </bookViews>
@@ -14582,7 +14582,7 @@
     </row>
     <row r="18" spans="1:12" s="23" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B18" s="28" t="s">
         <v>1</v>

</xml_diff>

<commit_message>
Added _expr columns to wide column configuration, to allow setting target slots as LinkML expr code blocks
</commit_message>
<xml_diff>
--- a/data/mapping_config_files/NWSS-to-ODM-dictionary.xlsx
+++ b/data/mapping_config_files/NWSS-to-ODM-dictionary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-MapGenerator/PHES-ODM-MapGenerator/data/mapping_config_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C6C5052-DB9B-1142-8E50-8770330E035B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A5DC79A-7FEE-6549-9EC3-331B947A808C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2020" yWindow="500" windowWidth="38940" windowHeight="20920" xr2:uid="{77810E24-F86B-BC44-A0D5-8790E6EC60B4}"/>
+    <workbookView xWindow="2020" yWindow="500" windowWidth="38940" windowHeight="20920" activeTab="2" xr2:uid="{77810E24-F86B-BC44-A0D5-8790E6EC60B4}"/>
   </bookViews>
   <sheets>
     <sheet name="maps" sheetId="1" r:id="rId1"/>
@@ -18,16 +18,15 @@
     <sheet name="wide_qualityReports" sheetId="7" r:id="rId3"/>
     <sheet name="enums" sheetId="3" r:id="rId4"/>
     <sheet name="id_gen" sheetId="4" r:id="rId5"/>
-    <sheet name="Sheet1" sheetId="5" r:id="rId6"/>
-    <sheet name="maps original" sheetId="6" r:id="rId7"/>
+    <sheet name="maps original" sheetId="6" r:id="rId6"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId8"/>
+    <externalReference r:id="rId7"/>
   </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">enums!$A$1:$J$185</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">maps!$A$1:$L$91</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'maps original'!$A$1:$L$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'maps original'!$A$1:$L$87</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">wide!$A$1:$N$136</definedName>
     <definedName name="partID">[1]parts!$A:$A</definedName>
     <definedName name="partLabel">[1]parts!$B:$B</definedName>
@@ -52,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3244" uniqueCount="838">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3216" uniqueCount="836">
   <si>
     <t>Reporter</t>
   </si>
@@ -2565,27 +2564,15 @@
     <t>{{ntc_amplify}}</t>
   </si>
   <si>
-    <t>{{inhibition_detect}}</t>
-  </si>
-  <si>
     <t>{{id:qualityReportID4}}</t>
   </si>
   <si>
-    <t>flagAI OR flagFI</t>
-  </si>
-  <si>
-    <t>{{inhibition_adjust}}</t>
-  </si>
-  <si>
     <t>{{id:qualityReportID5}}</t>
   </si>
   <si>
     <t>qualityReportID_target</t>
   </si>
   <si>
-    <t>{{id:qualityReportID6}}</t>
-  </si>
-  <si>
     <t>{{quality_flag}}</t>
   </si>
   <si>
@@ -2593,6 +2580,18 @@
   </si>
   <si>
     <t>Added by Martin</t>
+  </si>
+  <si>
+    <t>qualityFlag_expr</t>
+  </si>
+  <si>
+    <t>def get_qualityFlag(inhibition_detect: str, inhibition_adjust: str) -&gt; str:
+    if inhibition_detect == "yes" and inhibition_adjust == "yes":
+        return "flagAI"
+    elif inhibition_detect == "yes" and inhibition_adjust == "no":
+        return "flagFI"
+    return "ignore"
+target = get_qualityFlag(src.inhibition_detect, src.inhibition_adjust)</t>
   </si>
 </sst>
 </file>
@@ -2810,7 +2809,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -2863,6 +2862,9 @@
     <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -14292,7 +14294,7 @@
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
       <c r="L5" t="s">
-        <v>837</v>
+        <v>833</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
@@ -14564,7 +14566,7 @@
       <c r="J16" s="6"/>
       <c r="K16" s="2"/>
       <c r="L16" s="22" t="s">
-        <v>837</v>
+        <v>833</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.2">
@@ -16564,12 +16566,14 @@
       <c r="A94" t="b">
         <v>1</v>
       </c>
+      <c r="B94" s="2"/>
       <c r="C94" s="2" t="s">
         <v>635</v>
       </c>
       <c r="D94" s="2" t="s">
         <v>812</v>
       </c>
+      <c r="E94" s="2"/>
       <c r="F94" s="2" t="s">
         <v>79</v>
       </c>
@@ -16580,17 +16584,22 @@
         <f t="shared" ref="H94:H101" si="0">"{{"&amp;D94&amp;"}}"</f>
         <v>{{id:addressID}}</v>
       </c>
+      <c r="I94" s="2"/>
+      <c r="J94" s="2"/>
+      <c r="K94" s="2"/>
     </row>
     <row r="95" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A95" t="b">
         <v>1</v>
       </c>
+      <c r="B95" s="2"/>
       <c r="C95" s="2" t="s">
         <v>635</v>
       </c>
       <c r="D95" s="2" t="s">
         <v>807</v>
       </c>
+      <c r="E95" s="2"/>
       <c r="F95" s="2" t="s">
         <v>115</v>
       </c>
@@ -16601,17 +16610,22 @@
         <f>"{{"&amp;D95&amp;"}}"</f>
         <v>{{id:datasetID}}</v>
       </c>
+      <c r="I95" s="2"/>
+      <c r="J95" s="2"/>
+      <c r="K95" s="2"/>
     </row>
     <row r="96" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A96" t="b">
         <v>1</v>
       </c>
+      <c r="B96" s="2"/>
       <c r="C96" s="2" t="s">
         <v>635</v>
       </c>
       <c r="D96" s="2" t="s">
         <v>805</v>
       </c>
+      <c r="E96" s="2"/>
       <c r="F96" s="2" t="s">
         <v>115</v>
       </c>
@@ -16622,17 +16636,22 @@
         <f>"{{"&amp;D96&amp;"}}"</f>
         <v>{{id:measureRepID}}</v>
       </c>
-    </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I96" s="2"/>
+      <c r="J96" s="2"/>
+      <c r="K96" s="2"/>
+    </row>
+    <row r="97" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A97" t="b">
         <v>1</v>
       </c>
+      <c r="B97" s="2"/>
       <c r="C97" s="2" t="s">
         <v>635</v>
       </c>
-      <c r="D97" t="s">
+      <c r="D97" s="2" t="s">
         <v>808</v>
       </c>
+      <c r="E97" s="2"/>
       <c r="F97" s="2" t="s">
         <v>115</v>
       </c>
@@ -16643,17 +16662,22 @@
         <f>"{{"&amp;D97&amp;"}}"</f>
         <v>{{id:measureSetRepID}}</v>
       </c>
-    </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I97" s="2"/>
+      <c r="J97" s="2"/>
+      <c r="K97" s="2"/>
+    </row>
+    <row r="98" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A98" t="b">
         <v>1</v>
       </c>
+      <c r="B98" s="2"/>
       <c r="C98" s="2" t="s">
         <v>635</v>
       </c>
       <c r="D98" s="2" t="s">
         <v>805</v>
       </c>
+      <c r="E98" s="2"/>
       <c r="F98" s="2" t="s">
         <v>147</v>
       </c>
@@ -16664,17 +16688,22 @@
         <f t="shared" si="0"/>
         <v>{{id:measureRepID}}</v>
       </c>
-    </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I98" s="2"/>
+      <c r="J98" s="2"/>
+      <c r="K98" s="2"/>
+    </row>
+    <row r="99" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A99" t="b">
         <v>1</v>
       </c>
+      <c r="B99" s="2"/>
       <c r="C99" s="2" t="s">
         <v>635</v>
       </c>
-      <c r="D99" t="s">
+      <c r="D99" s="2" t="s">
         <v>808</v>
       </c>
+      <c r="E99" s="2"/>
       <c r="F99" s="2" t="s">
         <v>147</v>
       </c>
@@ -16685,17 +16714,22 @@
         <f t="shared" si="0"/>
         <v>{{id:measureSetRepID}}</v>
       </c>
-    </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I99" s="2"/>
+      <c r="J99" s="2"/>
+      <c r="K99" s="2"/>
+    </row>
+    <row r="100" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A100" t="b">
         <v>1</v>
       </c>
+      <c r="B100" s="2"/>
       <c r="C100" s="2" t="s">
         <v>635</v>
       </c>
       <c r="D100" s="2" t="s">
         <v>810</v>
       </c>
+      <c r="E100" s="2"/>
       <c r="F100" s="2" t="s">
         <v>152</v>
       </c>
@@ -16706,17 +16740,22 @@
         <f t="shared" si="0"/>
         <v>{{id:instrumentID}}</v>
       </c>
-    </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I100" s="2"/>
+      <c r="J100" s="2"/>
+      <c r="K100" s="2"/>
+    </row>
+    <row r="101" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A101" t="b">
         <v>1</v>
       </c>
+      <c r="B101" s="2"/>
       <c r="C101" s="2" t="s">
         <v>635</v>
       </c>
       <c r="D101" s="2" t="s">
         <v>809</v>
       </c>
+      <c r="E101" s="2"/>
       <c r="F101" s="2" t="s">
         <v>152</v>
       </c>
@@ -16727,17 +16766,22 @@
         <f t="shared" si="0"/>
         <v>{{id:stepID}}</v>
       </c>
-    </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I101" s="2"/>
+      <c r="J101" s="2"/>
+      <c r="K101" s="2"/>
+    </row>
+    <row r="102" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A102" t="b">
         <v>1</v>
       </c>
+      <c r="B102" s="2"/>
       <c r="C102" s="2" t="s">
         <v>635</v>
       </c>
       <c r="D102" s="2" t="s">
         <v>807</v>
       </c>
+      <c r="E102" s="2"/>
       <c r="F102" s="2" t="s">
         <v>476</v>
       </c>
@@ -16748,17 +16792,22 @@
         <f>"{{"&amp;D102&amp;"}}"</f>
         <v>{{id:datasetID}}</v>
       </c>
-    </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I102" s="2"/>
+      <c r="J102" s="2"/>
+      <c r="K102" s="2"/>
+    </row>
+    <row r="103" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A103" t="b">
         <v>1</v>
       </c>
+      <c r="B103" s="2"/>
       <c r="C103" s="2" t="s">
         <v>635</v>
       </c>
       <c r="D103" s="2" t="s">
         <v>807</v>
       </c>
+      <c r="E103" s="2"/>
       <c r="F103" s="2" t="s">
         <v>118</v>
       </c>
@@ -16769,17 +16818,22 @@
         <f>"{{"&amp;D103&amp;"}}"</f>
         <v>{{id:datasetID}}</v>
       </c>
-    </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="I103" s="2"/>
+      <c r="J103" s="2"/>
+      <c r="K103" s="2"/>
+    </row>
+    <row r="104" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A104" t="b">
         <v>1</v>
       </c>
+      <c r="B104" s="2"/>
       <c r="C104" s="2" t="s">
         <v>635</v>
       </c>
       <c r="D104" s="2" t="s">
         <v>807</v>
       </c>
+      <c r="E104" s="2"/>
       <c r="F104" s="2" t="s">
         <v>77</v>
       </c>
@@ -16790,6 +16844,9 @@
         <f>"{{"&amp;D104&amp;"}}"</f>
         <v>{{id:datasetID}}</v>
       </c>
+      <c r="I104" s="2"/>
+      <c r="J104" s="2"/>
+      <c r="K104" s="2"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:L91" xr:uid="{3154BFCE-06D9-9649-B340-B23DCF20DD83}"/>
@@ -17309,7 +17366,7 @@
         <v>28</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>836</v>
+        <v>832</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>152</v>
@@ -19803,7 +19860,7 @@
         <v>37</v>
       </c>
       <c r="D82" s="3" t="s">
-        <v>836</v>
+        <v>832</v>
       </c>
       <c r="E82" s="2" t="s">
         <v>152</v>
@@ -20428,7 +20485,7 @@
         <v>38</v>
       </c>
       <c r="D99" s="3" t="s">
-        <v>836</v>
+        <v>832</v>
       </c>
       <c r="E99" s="2" t="s">
         <v>152</v>
@@ -21827,8 +21884,8 @@
     <cfRule type="duplicateValues" dxfId="8" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K94">
-    <cfRule type="duplicateValues" dxfId="7" priority="2"/>
-    <cfRule type="duplicateValues" dxfId="6" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K121:M121">
     <cfRule type="duplicateValues" dxfId="5" priority="7"/>
@@ -21852,7 +21909,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B4CA3B6-4765-0A43-8534-6DA7BF8A336D}">
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="18.6640625" bestFit="1" customWidth="1"/>
@@ -21860,10 +21917,10 @@
     <col min="6" max="6" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.83203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="23" customWidth="1"/>
-    <col min="9" max="9" width="22.33203125" customWidth="1"/>
+    <col min="9" max="10" width="22.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="24" customFormat="1" ht="20" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" s="24" customFormat="1" ht="20" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="24" t="s">
         <v>680</v>
       </c>
@@ -21886,16 +21943,19 @@
         <v>698</v>
       </c>
       <c r="H1" s="9" t="s">
-        <v>833</v>
+        <v>830</v>
       </c>
       <c r="I1" s="11" t="s">
         <v>821</v>
       </c>
-      <c r="J1" s="12" t="s">
+      <c r="J1" s="11" t="s">
+        <v>834</v>
+      </c>
+      <c r="K1" s="12" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" t="b">
         <v>1</v>
       </c>
@@ -21921,7 +21981,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" t="b">
         <v>1</v>
       </c>
@@ -21941,7 +22001,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" t="b">
         <v>1</v>
       </c>
@@ -21952,7 +22012,7 @@
         <v>56</v>
       </c>
       <c r="D4" t="s">
-        <v>836</v>
+        <v>832</v>
       </c>
       <c r="E4" t="s">
         <v>147</v>
@@ -21961,7 +22021,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" t="b">
         <v>1</v>
       </c>
@@ -21987,7 +22047,7 @@
         <v>825</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" t="b">
         <v>1</v>
       </c>
@@ -22007,7 +22067,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" t="b">
         <v>1</v>
       </c>
@@ -22018,7 +22078,7 @@
         <v>64</v>
       </c>
       <c r="D7" t="s">
-        <v>836</v>
+        <v>832</v>
       </c>
       <c r="E7" t="s">
         <v>147</v>
@@ -22027,7 +22087,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A8" t="b">
         <v>1</v>
       </c>
@@ -22053,7 +22113,7 @@
         <v>827</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A9" t="b">
         <v>1</v>
       </c>
@@ -22073,7 +22133,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:11" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" t="b">
         <v>1</v>
       </c>
@@ -22083,23 +22143,17 @@
       <c r="C10" t="s">
         <v>68</v>
       </c>
-      <c r="D10" t="s">
-        <v>141</v>
-      </c>
       <c r="E10" t="s">
         <v>147</v>
       </c>
-      <c r="F10" t="s">
-        <v>830</v>
-      </c>
       <c r="H10" t="s">
-        <v>829</v>
-      </c>
-      <c r="I10" t="s">
         <v>828</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J10" s="34" t="s">
+        <v>835</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A11" t="b">
         <v>1</v>
       </c>
@@ -22107,19 +22161,25 @@
         <v>635</v>
       </c>
       <c r="C11" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="D11" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E11" t="s">
         <v>147</v>
       </c>
       <c r="F11" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+        <v>149</v>
+      </c>
+      <c r="H11" t="s">
+        <v>829</v>
+      </c>
+      <c r="I11" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A12" t="b">
         <v>1</v>
       </c>
@@ -22127,19 +22187,19 @@
         <v>635</v>
       </c>
       <c r="C12" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="D12" t="s">
-        <v>603</v>
+        <v>142</v>
       </c>
       <c r="E12" t="s">
         <v>147</v>
       </c>
       <c r="F12" t="s">
-        <v>598</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A13" t="b">
         <v>1</v>
       </c>
@@ -22147,127 +22207,15 @@
         <v>635</v>
       </c>
       <c r="C13" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="D13" t="s">
-        <v>141</v>
+        <v>832</v>
       </c>
       <c r="E13" t="s">
         <v>147</v>
       </c>
       <c r="F13" t="s">
-        <v>604</v>
-      </c>
-      <c r="H13" t="s">
-        <v>832</v>
-      </c>
-      <c r="I13" t="s">
-        <v>831</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A14" t="b">
-        <v>1</v>
-      </c>
-      <c r="B14" t="s">
-        <v>635</v>
-      </c>
-      <c r="C14" t="s">
-        <v>69</v>
-      </c>
-      <c r="D14" t="s">
-        <v>142</v>
-      </c>
-      <c r="E14" t="s">
-        <v>147</v>
-      </c>
-      <c r="F14" t="s">
-        <v>605</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A15" t="b">
-        <v>1</v>
-      </c>
-      <c r="B15" t="s">
-        <v>635</v>
-      </c>
-      <c r="C15" t="s">
-        <v>69</v>
-      </c>
-      <c r="D15" t="s">
-        <v>836</v>
-      </c>
-      <c r="E15" t="s">
-        <v>147</v>
-      </c>
-      <c r="F15" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A16" t="b">
-        <v>1</v>
-      </c>
-      <c r="B16" t="s">
-        <v>635</v>
-      </c>
-      <c r="C16" t="s">
-        <v>73</v>
-      </c>
-      <c r="D16" t="s">
-        <v>141</v>
-      </c>
-      <c r="E16" t="s">
-        <v>147</v>
-      </c>
-      <c r="F16" t="s">
-        <v>149</v>
-      </c>
-      <c r="H16" t="s">
-        <v>834</v>
-      </c>
-      <c r="I16" t="s">
-        <v>835</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A17" t="b">
-        <v>1</v>
-      </c>
-      <c r="B17" t="s">
-        <v>635</v>
-      </c>
-      <c r="C17" t="s">
-        <v>73</v>
-      </c>
-      <c r="D17" t="s">
-        <v>142</v>
-      </c>
-      <c r="E17" t="s">
-        <v>147</v>
-      </c>
-      <c r="F17" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A18" t="b">
-        <v>1</v>
-      </c>
-      <c r="B18" t="s">
-        <v>635</v>
-      </c>
-      <c r="C18" t="s">
-        <v>73</v>
-      </c>
-      <c r="D18" t="s">
-        <v>836</v>
-      </c>
-      <c r="E18" t="s">
-        <v>147</v>
-      </c>
-      <c r="F18" t="s">
         <v>150</v>
       </c>
     </row>
@@ -26904,15 +26852,6 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79BA2CFD-36F5-ED48-BA61-D06C52A754BA}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6FF6C9F4-4010-9243-98AE-74EEEFFCAC53}">
   <dimension ref="A1:L87"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
Changed wide _target columns to _value columns. Changed mapping config exprValue columns to targetExpr columns
</commit_message>
<xml_diff>
--- a/data/mapping_config_files/NWSS-to-ODM-dictionary.xlsx
+++ b/data/mapping_config_files/NWSS-to-ODM-dictionary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-MapGenerator/PHES-ODM-MapGenerator/data/mapping_config_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A5DC79A-7FEE-6549-9EC3-331B947A808C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69C406B1-0321-6E49-B1E5-D658FAC8A4E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2020" yWindow="500" windowWidth="38940" windowHeight="20920" activeTab="2" xr2:uid="{77810E24-F86B-BC44-A0D5-8790E6EC60B4}"/>
+    <workbookView xWindow="2020" yWindow="500" windowWidth="38940" windowHeight="20920" xr2:uid="{77810E24-F86B-BC44-A0D5-8790E6EC60B4}"/>
   </bookViews>
   <sheets>
     <sheet name="maps" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3216" uniqueCount="836">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3216" uniqueCount="837">
   <si>
     <t>Reporter</t>
   </si>
@@ -2393,48 +2393,6 @@
     <t>custodyCont</t>
   </si>
   <si>
-    <t>specimen_target</t>
-  </si>
-  <si>
-    <t>measure_target</t>
-  </si>
-  <si>
-    <t>method_target</t>
-  </si>
-  <si>
-    <t>value_target</t>
-  </si>
-  <si>
-    <t>unit_target</t>
-  </si>
-  <si>
-    <t>aggregation_target</t>
-  </si>
-  <si>
-    <t>{ "notes_target" : "{{pretreatment_specify}}" }</t>
-  </si>
-  <si>
-    <t>{"reflink_target": "{{stan_ref}}"}</t>
-  </si>
-  <si>
-    <t>{"reflink_target": "{{pcr_gene_target_ref}}", "group_target": "{{pcr_target}}"}</t>
-  </si>
-  <si>
-    <t>{"reflink_target": "{{pcr_gene_target_ref}}"}</t>
-  </si>
-  <si>
-    <t>{"reflink_target": "{{lod_ref}}"}</t>
-  </si>
-  <si>
-    <t>{"reflink_target": "{{hum_frac_target_mic_ref}}"}</t>
-  </si>
-  <si>
-    <t>{"reflink_target": "{{hum_frac_target_chem_ref}}"}</t>
-  </si>
-  <si>
-    <t>{"reflink_target": "{{other_norm_ref}}"}</t>
-  </si>
-  <si>
     <t>id</t>
   </si>
   <si>
@@ -2543,9 +2501,6 @@
     <t>flagJcaOnOttOttawasite1202008021000covN1002</t>
   </si>
   <si>
-    <t>qualityFlag_target</t>
-  </si>
-  <si>
     <t>{{qc_ignore}}</t>
   </si>
   <si>
@@ -2568,9 +2523,6 @@
   </si>
   <si>
     <t>{{id:qualityReportID5}}</t>
-  </si>
-  <si>
-    <t>qualityReportID_target</t>
   </si>
   <si>
     <t>{{quality_flag}}</t>
@@ -2592,6 +2544,57 @@
         return "flagFI"
     return "ignore"
 target = get_qualityFlag(src.inhibition_detect, src.inhibition_adjust)</t>
+  </si>
+  <si>
+    <t>qualityReportID_value</t>
+  </si>
+  <si>
+    <t>qualityFlag_value</t>
+  </si>
+  <si>
+    <t>{ "notes_value" : "{{pretreatment_specify}}" }</t>
+  </si>
+  <si>
+    <t>{"reflink_value": "{{stan_ref}}"}</t>
+  </si>
+  <si>
+    <t>{"reflink_value": "{{pcr_gene_target_ref}}", "group_value": "{{pcr_target}}"}</t>
+  </si>
+  <si>
+    <t>{"reflink_value": "{{pcr_gene_target_ref}}"}</t>
+  </si>
+  <si>
+    <t>{"reflink_value": "{{lod_ref}}"}</t>
+  </si>
+  <si>
+    <t>{"reflink_value": "{{hum_frac_target_mic_ref}}"}</t>
+  </si>
+  <si>
+    <t>{"reflink_value": "{{hum_frac_target_chem_ref}}"}</t>
+  </si>
+  <si>
+    <t>{"reflink_value": "{{other_norm_ref}}"}</t>
+  </si>
+  <si>
+    <t>specimen_value</t>
+  </si>
+  <si>
+    <t>measure_value</t>
+  </si>
+  <si>
+    <t>method_value</t>
+  </si>
+  <si>
+    <t>value_value</t>
+  </si>
+  <si>
+    <t>unit_value</t>
+  </si>
+  <si>
+    <t>aggregation_value</t>
+  </si>
+  <si>
+    <t>targetExpr</t>
   </si>
 </sst>
 </file>
@@ -14172,7 +14175,7 @@
         <v>640</v>
       </c>
       <c r="I1" s="9" t="s">
-        <v>681</v>
+        <v>836</v>
       </c>
       <c r="J1" s="9" t="s">
         <v>682</v>
@@ -14294,7 +14297,7 @@
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
       <c r="L5" t="s">
-        <v>833</v>
+        <v>817</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
@@ -14566,7 +14569,7 @@
       <c r="J16" s="6"/>
       <c r="K16" s="2"/>
       <c r="L16" s="22" t="s">
-        <v>833</v>
+        <v>817</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.2">
@@ -16545,7 +16548,7 @@
         <v>635</v>
       </c>
       <c r="D93" s="2" t="s">
-        <v>807</v>
+        <v>793</v>
       </c>
       <c r="E93" s="2"/>
       <c r="F93" s="2" t="s">
@@ -16571,7 +16574,7 @@
         <v>635</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>812</v>
+        <v>798</v>
       </c>
       <c r="E94" s="2"/>
       <c r="F94" s="2" t="s">
@@ -16597,7 +16600,7 @@
         <v>635</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>807</v>
+        <v>793</v>
       </c>
       <c r="E95" s="2"/>
       <c r="F95" s="2" t="s">
@@ -16623,7 +16626,7 @@
         <v>635</v>
       </c>
       <c r="D96" s="2" t="s">
-        <v>805</v>
+        <v>791</v>
       </c>
       <c r="E96" s="2"/>
       <c r="F96" s="2" t="s">
@@ -16649,7 +16652,7 @@
         <v>635</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>808</v>
+        <v>794</v>
       </c>
       <c r="E97" s="2"/>
       <c r="F97" s="2" t="s">
@@ -16675,7 +16678,7 @@
         <v>635</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>805</v>
+        <v>791</v>
       </c>
       <c r="E98" s="2"/>
       <c r="F98" s="2" t="s">
@@ -16701,7 +16704,7 @@
         <v>635</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>808</v>
+        <v>794</v>
       </c>
       <c r="E99" s="2"/>
       <c r="F99" s="2" t="s">
@@ -16727,7 +16730,7 @@
         <v>635</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>810</v>
+        <v>796</v>
       </c>
       <c r="E100" s="2"/>
       <c r="F100" s="2" t="s">
@@ -16753,7 +16756,7 @@
         <v>635</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>809</v>
+        <v>795</v>
       </c>
       <c r="E101" s="2"/>
       <c r="F101" s="2" t="s">
@@ -16779,7 +16782,7 @@
         <v>635</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>807</v>
+        <v>793</v>
       </c>
       <c r="E102" s="2"/>
       <c r="F102" s="2" t="s">
@@ -16805,7 +16808,7 @@
         <v>635</v>
       </c>
       <c r="D103" s="2" t="s">
-        <v>807</v>
+        <v>793</v>
       </c>
       <c r="E103" s="2"/>
       <c r="F103" s="2" t="s">
@@ -16831,7 +16834,7 @@
         <v>635</v>
       </c>
       <c r="D104" s="2" t="s">
-        <v>807</v>
+        <v>793</v>
       </c>
       <c r="E104" s="2"/>
       <c r="F104" s="2" t="s">
@@ -16897,22 +16900,22 @@
         <v>698</v>
       </c>
       <c r="H1" s="11" t="s">
-        <v>771</v>
+        <v>830</v>
       </c>
       <c r="I1" s="11" t="s">
-        <v>772</v>
+        <v>831</v>
       </c>
       <c r="J1" s="11" t="s">
-        <v>773</v>
+        <v>832</v>
       </c>
       <c r="K1" s="11" t="s">
-        <v>774</v>
+        <v>833</v>
       </c>
       <c r="L1" s="11" t="s">
-        <v>775</v>
+        <v>834</v>
       </c>
       <c r="M1" s="11" t="s">
-        <v>776</v>
+        <v>835</v>
       </c>
       <c r="N1" s="12" t="s">
         <v>121</v>
@@ -17164,7 +17167,7 @@
         <v>650</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>777</v>
+        <v>822</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>165</v>
@@ -17366,7 +17369,7 @@
         <v>28</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>832</v>
+        <v>816</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>152</v>
@@ -19860,7 +19863,7 @@
         <v>37</v>
       </c>
       <c r="D82" s="3" t="s">
-        <v>832</v>
+        <v>816</v>
       </c>
       <c r="E82" s="2" t="s">
         <v>152</v>
@@ -20485,7 +20488,7 @@
         <v>38</v>
       </c>
       <c r="D99" s="3" t="s">
-        <v>832</v>
+        <v>816</v>
       </c>
       <c r="E99" s="2" t="s">
         <v>152</v>
@@ -21147,7 +21150,7 @@
         <v>408</v>
       </c>
       <c r="G118" s="2" t="s">
-        <v>778</v>
+        <v>823</v>
       </c>
       <c r="H118" s="2" t="s">
         <v>76</v>
@@ -21523,7 +21526,7 @@
         <v>650</v>
       </c>
       <c r="G128" s="2" t="s">
-        <v>779</v>
+        <v>824</v>
       </c>
       <c r="H128" s="2" t="s">
         <v>165</v>
@@ -21565,7 +21568,7 @@
         <v>650</v>
       </c>
       <c r="G129" s="2" t="s">
-        <v>780</v>
+        <v>825</v>
       </c>
       <c r="H129" s="2" t="s">
         <v>165</v>
@@ -21607,7 +21610,7 @@
         <v>650</v>
       </c>
       <c r="G130" s="2" t="s">
-        <v>780</v>
+        <v>825</v>
       </c>
       <c r="H130" s="2" t="s">
         <v>165</v>
@@ -21649,7 +21652,7 @@
         <v>650</v>
       </c>
       <c r="G131" s="2" t="s">
-        <v>780</v>
+        <v>825</v>
       </c>
       <c r="H131" s="2" t="s">
         <v>165</v>
@@ -21691,7 +21694,7 @@
         <v>650</v>
       </c>
       <c r="G132" s="2" t="s">
-        <v>781</v>
+        <v>826</v>
       </c>
       <c r="H132" s="2" t="s">
         <v>165</v>
@@ -21773,7 +21776,7 @@
         <v>650</v>
       </c>
       <c r="G134" s="2" t="s">
-        <v>782</v>
+        <v>827</v>
       </c>
       <c r="H134" s="2" t="s">
         <v>165</v>
@@ -21813,7 +21816,7 @@
         <v>650</v>
       </c>
       <c r="G135" s="2" t="s">
-        <v>783</v>
+        <v>828</v>
       </c>
       <c r="H135" s="2" t="s">
         <v>165</v>
@@ -21853,7 +21856,7 @@
         <v>650</v>
       </c>
       <c r="G136" s="2" t="s">
-        <v>784</v>
+        <v>829</v>
       </c>
       <c r="H136" s="2" t="s">
         <v>165</v>
@@ -21909,7 +21912,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B4CA3B6-4765-0A43-8534-6DA7BF8A336D}">
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="18.6640625" bestFit="1" customWidth="1"/>
@@ -21943,13 +21946,13 @@
         <v>698</v>
       </c>
       <c r="H1" s="9" t="s">
-        <v>830</v>
+        <v>820</v>
       </c>
       <c r="I1" s="11" t="s">
         <v>821</v>
       </c>
       <c r="J1" s="11" t="s">
-        <v>834</v>
+        <v>818</v>
       </c>
       <c r="K1" s="12" t="s">
         <v>121</v>
@@ -21975,10 +21978,10 @@
         <v>149</v>
       </c>
       <c r="H2" t="s">
-        <v>823</v>
+        <v>808</v>
       </c>
       <c r="I2" t="s">
-        <v>822</v>
+        <v>807</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
@@ -22012,7 +22015,7 @@
         <v>56</v>
       </c>
       <c r="D4" t="s">
-        <v>832</v>
+        <v>816</v>
       </c>
       <c r="E4" t="s">
         <v>147</v>
@@ -22021,32 +22024,6 @@
         <v>150</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A5" t="b">
-        <v>1</v>
-      </c>
-      <c r="B5" t="s">
-        <v>635</v>
-      </c>
-      <c r="C5" t="s">
-        <v>64</v>
-      </c>
-      <c r="D5" t="s">
-        <v>141</v>
-      </c>
-      <c r="E5" t="s">
-        <v>147</v>
-      </c>
-      <c r="F5" t="s">
-        <v>596</v>
-      </c>
-      <c r="H5" t="s">
-        <v>824</v>
-      </c>
-      <c r="I5" t="s">
-        <v>825</v>
-      </c>
-    </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" t="b">
         <v>1</v>
@@ -22058,13 +22035,19 @@
         <v>64</v>
       </c>
       <c r="D6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E6" t="s">
         <v>147</v>
       </c>
       <c r="F6" t="s">
-        <v>598</v>
+        <v>596</v>
+      </c>
+      <c r="H6" t="s">
+        <v>809</v>
+      </c>
+      <c r="I6" t="s">
+        <v>810</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
@@ -22078,7 +22061,7 @@
         <v>64</v>
       </c>
       <c r="D7" t="s">
-        <v>832</v>
+        <v>142</v>
       </c>
       <c r="E7" t="s">
         <v>147</v>
@@ -22095,62 +22078,42 @@
         <v>635</v>
       </c>
       <c r="C8" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D8" t="s">
-        <v>141</v>
+        <v>816</v>
       </c>
       <c r="E8" t="s">
         <v>147</v>
       </c>
       <c r="F8" t="s">
-        <v>602</v>
-      </c>
-      <c r="H8" t="s">
-        <v>826</v>
-      </c>
-      <c r="I8" t="s">
-        <v>827</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A9" t="b">
-        <v>1</v>
-      </c>
-      <c r="B9" t="s">
-        <v>635</v>
-      </c>
-      <c r="C9" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A10" t="b">
+        <v>1</v>
+      </c>
+      <c r="B10" t="s">
+        <v>635</v>
+      </c>
+      <c r="C10" t="s">
         <v>66</v>
       </c>
-      <c r="D9" t="s">
-        <v>142</v>
-      </c>
-      <c r="E9" t="s">
-        <v>147</v>
-      </c>
-      <c r="F9" t="s">
-        <v>598</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="19" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" t="b">
-        <v>1</v>
-      </c>
-      <c r="B10" t="s">
-        <v>635</v>
-      </c>
-      <c r="C10" t="s">
-        <v>68</v>
+      <c r="D10" t="s">
+        <v>141</v>
       </c>
       <c r="E10" t="s">
         <v>147</v>
       </c>
+      <c r="F10" t="s">
+        <v>602</v>
+      </c>
       <c r="H10" t="s">
-        <v>828</v>
-      </c>
-      <c r="J10" s="34" t="s">
-        <v>835</v>
+        <v>811</v>
+      </c>
+      <c r="I10" t="s">
+        <v>812</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.2">
@@ -22161,45 +22124,19 @@
         <v>635</v>
       </c>
       <c r="C11" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="D11" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E11" t="s">
         <v>147</v>
       </c>
       <c r="F11" t="s">
-        <v>149</v>
-      </c>
-      <c r="H11" t="s">
-        <v>829</v>
-      </c>
-      <c r="I11" t="s">
-        <v>831</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A12" t="b">
-        <v>1</v>
-      </c>
-      <c r="B12" t="s">
-        <v>635</v>
-      </c>
-      <c r="C12" t="s">
-        <v>73</v>
-      </c>
-      <c r="D12" t="s">
-        <v>142</v>
-      </c>
-      <c r="E12" t="s">
-        <v>147</v>
-      </c>
-      <c r="F12" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="19" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" t="b">
         <v>1</v>
       </c>
@@ -22207,15 +22144,84 @@
         <v>635</v>
       </c>
       <c r="C13" t="s">
-        <v>73</v>
-      </c>
-      <c r="D13" t="s">
-        <v>832</v>
+        <v>68</v>
       </c>
       <c r="E13" t="s">
         <v>147</v>
       </c>
-      <c r="F13" t="s">
+      <c r="H13" t="s">
+        <v>813</v>
+      </c>
+      <c r="J13" s="34" t="s">
+        <v>819</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="J14" s="34"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A15" t="b">
+        <v>1</v>
+      </c>
+      <c r="B15" t="s">
+        <v>635</v>
+      </c>
+      <c r="C15" t="s">
+        <v>73</v>
+      </c>
+      <c r="D15" t="s">
+        <v>141</v>
+      </c>
+      <c r="E15" t="s">
+        <v>147</v>
+      </c>
+      <c r="F15" t="s">
+        <v>149</v>
+      </c>
+      <c r="H15" t="s">
+        <v>814</v>
+      </c>
+      <c r="I15" t="s">
+        <v>815</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A16" t="b">
+        <v>1</v>
+      </c>
+      <c r="B16" t="s">
+        <v>635</v>
+      </c>
+      <c r="C16" t="s">
+        <v>73</v>
+      </c>
+      <c r="D16" t="s">
+        <v>142</v>
+      </c>
+      <c r="E16" t="s">
+        <v>147</v>
+      </c>
+      <c r="F16" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17" t="b">
+        <v>1</v>
+      </c>
+      <c r="B17" t="s">
+        <v>635</v>
+      </c>
+      <c r="C17" t="s">
+        <v>73</v>
+      </c>
+      <c r="D17" t="s">
+        <v>816</v>
+      </c>
+      <c r="E17" t="s">
+        <v>147</v>
+      </c>
+      <c r="F17" t="s">
         <v>150</v>
       </c>
     </row>
@@ -25996,13 +26002,13 @@
         <v>636</v>
       </c>
       <c r="E1" s="23" t="s">
-        <v>785</v>
+        <v>771</v>
       </c>
       <c r="F1" s="23" t="s">
-        <v>803</v>
+        <v>789</v>
       </c>
       <c r="G1" s="23" t="s">
-        <v>804</v>
+        <v>790</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
@@ -26016,13 +26022,13 @@
         <v>747</v>
       </c>
       <c r="E2" t="s">
-        <v>812</v>
+        <v>798</v>
       </c>
       <c r="F2" t="s">
-        <v>814</v>
+        <v>800</v>
       </c>
       <c r="G2" t="s">
-        <v>813</v>
+        <v>799</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -26033,7 +26039,7 @@
         <v>743</v>
       </c>
       <c r="E3" t="s">
-        <v>807</v>
+        <v>793</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -26047,13 +26053,13 @@
         <v>742</v>
       </c>
       <c r="E5" t="s">
-        <v>805</v>
+        <v>791</v>
       </c>
       <c r="F5" t="s">
-        <v>791</v>
+        <v>777</v>
       </c>
       <c r="G5" t="s">
-        <v>786</v>
+        <v>772</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -26073,10 +26079,10 @@
         <v>719</v>
       </c>
       <c r="F6" t="s">
-        <v>790</v>
+        <v>776</v>
       </c>
       <c r="G6" t="s">
-        <v>789</v>
+        <v>775</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -26093,10 +26099,10 @@
         <v>716</v>
       </c>
       <c r="F7" t="s">
-        <v>792</v>
+        <v>778</v>
       </c>
       <c r="G7" t="s">
-        <v>787</v>
+        <v>773</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
@@ -26110,13 +26116,13 @@
         <v>745</v>
       </c>
       <c r="E8" t="s">
-        <v>806</v>
+        <v>792</v>
       </c>
       <c r="F8" t="s">
-        <v>795</v>
+        <v>781</v>
       </c>
       <c r="G8" t="s">
-        <v>794</v>
+        <v>780</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
@@ -26133,10 +26139,10 @@
         <v>710</v>
       </c>
       <c r="F9" t="s">
-        <v>793</v>
+        <v>779</v>
       </c>
       <c r="G9" t="s">
-        <v>788</v>
+        <v>774</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
@@ -26150,13 +26156,13 @@
         <v>743</v>
       </c>
       <c r="E10" t="s">
-        <v>807</v>
+        <v>793</v>
       </c>
       <c r="F10" t="s">
-        <v>797</v>
+        <v>783</v>
       </c>
       <c r="G10" t="s">
-        <v>796</v>
+        <v>782</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
@@ -26170,13 +26176,13 @@
         <v>744</v>
       </c>
       <c r="E11" t="s">
-        <v>808</v>
+        <v>794</v>
       </c>
       <c r="F11" t="s">
-        <v>799</v>
+        <v>785</v>
       </c>
       <c r="G11" t="s">
-        <v>798</v>
+        <v>784</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
@@ -26193,10 +26199,10 @@
         <v>717</v>
       </c>
       <c r="F12" t="s">
-        <v>797</v>
+        <v>783</v>
       </c>
       <c r="G12" t="s">
-        <v>800</v>
+        <v>786</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
@@ -26216,10 +26222,10 @@
         <v>709</v>
       </c>
       <c r="F13" t="s">
-        <v>801</v>
+        <v>787</v>
       </c>
       <c r="G13" t="s">
-        <v>802</v>
+        <v>788</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
@@ -26264,7 +26270,7 @@
         <v>743</v>
       </c>
       <c r="E17" t="s">
-        <v>807</v>
+        <v>793</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
@@ -26306,13 +26312,13 @@
         <v>752</v>
       </c>
       <c r="E21" t="s">
-        <v>809</v>
+        <v>795</v>
       </c>
       <c r="F21" t="s">
-        <v>818</v>
+        <v>804</v>
       </c>
       <c r="G21" t="s">
-        <v>817</v>
+        <v>803</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
@@ -26354,13 +26360,13 @@
         <v>753</v>
       </c>
       <c r="E24" t="s">
-        <v>810</v>
+        <v>796</v>
       </c>
       <c r="F24" t="s">
-        <v>816</v>
+        <v>802</v>
       </c>
       <c r="G24" t="s">
-        <v>815</v>
+        <v>801</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
@@ -26374,13 +26380,13 @@
         <v>749</v>
       </c>
       <c r="E26" t="s">
-        <v>811</v>
+        <v>797</v>
       </c>
       <c r="F26" t="s">
-        <v>820</v>
+        <v>806</v>
       </c>
       <c r="G26" t="s">
-        <v>819</v>
+        <v>805</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
@@ -26394,7 +26400,7 @@
         <v>742</v>
       </c>
       <c r="E27" t="s">
-        <v>805</v>
+        <v>791</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
@@ -26422,7 +26428,7 @@
         <v>744</v>
       </c>
       <c r="E29" t="s">
-        <v>808</v>
+        <v>794</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
@@ -26512,7 +26518,7 @@
         <v>743</v>
       </c>
       <c r="E36" t="s">
-        <v>807</v>
+        <v>793</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
@@ -26554,7 +26560,7 @@
         <v>743</v>
       </c>
       <c r="E40" t="s">
-        <v>807</v>
+        <v>793</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
@@ -26568,13 +26574,13 @@
         <v>745</v>
       </c>
       <c r="E41" t="s">
-        <v>806</v>
+        <v>792</v>
       </c>
       <c r="F41" t="s">
-        <v>795</v>
+        <v>781</v>
       </c>
       <c r="G41" t="s">
-        <v>794</v>
+        <v>780</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
@@ -26588,7 +26594,7 @@
         <v>747</v>
       </c>
       <c r="E42" t="s">
-        <v>812</v>
+        <v>798</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Replaced NA with blank string, [empty] with <empty>
</commit_message>
<xml_diff>
--- a/data/mapping_config_files/NWSS-to-ODM-dictionary.xlsx
+++ b/data/mapping_config_files/NWSS-to-ODM-dictionary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-MapGenerator/PHES-ODM-MapGenerator/data/mapping_config_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69C406B1-0321-6E49-B1E5-D658FAC8A4E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F954EFD8-4B08-3F45-A3DC-4037CFB16FDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2020" yWindow="500" windowWidth="38940" windowHeight="20920" xr2:uid="{77810E24-F86B-BC44-A0D5-8790E6EC60B4}"/>
+    <workbookView xWindow="2020" yWindow="500" windowWidth="38940" windowHeight="20920" activeTab="3" xr2:uid="{77810E24-F86B-BC44-A0D5-8790E6EC60B4}"/>
   </bookViews>
   <sheets>
     <sheet name="maps" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3216" uniqueCount="837">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2995" uniqueCount="837">
   <si>
     <t>Reporter</t>
   </si>
@@ -2601,7 +2601,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="15" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -2685,6 +2685,17 @@
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -2812,7 +2823,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -2868,6 +2879,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -14197,9 +14214,7 @@
       <c r="D2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="E2" s="2"/>
       <c r="F2" s="1" t="s">
         <v>115</v>
       </c>
@@ -14229,9 +14244,7 @@
       <c r="D3" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="E3" s="2"/>
       <c r="F3" s="2" t="s">
         <v>115</v>
       </c>
@@ -14325,9 +14338,7 @@
       <c r="D7" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E7" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="E7" s="2"/>
       <c r="F7" s="2" t="s">
         <v>77</v>
       </c>
@@ -14386,9 +14397,7 @@
       <c r="D9" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E9" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="E9" s="2"/>
       <c r="F9" s="2" t="s">
         <v>79</v>
       </c>
@@ -14415,9 +14424,7 @@
       <c r="D10" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E10" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="E10" s="2"/>
       <c r="F10" s="2" t="s">
         <v>77</v>
       </c>
@@ -14586,36 +14593,34 @@
       <c r="L17" s="23"/>
     </row>
     <row r="18" spans="1:12" s="23" customFormat="1" ht="17" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="23" t="b">
-        <v>1</v>
-      </c>
-      <c r="B18" s="28" t="s">
-        <v>1</v>
-      </c>
-      <c r="C18" s="28" t="s">
-        <v>635</v>
-      </c>
-      <c r="D18" s="28" t="s">
+      <c r="A18" s="35" t="b">
+        <v>1</v>
+      </c>
+      <c r="B18" s="36" t="s">
+        <v>1</v>
+      </c>
+      <c r="C18" s="36" t="s">
+        <v>635</v>
+      </c>
+      <c r="D18" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="E18" s="29" t="s">
+      <c r="E18" s="37" t="s">
         <v>85</v>
       </c>
-      <c r="F18" s="28" t="s">
+      <c r="F18" s="36" t="s">
         <v>77</v>
       </c>
-      <c r="G18" s="28" t="s">
+      <c r="G18" s="36" t="s">
         <v>101</v>
       </c>
-      <c r="H18" s="28" t="s">
+      <c r="H18" s="36" t="s">
         <v>76</v>
       </c>
-      <c r="I18" s="28"/>
-      <c r="J18" s="28"/>
-      <c r="K18" s="28"/>
-      <c r="L18" s="19" t="s">
-        <v>738</v>
-      </c>
+      <c r="I18" s="36"/>
+      <c r="J18" s="36"/>
+      <c r="K18" s="36"/>
+      <c r="L18" s="38"/>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" t="b">
@@ -15242,9 +15247,7 @@
       <c r="D41" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E41" s="3" t="s">
-        <v>76</v>
-      </c>
+      <c r="E41" s="3"/>
       <c r="F41" s="2" t="s">
         <v>118</v>
       </c>
@@ -15527,9 +15530,7 @@
       <c r="D52" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="E52" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="E52" s="2"/>
       <c r="F52" s="2" t="s">
         <v>118</v>
       </c>
@@ -15556,9 +15557,7 @@
       <c r="D53" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="E53" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="E53" s="2"/>
       <c r="F53" s="2" t="s">
         <v>118</v>
       </c>
@@ -15585,9 +15584,7 @@
       <c r="D54" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="E54" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="E54" s="2"/>
       <c r="F54" s="2" t="s">
         <v>118</v>
       </c>
@@ -15626,9 +15623,7 @@
       <c r="D56" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="E56" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="E56" s="2"/>
       <c r="F56" s="2" t="s">
         <v>118</v>
       </c>
@@ -15655,9 +15650,7 @@
       <c r="D57" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="E57" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="E57" s="2"/>
       <c r="F57" s="2" t="s">
         <v>118</v>
       </c>
@@ -15755,7 +15748,7 @@
         <v>57</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>143</v>
+        <v>816</v>
       </c>
       <c r="F61" s="2" t="s">
         <v>118</v>
@@ -15860,7 +15853,7 @@
         <v>58</v>
       </c>
       <c r="E65" s="2" t="s">
-        <v>143</v>
+        <v>816</v>
       </c>
       <c r="F65" s="2" t="s">
         <v>118</v>
@@ -15968,7 +15961,7 @@
         <v>56</v>
       </c>
       <c r="E69" s="2" t="s">
-        <v>143</v>
+        <v>816</v>
       </c>
       <c r="F69" s="2" t="s">
         <v>147</v>
@@ -16071,7 +16064,7 @@
         <v>64</v>
       </c>
       <c r="E73" s="3" t="s">
-        <v>143</v>
+        <v>816</v>
       </c>
       <c r="F73" s="2" t="s">
         <v>147</v>
@@ -16350,7 +16343,7 @@
         <v>69</v>
       </c>
       <c r="E84" s="3" t="s">
-        <v>143</v>
+        <v>816</v>
       </c>
       <c r="F84" s="2" t="s">
         <v>147</v>
@@ -16358,9 +16351,7 @@
       <c r="G84" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="H84" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="H84" s="2"/>
       <c r="I84" s="2"/>
       <c r="J84" s="2"/>
       <c r="K84" s="1" t="s">
@@ -16455,7 +16446,7 @@
         <v>73</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>143</v>
+        <v>816</v>
       </c>
       <c r="F88" s="2" t="s">
         <v>147</v>
@@ -16869,7 +16860,7 @@
     <col min="2" max="2" width="28.6640625" customWidth="1"/>
     <col min="3" max="4" width="25.5" customWidth="1"/>
     <col min="5" max="7" width="22.5" customWidth="1"/>
-    <col min="8" max="8" width="14.83203125" customWidth="1"/>
+    <col min="8" max="8" width="28" customWidth="1"/>
     <col min="9" max="10" width="29.33203125" customWidth="1"/>
     <col min="11" max="11" width="23.5" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="15.5" customWidth="1"/>
@@ -17065,12 +17056,8 @@
       <c r="K5" s="2" t="s">
         <v>654</v>
       </c>
-      <c r="L5" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M5" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L5" s="2"/>
+      <c r="M5" s="2"/>
       <c r="N5" s="2"/>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
@@ -17181,12 +17168,8 @@
       <c r="K8" s="2" t="s">
         <v>641</v>
       </c>
-      <c r="L8" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M8" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L8" s="2"/>
+      <c r="M8" s="2"/>
       <c r="N8" s="2"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
@@ -17224,9 +17207,7 @@
         <v>423</v>
       </c>
       <c r="G10" s="2"/>
-      <c r="H10" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="H10" s="2"/>
       <c r="I10" s="2" t="s">
         <v>650</v>
       </c>
@@ -17236,12 +17217,8 @@
       <c r="K10" s="2" t="s">
         <v>684</v>
       </c>
-      <c r="L10" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M10" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L10" s="2"/>
+      <c r="M10" s="2"/>
       <c r="N10" s="2"/>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
@@ -17274,12 +17251,8 @@
       <c r="K11" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L11" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M11" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L11" s="2"/>
+      <c r="M11" s="2"/>
       <c r="N11" s="2"/>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.2">
@@ -17312,12 +17285,8 @@
       <c r="K12" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L12" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M12" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L12" s="2"/>
+      <c r="M12" s="2"/>
       <c r="N12" s="2"/>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.2">
@@ -17350,12 +17319,8 @@
       <c r="K13" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L13" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M13" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L13" s="2"/>
+      <c r="M13" s="2"/>
       <c r="N13" s="2"/>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.2">
@@ -17374,9 +17339,7 @@
       <c r="E14" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="F14" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="F14" s="2"/>
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
       <c r="I14" s="2" t="s">
@@ -17388,12 +17351,8 @@
       <c r="K14" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L14" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M14" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L14" s="2"/>
+      <c r="M14" s="2"/>
       <c r="N14" s="2"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.2">
@@ -17431,9 +17390,7 @@
         <v>429</v>
       </c>
       <c r="G16" s="2"/>
-      <c r="H16" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="H16" s="2"/>
       <c r="I16" s="2" t="s">
         <v>650</v>
       </c>
@@ -17443,12 +17400,8 @@
       <c r="K16" s="2" t="s">
         <v>685</v>
       </c>
-      <c r="L16" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M16" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L16" s="2"/>
+      <c r="M16" s="2"/>
       <c r="N16" s="2"/>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.2">
@@ -17481,12 +17434,8 @@
       <c r="K17" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L17" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M17" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L17" s="2"/>
+      <c r="M17" s="2"/>
       <c r="N17" s="2"/>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.2">
@@ -17519,12 +17468,8 @@
       <c r="K18" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L18" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M18" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L18" s="2"/>
+      <c r="M18" s="2"/>
       <c r="N18" s="2"/>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.2">
@@ -17557,12 +17502,8 @@
       <c r="K19" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L19" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M19" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L19" s="2"/>
+      <c r="M19" s="2"/>
       <c r="N19" s="2"/>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.2">
@@ -17593,12 +17534,8 @@
         <v>650</v>
       </c>
       <c r="K20" s="2"/>
-      <c r="L20" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M20" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L20" s="2"/>
+      <c r="M20" s="2"/>
       <c r="N20" s="2"/>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.2">
@@ -17631,12 +17568,8 @@
       <c r="K21" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L21" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M21" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L21" s="2"/>
+      <c r="M21" s="2"/>
       <c r="N21" s="2"/>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.2">
@@ -17669,12 +17602,8 @@
       <c r="K22" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L22" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M22" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L22" s="2"/>
+      <c r="M22" s="2"/>
       <c r="N22" s="2"/>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.2">
@@ -17707,12 +17636,8 @@
       <c r="K23" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L23" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M23" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L23" s="2"/>
+      <c r="M23" s="2"/>
       <c r="N23" s="2"/>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.2">
@@ -17745,12 +17670,8 @@
       <c r="K24" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L24" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M24" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L24" s="2"/>
+      <c r="M24" s="2"/>
       <c r="N24" s="2"/>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.2">
@@ -17783,12 +17704,8 @@
       <c r="K25" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L25" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M25" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L25" s="2"/>
+      <c r="M25" s="2"/>
       <c r="N25" s="2"/>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.2">
@@ -17821,12 +17738,8 @@
       <c r="K26" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L26" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M26" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L26" s="2"/>
+      <c r="M26" s="2"/>
       <c r="N26" s="2"/>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.2">
@@ -17859,12 +17772,8 @@
       <c r="K27" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L27" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M27" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L27" s="2"/>
+      <c r="M27" s="2"/>
       <c r="N27" s="2"/>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.2">
@@ -17897,12 +17806,8 @@
       <c r="K28" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L28" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M28" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L28" s="2"/>
+      <c r="M28" s="2"/>
       <c r="N28" s="2"/>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.2">
@@ -17935,12 +17840,8 @@
       <c r="K29" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L29" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M29" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L29" s="2"/>
+      <c r="M29" s="2"/>
       <c r="N29" s="2"/>
     </row>
     <row r="30" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -17973,12 +17874,8 @@
       <c r="K30" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L30" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M30" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L30" s="2"/>
+      <c r="M30" s="2"/>
       <c r="N30" s="2"/>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.2">
@@ -18011,12 +17908,8 @@
       <c r="K31" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L31" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M31" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L31" s="2"/>
+      <c r="M31" s="2"/>
       <c r="N31" s="2"/>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.2">
@@ -18049,12 +17942,8 @@
       <c r="K32" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L32" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M32" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L32" s="2"/>
+      <c r="M32" s="2"/>
       <c r="N32" s="2"/>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.2">
@@ -18087,12 +17976,8 @@
       <c r="K33" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L33" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M33" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L33" s="2"/>
+      <c r="M33" s="2"/>
       <c r="N33" s="2"/>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.2">
@@ -18125,12 +18010,8 @@
       <c r="K34" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L34" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M34" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L34" s="2"/>
+      <c r="M34" s="2"/>
       <c r="N34" s="2"/>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.2">
@@ -18163,12 +18044,8 @@
       <c r="K35" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L35" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M35" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L35" s="2"/>
+      <c r="M35" s="2"/>
       <c r="N35" s="2"/>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.2">
@@ -18201,12 +18078,8 @@
       <c r="K36" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L36" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M36" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L36" s="2"/>
+      <c r="M36" s="2"/>
       <c r="N36" s="2"/>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.2">
@@ -18239,12 +18112,8 @@
       <c r="K37" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L37" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M37" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L37" s="2"/>
+      <c r="M37" s="2"/>
       <c r="N37" s="2"/>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.2">
@@ -18277,12 +18146,8 @@
       <c r="K38" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L38" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M38" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L38" s="2"/>
+      <c r="M38" s="2"/>
       <c r="N38" s="2"/>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.2">
@@ -18315,12 +18180,8 @@
       <c r="K39" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L39" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M39" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L39" s="2"/>
+      <c r="M39" s="2"/>
       <c r="N39" s="2"/>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.2">
@@ -18358,9 +18219,7 @@
         <v>447</v>
       </c>
       <c r="G41" s="2"/>
-      <c r="H41" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="H41" s="2"/>
       <c r="I41" s="2" t="s">
         <v>650</v>
       </c>
@@ -18370,12 +18229,8 @@
       <c r="K41" s="2" t="s">
         <v>686</v>
       </c>
-      <c r="L41" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M41" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L41" s="2"/>
+      <c r="M41" s="2"/>
       <c r="N41" s="2"/>
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.2">
@@ -18408,12 +18263,8 @@
       <c r="K42" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L42" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M42" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L42" s="2"/>
+      <c r="M42" s="2"/>
       <c r="N42" s="2"/>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.2">
@@ -18446,12 +18297,8 @@
       <c r="K43" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L43" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M43" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L43" s="2"/>
+      <c r="M43" s="2"/>
       <c r="N43" s="2"/>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.2">
@@ -18484,12 +18331,8 @@
       <c r="K44" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L44" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M44" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L44" s="2"/>
+      <c r="M44" s="2"/>
       <c r="N44" s="2"/>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.2">
@@ -18522,12 +18365,8 @@
       <c r="K45" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L45" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M45" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L45" s="2"/>
+      <c r="M45" s="2"/>
       <c r="N45" s="2"/>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.2">
@@ -18560,12 +18399,8 @@
       <c r="K46" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L46" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M46" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L46" s="2"/>
+      <c r="M46" s="2"/>
       <c r="N46" s="2"/>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.2">
@@ -18598,12 +18433,8 @@
       <c r="K47" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L47" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M47" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L47" s="2"/>
+      <c r="M47" s="2"/>
       <c r="N47" s="2"/>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.2">
@@ -18636,12 +18467,8 @@
       <c r="K48" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L48" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M48" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L48" s="2"/>
+      <c r="M48" s="2"/>
       <c r="N48" s="2"/>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.2">
@@ -18674,12 +18501,8 @@
       <c r="K49" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L49" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M49" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L49" s="2"/>
+      <c r="M49" s="2"/>
       <c r="N49" s="2"/>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.2">
@@ -18712,12 +18535,8 @@
       <c r="K50" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L50" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M50" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L50" s="2"/>
+      <c r="M50" s="2"/>
       <c r="N50" s="2"/>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.2">
@@ -18750,12 +18569,8 @@
       <c r="K51" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L51" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M51" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L51" s="2"/>
+      <c r="M51" s="2"/>
       <c r="N51" s="2"/>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.2">
@@ -18788,12 +18603,8 @@
       <c r="K52" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L52" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M52" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L52" s="2"/>
+      <c r="M52" s="2"/>
       <c r="N52" s="2"/>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.2">
@@ -18826,12 +18637,8 @@
       <c r="K53" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L53" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M53" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L53" s="2"/>
+      <c r="M53" s="2"/>
       <c r="N53" s="2"/>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.2">
@@ -18864,12 +18671,8 @@
       <c r="K54" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L54" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M54" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L54" s="2"/>
+      <c r="M54" s="2"/>
       <c r="N54" s="2"/>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.2">
@@ -18902,12 +18705,8 @@
       <c r="K55" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L55" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M55" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L55" s="2"/>
+      <c r="M55" s="2"/>
       <c r="N55" s="2"/>
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.2">
@@ -18940,12 +18739,8 @@
       <c r="K56" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L56" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M56" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L56" s="2"/>
+      <c r="M56" s="2"/>
       <c r="N56" s="2"/>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.2">
@@ -18978,12 +18773,8 @@
       <c r="K57" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L57" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M57" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L57" s="2"/>
+      <c r="M57" s="2"/>
       <c r="N57" s="2"/>
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.2">
@@ -19016,12 +18807,8 @@
       <c r="K58" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L58" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M58" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L58" s="2"/>
+      <c r="M58" s="2"/>
       <c r="N58" s="2"/>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.2">
@@ -19054,12 +18841,8 @@
       <c r="K59" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L59" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M59" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L59" s="2"/>
+      <c r="M59" s="2"/>
       <c r="N59" s="2"/>
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.2">
@@ -19092,12 +18875,8 @@
       <c r="K60" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L60" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M60" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L60" s="2"/>
+      <c r="M60" s="2"/>
       <c r="N60" s="2"/>
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.2">
@@ -19130,12 +18909,8 @@
       <c r="K61" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L61" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M61" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L61" s="2"/>
+      <c r="M61" s="2"/>
       <c r="N61" s="2"/>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.2">
@@ -19168,12 +18943,8 @@
       <c r="K62" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L62" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M62" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L62" s="2"/>
+      <c r="M62" s="2"/>
       <c r="N62" s="2"/>
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.2">
@@ -19206,12 +18977,8 @@
       <c r="K63" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L63" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M63" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L63" s="2"/>
+      <c r="M63" s="2"/>
       <c r="N63" s="2"/>
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.2">
@@ -19244,12 +19011,8 @@
       <c r="K64" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L64" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M64" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L64" s="2"/>
+      <c r="M64" s="2"/>
       <c r="N64" s="2"/>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.2">
@@ -19282,12 +19045,8 @@
       <c r="K65" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L65" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M65" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L65" s="2"/>
+      <c r="M65" s="2"/>
       <c r="N65" s="2"/>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.2">
@@ -19320,12 +19079,8 @@
       <c r="K66" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L66" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M66" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L66" s="2"/>
+      <c r="M66" s="2"/>
       <c r="N66" s="2"/>
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.2">
@@ -19358,12 +19113,8 @@
       <c r="K67" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L67" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M67" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L67" s="2"/>
+      <c r="M67" s="2"/>
       <c r="N67" s="2"/>
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.2">
@@ -19396,12 +19147,8 @@
       <c r="K68" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L68" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M68" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L68" s="2"/>
+      <c r="M68" s="2"/>
       <c r="N68" s="2"/>
     </row>
     <row r="69" spans="1:14" x14ac:dyDescent="0.2">
@@ -19434,12 +19181,8 @@
       <c r="K69" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L69" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M69" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L69" s="2"/>
+      <c r="M69" s="2"/>
       <c r="N69" s="2"/>
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.2">
@@ -19472,12 +19215,8 @@
       <c r="K70" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L70" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M70" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L70" s="2"/>
+      <c r="M70" s="2"/>
       <c r="N70" s="2"/>
     </row>
     <row r="71" spans="1:14" x14ac:dyDescent="0.2">
@@ -19510,12 +19249,8 @@
       <c r="K71" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L71" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M71" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L71" s="2"/>
+      <c r="M71" s="2"/>
       <c r="N71" s="2"/>
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.2">
@@ -19548,12 +19283,8 @@
       <c r="K72" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L72" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M72" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L72" s="2"/>
+      <c r="M72" s="2"/>
       <c r="N72" s="2"/>
     </row>
     <row r="73" spans="1:14" x14ac:dyDescent="0.2">
@@ -19586,12 +19317,8 @@
       <c r="K73" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L73" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M73" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L73" s="2"/>
+      <c r="M73" s="2"/>
       <c r="N73" s="2"/>
     </row>
     <row r="74" spans="1:14" x14ac:dyDescent="0.2">
@@ -19779,9 +19506,7 @@
         <v>650</v>
       </c>
       <c r="G79" s="2"/>
-      <c r="H79" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="H79" s="2"/>
       <c r="I79" s="2" t="s">
         <v>650</v>
       </c>
@@ -19817,9 +19542,7 @@
         <v>650</v>
       </c>
       <c r="G80" s="2"/>
-      <c r="H80" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="H80" s="2"/>
       <c r="I80" s="2" t="s">
         <v>650</v>
       </c>
@@ -19829,12 +19552,8 @@
       <c r="K80" s="2" t="s">
         <v>662</v>
       </c>
-      <c r="L80" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M80" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L80" s="2"/>
+      <c r="M80" s="2"/>
       <c r="N80" s="2"/>
     </row>
     <row r="81" spans="1:14" x14ac:dyDescent="0.2">
@@ -19868,13 +19587,9 @@
       <c r="E82" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="F82" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="F82" s="2"/>
       <c r="G82" s="2"/>
-      <c r="H82" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="H82" s="2"/>
       <c r="I82" s="2" t="s">
         <v>650</v>
       </c>
@@ -19884,12 +19599,8 @@
       <c r="K82" s="2" t="s">
         <v>687</v>
       </c>
-      <c r="L82" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M82" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L82" s="2"/>
+      <c r="M82" s="2"/>
       <c r="N82" s="2"/>
     </row>
     <row r="83" spans="1:14" x14ac:dyDescent="0.2">
@@ -19922,12 +19633,8 @@
       <c r="K83" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L83" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M83" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L83" s="2"/>
+      <c r="M83" s="2"/>
       <c r="N83" s="2"/>
     </row>
     <row r="84" spans="1:14" x14ac:dyDescent="0.2">
@@ -19960,12 +19667,8 @@
       <c r="K84" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L84" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M84" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L84" s="2"/>
+      <c r="M84" s="2"/>
       <c r="N84" s="2"/>
     </row>
     <row r="85" spans="1:14" x14ac:dyDescent="0.2">
@@ -19998,12 +19701,8 @@
       <c r="K85" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L85" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M85" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L85" s="2"/>
+      <c r="M85" s="2"/>
       <c r="N85" s="2"/>
     </row>
     <row r="86" spans="1:14" x14ac:dyDescent="0.2">
@@ -20036,12 +19735,8 @@
       <c r="K86" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L86" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M86" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L86" s="2"/>
+      <c r="M86" s="2"/>
       <c r="N86" s="2"/>
     </row>
     <row r="87" spans="1:14" x14ac:dyDescent="0.2">
@@ -20074,12 +19769,8 @@
       <c r="K87" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L87" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M87" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L87" s="2"/>
+      <c r="M87" s="2"/>
       <c r="N87" s="2"/>
     </row>
     <row r="88" spans="1:14" x14ac:dyDescent="0.2">
@@ -20112,12 +19803,8 @@
       <c r="K88" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L88" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M88" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L88" s="2"/>
+      <c r="M88" s="2"/>
       <c r="N88" s="2"/>
     </row>
     <row r="89" spans="1:14" x14ac:dyDescent="0.2">
@@ -20150,12 +19837,8 @@
       <c r="K89" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L89" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M89" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L89" s="2"/>
+      <c r="M89" s="2"/>
       <c r="N89" s="2"/>
     </row>
     <row r="90" spans="1:14" x14ac:dyDescent="0.2">
@@ -20188,12 +19871,8 @@
       <c r="K90" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L90" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M90" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L90" s="2"/>
+      <c r="M90" s="2"/>
       <c r="N90" s="2"/>
     </row>
     <row r="91" spans="1:14" x14ac:dyDescent="0.2">
@@ -20226,12 +19905,8 @@
       <c r="K91" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L91" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M91" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L91" s="2"/>
+      <c r="M91" s="2"/>
       <c r="N91" s="2"/>
     </row>
     <row r="92" spans="1:14" x14ac:dyDescent="0.2">
@@ -20264,12 +19939,8 @@
       <c r="K92" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L92" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M92" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L92" s="2"/>
+      <c r="M92" s="2"/>
       <c r="N92" s="2"/>
     </row>
     <row r="93" spans="1:14" x14ac:dyDescent="0.2">
@@ -20302,12 +19973,8 @@
       <c r="K93" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L93" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M93" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L93" s="2"/>
+      <c r="M93" s="2"/>
       <c r="N93" s="2"/>
     </row>
     <row r="94" spans="1:14" x14ac:dyDescent="0.2">
@@ -20340,12 +20007,8 @@
       <c r="K94" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L94" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M94" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L94" s="2"/>
+      <c r="M94" s="2"/>
       <c r="N94" s="2"/>
     </row>
     <row r="95" spans="1:14" x14ac:dyDescent="0.2">
@@ -20378,12 +20041,8 @@
       <c r="K95" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L95" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M95" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L95" s="2"/>
+      <c r="M95" s="2"/>
       <c r="N95" s="2"/>
     </row>
     <row r="96" spans="1:14" x14ac:dyDescent="0.2">
@@ -20416,12 +20075,8 @@
       <c r="K96" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L96" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M96" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L96" s="2"/>
+      <c r="M96" s="2"/>
       <c r="N96" s="2"/>
     </row>
     <row r="97" spans="1:14" x14ac:dyDescent="0.2">
@@ -20454,12 +20109,8 @@
       <c r="K97" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L97" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M97" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L97" s="2"/>
+      <c r="M97" s="2"/>
       <c r="N97" s="2"/>
     </row>
     <row r="98" spans="1:14" x14ac:dyDescent="0.2">
@@ -20493,13 +20144,9 @@
       <c r="E99" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="F99" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="F99" s="2"/>
       <c r="G99" s="2"/>
-      <c r="H99" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="H99" s="2"/>
       <c r="I99" s="2" t="s">
         <v>650</v>
       </c>
@@ -20509,12 +20156,8 @@
       <c r="K99" s="2" t="s">
         <v>688</v>
       </c>
-      <c r="L99" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M99" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L99" s="2"/>
+      <c r="M99" s="2"/>
       <c r="N99" s="2"/>
     </row>
     <row r="100" spans="1:14" x14ac:dyDescent="0.2">
@@ -20547,12 +20190,8 @@
       <c r="K100" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L100" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M100" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L100" s="2"/>
+      <c r="M100" s="2"/>
       <c r="N100" s="2"/>
     </row>
     <row r="101" spans="1:14" x14ac:dyDescent="0.2">
@@ -20585,12 +20224,8 @@
       <c r="K101" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L101" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M101" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L101" s="2"/>
+      <c r="M101" s="2"/>
       <c r="N101" s="2"/>
     </row>
     <row r="102" spans="1:14" x14ac:dyDescent="0.2">
@@ -20623,12 +20258,8 @@
       <c r="K102" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L102" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M102" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L102" s="2"/>
+      <c r="M102" s="2"/>
       <c r="N102" s="2"/>
     </row>
     <row r="103" spans="1:14" x14ac:dyDescent="0.2">
@@ -20661,12 +20292,8 @@
       <c r="K103" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L103" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M103" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L103" s="2"/>
+      <c r="M103" s="2"/>
       <c r="N103" s="2"/>
     </row>
     <row r="104" spans="1:14" x14ac:dyDescent="0.2">
@@ -20699,12 +20326,8 @@
       <c r="K104" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L104" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M104" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L104" s="2"/>
+      <c r="M104" s="2"/>
       <c r="N104" s="2"/>
     </row>
     <row r="105" spans="1:14" x14ac:dyDescent="0.2">
@@ -20737,12 +20360,8 @@
       <c r="K105" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L105" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M105" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L105" s="2"/>
+      <c r="M105" s="2"/>
       <c r="N105" s="2"/>
     </row>
     <row r="106" spans="1:14" x14ac:dyDescent="0.2">
@@ -20816,9 +20435,7 @@
         <v>650</v>
       </c>
       <c r="G108" s="2"/>
-      <c r="H108" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="H108" s="2"/>
       <c r="I108" s="2" t="s">
         <v>650</v>
       </c>
@@ -20828,12 +20445,8 @@
       <c r="K108" s="2" t="s">
         <v>664</v>
       </c>
-      <c r="L108" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M108" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L108" s="2"/>
+      <c r="M108" s="2"/>
       <c r="N108" s="2"/>
     </row>
     <row r="109" spans="1:14" x14ac:dyDescent="0.2">
@@ -20871,9 +20484,7 @@
         <v>389</v>
       </c>
       <c r="G110" s="2"/>
-      <c r="H110" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="H110" s="2"/>
       <c r="I110" s="2" t="s">
         <v>650</v>
       </c>
@@ -20883,12 +20494,8 @@
       <c r="K110" s="2" t="s">
         <v>689</v>
       </c>
-      <c r="L110" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M110" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L110" s="2"/>
+      <c r="M110" s="2"/>
       <c r="N110" s="2"/>
     </row>
     <row r="111" spans="1:14" x14ac:dyDescent="0.2">
@@ -20921,12 +20528,8 @@
       <c r="K111" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L111" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M111" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L111" s="2"/>
+      <c r="M111" s="2"/>
       <c r="N111" s="2"/>
     </row>
     <row r="112" spans="1:14" x14ac:dyDescent="0.2">
@@ -20959,12 +20562,8 @@
       <c r="K112" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L112" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M112" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L112" s="2"/>
+      <c r="M112" s="2"/>
       <c r="N112" s="2"/>
     </row>
     <row r="113" spans="1:14" x14ac:dyDescent="0.2">
@@ -20997,12 +20596,8 @@
       <c r="K113" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L113" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M113" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L113" s="2"/>
+      <c r="M113" s="2"/>
       <c r="N113" s="2"/>
     </row>
     <row r="114" spans="1:14" x14ac:dyDescent="0.2">
@@ -21035,12 +20630,8 @@
       <c r="K114" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L114" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M114" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L114" s="2"/>
+      <c r="M114" s="2"/>
       <c r="N114" s="2"/>
     </row>
     <row r="115" spans="1:14" x14ac:dyDescent="0.2">
@@ -21073,12 +20664,8 @@
       <c r="K115" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L115" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M115" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L115" s="2"/>
+      <c r="M115" s="2"/>
       <c r="N115" s="2"/>
     </row>
     <row r="116" spans="1:14" x14ac:dyDescent="0.2">
@@ -21152,9 +20739,7 @@
       <c r="G118" s="2" t="s">
         <v>823</v>
       </c>
-      <c r="H118" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="H118" s="2"/>
       <c r="I118" s="2" t="s">
         <v>650</v>
       </c>
@@ -21164,12 +20749,8 @@
       <c r="K118" s="2" t="s">
         <v>690</v>
       </c>
-      <c r="L118" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M118" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L118" s="2"/>
+      <c r="M118" s="2"/>
       <c r="N118" s="2"/>
     </row>
     <row r="119" spans="1:14" x14ac:dyDescent="0.2">
@@ -21202,12 +20783,8 @@
       <c r="K119" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="L119" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="M119" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="L119" s="2"/>
+      <c r="M119" s="2"/>
       <c r="N119" s="2"/>
     </row>
     <row r="120" spans="1:14" x14ac:dyDescent="0.2">
@@ -21258,9 +20835,7 @@
       </c>
       <c r="F121" s="2"/>
       <c r="G121" s="2"/>
-      <c r="H121" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="H121" s="2"/>
       <c r="I121" s="2" t="s">
         <v>650</v>
       </c>
@@ -25132,7 +24707,7 @@
         <v>701</v>
       </c>
       <c r="E144" s="2" t="s">
-        <v>143</v>
+        <v>816</v>
       </c>
       <c r="F144" s="2"/>
       <c r="G144" s="2"/>
@@ -25234,7 +24809,7 @@
         <v>702</v>
       </c>
       <c r="E149" s="2" t="s">
-        <v>143</v>
+        <v>816</v>
       </c>
       <c r="F149" s="2"/>
       <c r="G149" s="2"/>
@@ -25456,7 +25031,7 @@
         <v>703</v>
       </c>
       <c r="E160" s="2" t="s">
-        <v>143</v>
+        <v>816</v>
       </c>
       <c r="F160" s="2"/>
       <c r="G160" s="2"/>
@@ -25960,7 +25535,7 @@
         <v>705</v>
       </c>
       <c r="E185" s="2" t="s">
-        <v>143</v>
+        <v>816</v>
       </c>
       <c r="F185" s="2"/>
       <c r="G185" s="2"/>

</xml_diff>

<commit_message>
Split up NWSS to ODM config 'wide' tab into 'wide_qualityReports' and 'wide_measures'
</commit_message>
<xml_diff>
--- a/data/mapping_config_files/NWSS-to-ODM-dictionary.xlsx
+++ b/data/mapping_config_files/NWSS-to-ODM-dictionary.xlsx
@@ -8,26 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-MapGenerator/PHES-ODM-MapGenerator/data/mapping_config_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F954EFD8-4B08-3F45-A3DC-4037CFB16FDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{047DCD60-FE69-034B-BFC5-840057F0F7C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2020" yWindow="500" windowWidth="38940" windowHeight="20920" activeTab="3" xr2:uid="{77810E24-F86B-BC44-A0D5-8790E6EC60B4}"/>
+    <workbookView xWindow="7400" yWindow="500" windowWidth="38940" windowHeight="20920" activeTab="1" xr2:uid="{77810E24-F86B-BC44-A0D5-8790E6EC60B4}"/>
   </bookViews>
   <sheets>
     <sheet name="maps" sheetId="1" r:id="rId1"/>
-    <sheet name="wide" sheetId="2" r:id="rId2"/>
-    <sheet name="wide_qualityReports" sheetId="7" r:id="rId3"/>
-    <sheet name="enums" sheetId="3" r:id="rId4"/>
-    <sheet name="id_gen" sheetId="4" r:id="rId5"/>
-    <sheet name="maps original" sheetId="6" r:id="rId6"/>
+    <sheet name="wide_measures" sheetId="2" r:id="rId2"/>
+    <sheet name="wide_protocolSteps" sheetId="8" r:id="rId3"/>
+    <sheet name="wide_qualityReports" sheetId="7" r:id="rId4"/>
+    <sheet name="enums" sheetId="3" r:id="rId5"/>
+    <sheet name="id_gen" sheetId="4" r:id="rId6"/>
+    <sheet name="maps original" sheetId="6" r:id="rId7"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId7"/>
+    <externalReference r:id="rId8"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">enums!$A$1:$J$185</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">enums!$A$1:$J$185</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">maps!$A$1:$L$91</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'maps original'!$A$1:$L$87</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">wide!$A$1:$N$136</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'maps original'!$A$1:$L$87</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">wide_measures!$A$1:$N$24</definedName>
     <definedName name="partID">[1]parts!$A:$A</definedName>
     <definedName name="partLabel">[1]parts!$B:$B</definedName>
   </definedNames>
@@ -51,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2995" uniqueCount="837">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3009" uniqueCount="837">
   <si>
     <t>Reporter</t>
   </si>
@@ -16854,7 +16855,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B39AC7DD-3F73-2C47-925D-21E5B4EBE6FC}">
-  <dimension ref="A1:N136"/>
+  <dimension ref="A1:N24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="28.6640625" customWidth="1"/>
@@ -17173,16 +17174,972 @@
       <c r="N8" s="2"/>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
+      <c r="A9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>39</v>
+      </c>
       <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
+      <c r="E9" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>581</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>663</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>582</v>
+      </c>
+      <c r="M9" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="N9" s="2"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A10" t="b">
+        <v>1</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>665</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="M10" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="N10" s="2"/>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A11" t="b">
+        <v>1</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>666</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="M11" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="N11" s="2"/>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A12" t="b">
+        <v>1</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>667</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="M12" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="N12" s="2"/>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A13" t="b">
+        <v>1</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>668</v>
+      </c>
+      <c r="L13" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="M13" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="N13" s="2"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A14" t="b">
+        <v>1</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>669</v>
+      </c>
+      <c r="L14" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="M14" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="N14" s="2"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A15" t="b">
+        <v>1</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>670</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="M15" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="N15" s="2"/>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A16" t="b">
+        <v>1</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>824</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="I16" s="1" t="s">
+        <v>642</v>
+      </c>
+      <c r="J16" s="1" t="s">
+        <v>650</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>671</v>
+      </c>
+      <c r="L16" s="1" t="s">
+        <v>646</v>
+      </c>
+      <c r="M16" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="N16" s="2" t="s">
+        <v>721</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A17" t="b">
+        <v>1</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>825</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>642</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>650</v>
+      </c>
+      <c r="K17" s="2" t="s">
+        <v>672</v>
+      </c>
+      <c r="L17" s="1" t="s">
+        <v>646</v>
+      </c>
+      <c r="M17" s="2" t="s">
+        <v>592</v>
+      </c>
+      <c r="N17" s="1" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A18" t="b">
+        <v>1</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>825</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>642</v>
+      </c>
+      <c r="J18" s="1" t="s">
+        <v>650</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>673</v>
+      </c>
+      <c r="L18" s="1" t="s">
+        <v>646</v>
+      </c>
+      <c r="M18" s="2" t="s">
+        <v>594</v>
+      </c>
+      <c r="N18" s="1" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A19" t="b">
+        <v>1</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>825</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>642</v>
+      </c>
+      <c r="J19" s="1" t="s">
+        <v>650</v>
+      </c>
+      <c r="K19" s="2" t="s">
+        <v>674</v>
+      </c>
+      <c r="L19" s="1" t="s">
+        <v>646</v>
+      </c>
+      <c r="M19" s="2" t="s">
+        <v>595</v>
+      </c>
+      <c r="N19" s="1" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A20" t="b">
+        <v>1</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>826</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>599</v>
+      </c>
+      <c r="J20" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="K20" s="2" t="s">
+        <v>675</v>
+      </c>
+      <c r="L20" s="2" t="s">
+        <v>646</v>
+      </c>
+      <c r="M20" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="N20" s="1" t="s">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A21" t="b">
+        <v>1</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D21" s="2"/>
+      <c r="E21" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="G21" s="2"/>
+      <c r="H21" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>601</v>
+      </c>
+      <c r="J21" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="K21" s="2" t="s">
+        <v>676</v>
+      </c>
+      <c r="L21" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="M21" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="N21" s="1" t="s">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A22" t="b">
+        <v>1</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D22" s="2"/>
+      <c r="E22" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>827</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="I22" s="1" t="s">
+        <v>643</v>
+      </c>
+      <c r="J22" s="1" t="s">
+        <v>650</v>
+      </c>
+      <c r="K22" s="2" t="s">
+        <v>677</v>
+      </c>
+      <c r="L22" s="1" t="s">
+        <v>647</v>
+      </c>
+      <c r="M22" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="N22" s="2"/>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A23" t="b">
+        <v>1</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D23" s="2"/>
+      <c r="E23" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>828</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="I23" s="1" t="s">
+        <v>644</v>
+      </c>
+      <c r="J23" s="1" t="s">
+        <v>650</v>
+      </c>
+      <c r="K23" s="2" t="s">
+        <v>678</v>
+      </c>
+      <c r="L23" s="1" t="s">
+        <v>648</v>
+      </c>
+      <c r="M23" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="N23" s="2"/>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A24" t="b">
+        <v>1</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>829</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="I24" s="1" t="s">
+        <v>645</v>
+      </c>
+      <c r="J24" s="1" t="s">
+        <v>650</v>
+      </c>
+      <c r="K24" s="2" t="s">
+        <v>679</v>
+      </c>
+      <c r="L24" s="1" t="s">
+        <v>649</v>
+      </c>
+      <c r="M24" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="N24" s="2"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:N24" xr:uid="{B39AC7DD-3F73-2C47-925D-21E5B4EBE6FC}"/>
+  <conditionalFormatting sqref="L10 I10:J10 L15:L16">
+    <cfRule type="duplicateValues" dxfId="8" priority="8"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L22">
+    <cfRule type="duplicateValues" dxfId="7" priority="5"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L23">
+    <cfRule type="duplicateValues" dxfId="6" priority="4"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L24">
+    <cfRule type="duplicateValues" dxfId="5" priority="3"/>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDC6A21B-0669-0743-9D12-F41DCA15CA4A}">
+  <dimension ref="A1:N112"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="37.83203125" customWidth="1"/>
+    <col min="5" max="5" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="24.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="22.83203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="11" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="96.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" s="24" customFormat="1" ht="20" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="24" t="s">
+        <v>680</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>634</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>636</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>637</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>638</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>640</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>698</v>
+      </c>
+      <c r="H1" s="11" t="s">
+        <v>830</v>
+      </c>
+      <c r="I1" s="11" t="s">
+        <v>831</v>
+      </c>
+      <c r="J1" s="11" t="s">
+        <v>832</v>
+      </c>
+      <c r="K1" s="11" t="s">
+        <v>833</v>
+      </c>
+      <c r="L1" s="11" t="s">
+        <v>834</v>
+      </c>
+      <c r="M1" s="11" t="s">
+        <v>835</v>
+      </c>
+      <c r="N1" s="12" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A2" t="b">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>684</v>
+      </c>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A3" t="b">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="L3" s="2"/>
+      <c r="M3" s="2"/>
+      <c r="N3" s="2"/>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A4" t="b">
+        <v>1</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>425</v>
+      </c>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="L4" s="2"/>
+      <c r="M4" s="2"/>
+      <c r="N4" s="2"/>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A5" t="b">
+        <v>1</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="L5" s="2"/>
+      <c r="M5" s="2"/>
+      <c r="N5" s="2"/>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A6" t="b">
+        <v>1</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>816</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="L6" s="2"/>
+      <c r="M6" s="2"/>
+      <c r="N6" s="2"/>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
+      <c r="N7" s="2"/>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A8" t="b">
+        <v>1</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>429</v>
+      </c>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>685</v>
+      </c>
+      <c r="L8" s="2"/>
+      <c r="M8" s="2"/>
+      <c r="N8" s="2"/>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A9" t="b">
+        <v>1</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>428</v>
+      </c>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
+      <c r="I9" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>650</v>
+      </c>
       <c r="L9" s="2"/>
       <c r="M9" s="2"/>
       <c r="N9" s="2"/>
@@ -17195,16 +18152,16 @@
         <v>635</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>423</v>
+        <v>430</v>
       </c>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
@@ -17212,10 +18169,10 @@
         <v>650</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>422</v>
+        <v>650</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>684</v>
+        <v>650</v>
       </c>
       <c r="L10" s="2"/>
       <c r="M10" s="2"/>
@@ -17229,16 +18186,16 @@
         <v>635</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F11" s="2" t="s">
-        <v>424</v>
+        <v>431</v>
       </c>
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
@@ -17263,16 +18220,16 @@
         <v>635</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>181</v>
+        <v>29</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>187</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>425</v>
+        <v>432</v>
       </c>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
@@ -17282,9 +18239,7 @@
       <c r="J12" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="K12" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="K12" s="2"/>
       <c r="L12" s="2"/>
       <c r="M12" s="2"/>
       <c r="N12" s="2"/>
@@ -17297,16 +18252,16 @@
         <v>635</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>426</v>
+        <v>433</v>
       </c>
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
@@ -17331,15 +18286,17 @@
         <v>635</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>816</v>
+        <v>189</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="F14" s="2"/>
+      <c r="F14" s="2" t="s">
+        <v>432</v>
+      </c>
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
       <c r="I14" s="2" t="s">
@@ -17356,16 +18313,35 @@
       <c r="N14" s="2"/>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
+      <c r="A15" t="b">
+        <v>1</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>434</v>
+      </c>
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
-      <c r="J15" s="2"/>
-      <c r="K15" s="2"/>
+      <c r="I15" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>650</v>
+      </c>
       <c r="L15" s="2"/>
       <c r="M15" s="2"/>
       <c r="N15" s="2"/>
@@ -17380,14 +18356,14 @@
       <c r="C16" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D16" s="4" t="s">
-        <v>183</v>
+      <c r="D16" s="3" t="s">
+        <v>191</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>429</v>
+        <v>435</v>
       </c>
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
@@ -17395,10 +18371,10 @@
         <v>650</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>427</v>
+        <v>650</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>685</v>
+        <v>650</v>
       </c>
       <c r="L16" s="2"/>
       <c r="M16" s="2"/>
@@ -17415,13 +18391,13 @@
         <v>29</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>428</v>
+        <v>436</v>
       </c>
       <c r="G17" s="2"/>
       <c r="H17" s="2"/>
@@ -17449,13 +18425,13 @@
         <v>29</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>430</v>
+        <v>438</v>
       </c>
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
@@ -17483,13 +18459,13 @@
         <v>29</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F19" s="2" t="s">
-        <v>431</v>
+        <v>437</v>
       </c>
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
@@ -17516,14 +18492,14 @@
       <c r="C20" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D20" s="4" t="s">
-        <v>187</v>
+      <c r="D20" s="3" t="s">
+        <v>195</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>432</v>
+        <v>439</v>
       </c>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
@@ -17533,7 +18509,9 @@
       <c r="J20" s="2" t="s">
         <v>650</v>
       </c>
-      <c r="K20" s="2"/>
+      <c r="K20" s="2" t="s">
+        <v>650</v>
+      </c>
       <c r="L20" s="2"/>
       <c r="M20" s="2"/>
       <c r="N20" s="2"/>
@@ -17549,13 +18527,13 @@
         <v>29</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>433</v>
+        <v>615</v>
       </c>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
@@ -17572,7 +18550,7 @@
       <c r="M21" s="2"/>
       <c r="N21" s="2"/>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" t="b">
         <v>1</v>
       </c>
@@ -17583,13 +18561,13 @@
         <v>29</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>432</v>
+        <v>440</v>
       </c>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
@@ -17617,13 +18595,13 @@
         <v>29</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>434</v>
+        <v>441</v>
       </c>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
@@ -17651,13 +18629,13 @@
         <v>29</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>435</v>
+        <v>442</v>
       </c>
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
@@ -17684,14 +18662,14 @@
       <c r="C25" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="D25" s="3" t="s">
-        <v>192</v>
+      <c r="D25" s="2" t="s">
+        <v>200</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F25" s="2" t="s">
-        <v>436</v>
+        <v>443</v>
       </c>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
@@ -17719,13 +18697,13 @@
         <v>29</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>438</v>
+        <v>445</v>
       </c>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
@@ -17753,13 +18731,13 @@
         <v>29</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>437</v>
+        <v>444</v>
       </c>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
@@ -17787,13 +18765,13 @@
         <v>29</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>439</v>
+        <v>616</v>
       </c>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
@@ -17821,13 +18799,13 @@
         <v>29</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F29" s="2" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
@@ -17844,7 +18822,7 @@
       <c r="M29" s="2"/>
       <c r="N29" s="2"/>
     </row>
-    <row r="30" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A30" t="b">
         <v>1</v>
       </c>
@@ -17855,13 +18833,13 @@
         <v>29</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F30" s="2" t="s">
-        <v>440</v>
+        <v>618</v>
       </c>
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
@@ -17889,13 +18867,13 @@
         <v>29</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>198</v>
+        <v>182</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>441</v>
+        <v>426</v>
       </c>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
@@ -17913,35 +18891,16 @@
       <c r="N31" s="2"/>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A32" t="b">
-        <v>1</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D32" s="3" t="s">
-        <v>199</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="F32" s="2" t="s">
-        <v>442</v>
-      </c>
+      <c r="B32" s="2"/>
+      <c r="C32" s="2"/>
+      <c r="D32" s="3"/>
+      <c r="E32" s="2"/>
+      <c r="F32" s="2"/>
       <c r="G32" s="2"/>
       <c r="H32" s="2"/>
-      <c r="I32" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="J32" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="K32" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="I32" s="2"/>
+      <c r="J32" s="2"/>
+      <c r="K32" s="2"/>
       <c r="L32" s="2"/>
       <c r="M32" s="2"/>
       <c r="N32" s="2"/>
@@ -17954,16 +18913,16 @@
         <v>635</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>200</v>
+        <v>30</v>
+      </c>
+      <c r="D33" s="14" t="s">
+        <v>221</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F33" s="2" t="s">
-        <v>443</v>
+        <v>447</v>
       </c>
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
@@ -17971,10 +18930,10 @@
         <v>650</v>
       </c>
       <c r="J33" s="2" t="s">
-        <v>650</v>
+        <v>446</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>650</v>
+        <v>686</v>
       </c>
       <c r="L33" s="2"/>
       <c r="M33" s="2"/>
@@ -17988,16 +18947,16 @@
         <v>635</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>201</v>
+        <v>219</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
@@ -18022,16 +18981,16 @@
         <v>635</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>202</v>
+        <v>233</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F35" s="2" t="s">
-        <v>444</v>
+        <v>619</v>
       </c>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
@@ -18056,16 +19015,16 @@
         <v>635</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>203</v>
+        <v>225</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>616</v>
+        <v>620</v>
       </c>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
@@ -18090,16 +19049,16 @@
         <v>635</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D37" s="3" t="s">
-        <v>204</v>
+        <v>30</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>232</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>617</v>
+        <v>621</v>
       </c>
       <c r="G37" s="2"/>
       <c r="H37" s="2"/>
@@ -18124,16 +19083,16 @@
         <v>635</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="D38" s="3" t="s">
-        <v>205</v>
+        <v>30</v>
+      </c>
+      <c r="D38" s="15" t="s">
+        <v>236</v>
       </c>
       <c r="E38" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>618</v>
+        <v>622</v>
       </c>
       <c r="G38" s="2"/>
       <c r="H38" s="2"/>
@@ -18158,16 +19117,16 @@
         <v>635</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>182</v>
+        <v>216</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>426</v>
+        <v>449</v>
       </c>
       <c r="G39" s="2"/>
       <c r="H39" s="2"/>
@@ -18185,16 +19144,35 @@
       <c r="N39" s="2"/>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B40" s="2"/>
-      <c r="C40" s="2"/>
-      <c r="D40" s="3"/>
-      <c r="E40" s="2"/>
-      <c r="F40" s="2"/>
+      <c r="A40" t="b">
+        <v>1</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>450</v>
+      </c>
       <c r="G40" s="2"/>
       <c r="H40" s="2"/>
-      <c r="I40" s="2"/>
-      <c r="J40" s="2"/>
-      <c r="K40" s="2"/>
+      <c r="I40" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="J40" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="K40" s="2" t="s">
+        <v>650</v>
+      </c>
       <c r="L40" s="2"/>
       <c r="M40" s="2"/>
       <c r="N40" s="2"/>
@@ -18209,14 +19187,14 @@
       <c r="C41" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D41" s="14" t="s">
-        <v>221</v>
+      <c r="D41" s="3" t="s">
+        <v>218</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F41" s="2" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="G41" s="2"/>
       <c r="H41" s="2"/>
@@ -18224,10 +19202,10 @@
         <v>650</v>
       </c>
       <c r="J41" s="2" t="s">
-        <v>446</v>
+        <v>650</v>
       </c>
       <c r="K41" s="2" t="s">
-        <v>686</v>
+        <v>650</v>
       </c>
       <c r="L41" s="2"/>
       <c r="M41" s="2"/>
@@ -18244,13 +19222,13 @@
         <v>30</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="E42" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F42" s="2" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="G42" s="2"/>
       <c r="H42" s="2"/>
@@ -18278,13 +19256,13 @@
         <v>30</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>233</v>
+        <v>213</v>
       </c>
       <c r="E43" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F43" s="2" t="s">
-        <v>619</v>
+        <v>453</v>
       </c>
       <c r="G43" s="2"/>
       <c r="H43" s="2"/>
@@ -18312,13 +19290,13 @@
         <v>30</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>225</v>
+        <v>215</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>620</v>
+        <v>454</v>
       </c>
       <c r="G44" s="2"/>
       <c r="H44" s="2"/>
@@ -18345,14 +19323,14 @@
       <c r="C45" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D45" s="2" t="s">
-        <v>232</v>
+      <c r="D45" s="3" t="s">
+        <v>196</v>
       </c>
       <c r="E45" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F45" s="2" t="s">
-        <v>621</v>
+        <v>455</v>
       </c>
       <c r="G45" s="2"/>
       <c r="H45" s="2"/>
@@ -18379,14 +19357,14 @@
       <c r="C46" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D46" s="15" t="s">
-        <v>236</v>
+      <c r="D46" s="3" t="s">
+        <v>226</v>
       </c>
       <c r="E46" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F46" s="2" t="s">
-        <v>622</v>
+        <v>456</v>
       </c>
       <c r="G46" s="2"/>
       <c r="H46" s="2"/>
@@ -18414,13 +19392,13 @@
         <v>30</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="E47" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F47" s="2" t="s">
-        <v>449</v>
+        <v>623</v>
       </c>
       <c r="G47" s="2"/>
       <c r="H47" s="2"/>
@@ -18448,13 +19426,13 @@
         <v>30</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>217</v>
+        <v>207</v>
       </c>
       <c r="E48" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F48" s="2" t="s">
-        <v>450</v>
+        <v>458</v>
       </c>
       <c r="G48" s="2"/>
       <c r="H48" s="2"/>
@@ -18481,14 +19459,14 @@
       <c r="C49" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D49" s="3" t="s">
-        <v>218</v>
+      <c r="D49" s="4" t="s">
+        <v>206</v>
       </c>
       <c r="E49" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F49" s="2" t="s">
-        <v>451</v>
+        <v>459</v>
       </c>
       <c r="G49" s="2"/>
       <c r="H49" s="2"/>
@@ -18516,13 +19494,13 @@
         <v>30</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="E50" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F50" s="2" t="s">
-        <v>452</v>
+        <v>457</v>
       </c>
       <c r="G50" s="2"/>
       <c r="H50" s="2"/>
@@ -18550,13 +19528,13 @@
         <v>30</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="E51" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F51" s="2" t="s">
-        <v>453</v>
+        <v>460</v>
       </c>
       <c r="G51" s="2"/>
       <c r="H51" s="2"/>
@@ -18584,13 +19562,13 @@
         <v>30</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="E52" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F52" s="2" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="G52" s="2"/>
       <c r="H52" s="2"/>
@@ -18618,13 +19596,13 @@
         <v>30</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>196</v>
+        <v>231</v>
       </c>
       <c r="E53" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F53" s="2" t="s">
-        <v>455</v>
+        <v>624</v>
       </c>
       <c r="G53" s="2"/>
       <c r="H53" s="2"/>
@@ -18652,13 +19630,13 @@
         <v>30</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>226</v>
+        <v>211</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F54" s="2" t="s">
-        <v>456</v>
+        <v>462</v>
       </c>
       <c r="G54" s="2"/>
       <c r="H54" s="2"/>
@@ -18686,13 +19664,13 @@
         <v>30</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="E55" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F55" s="2" t="s">
-        <v>623</v>
+        <v>463</v>
       </c>
       <c r="G55" s="2"/>
       <c r="H55" s="2"/>
@@ -18720,13 +19698,13 @@
         <v>30</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>207</v>
+        <v>234</v>
       </c>
       <c r="E56" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F56" s="2" t="s">
-        <v>458</v>
+        <v>625</v>
       </c>
       <c r="G56" s="2"/>
       <c r="H56" s="2"/>
@@ -18753,14 +19731,14 @@
       <c r="C57" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D57" s="4" t="s">
-        <v>206</v>
+      <c r="D57" s="2" t="s">
+        <v>224</v>
       </c>
       <c r="E57" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F57" s="2" t="s">
-        <v>459</v>
+        <v>464</v>
       </c>
       <c r="G57" s="2"/>
       <c r="H57" s="2"/>
@@ -18788,13 +19766,13 @@
         <v>30</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>212</v>
+        <v>235</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F58" s="2" t="s">
-        <v>457</v>
+        <v>626</v>
       </c>
       <c r="G58" s="2"/>
       <c r="H58" s="2"/>
@@ -18821,14 +19799,14 @@
       <c r="C59" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D59" s="3" t="s">
-        <v>210</v>
+      <c r="D59" s="15" t="s">
+        <v>227</v>
       </c>
       <c r="E59" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F59" s="2" t="s">
-        <v>460</v>
+        <v>627</v>
       </c>
       <c r="G59" s="2"/>
       <c r="H59" s="2"/>
@@ -18855,14 +19833,14 @@
       <c r="C60" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D60" s="3" t="s">
-        <v>222</v>
+      <c r="D60" s="15" t="s">
+        <v>228</v>
       </c>
       <c r="E60" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F60" s="2" t="s">
-        <v>461</v>
+        <v>628</v>
       </c>
       <c r="G60" s="2"/>
       <c r="H60" s="2"/>
@@ -18890,13 +19868,13 @@
         <v>30</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>231</v>
+        <v>220</v>
       </c>
       <c r="E61" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F61" s="2" t="s">
-        <v>624</v>
+        <v>465</v>
       </c>
       <c r="G61" s="2"/>
       <c r="H61" s="2"/>
@@ -18924,13 +19902,13 @@
         <v>30</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="E62" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F62" s="2" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
       <c r="G62" s="2"/>
       <c r="H62" s="2"/>
@@ -18958,13 +19936,13 @@
         <v>30</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>209</v>
+        <v>223</v>
       </c>
       <c r="E63" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F63" s="2" t="s">
-        <v>463</v>
+        <v>467</v>
       </c>
       <c r="G63" s="2"/>
       <c r="H63" s="2"/>
@@ -18991,14 +19969,14 @@
       <c r="C64" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D64" s="3" t="s">
-        <v>234</v>
+      <c r="D64" s="16" t="s">
+        <v>229</v>
       </c>
       <c r="E64" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F64" s="2" t="s">
-        <v>625</v>
+        <v>629</v>
       </c>
       <c r="G64" s="2"/>
       <c r="H64" s="2"/>
@@ -19025,14 +20003,14 @@
       <c r="C65" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D65" s="2" t="s">
-        <v>224</v>
+      <c r="D65" s="16" t="s">
+        <v>230</v>
       </c>
       <c r="E65" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F65" s="2" t="s">
-        <v>464</v>
+        <v>630</v>
       </c>
       <c r="G65" s="2"/>
       <c r="H65" s="2"/>
@@ -19050,35 +20028,16 @@
       <c r="N65" s="2"/>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A66" t="b">
-        <v>1</v>
-      </c>
-      <c r="B66" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="C66" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D66" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="E66" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="F66" s="2" t="s">
-        <v>626</v>
-      </c>
+      <c r="B66" s="2"/>
+      <c r="C66" s="2"/>
+      <c r="D66" s="16"/>
+      <c r="E66" s="2"/>
+      <c r="F66" s="2"/>
       <c r="G66" s="2"/>
       <c r="H66" s="2"/>
-      <c r="I66" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="J66" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="K66" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="I66" s="2"/>
+      <c r="J66" s="2"/>
+      <c r="K66" s="2"/>
       <c r="L66" s="2"/>
       <c r="M66" s="2"/>
       <c r="N66" s="2"/>
@@ -19091,30 +20050,34 @@
         <v>635</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D67" s="15" t="s">
-        <v>227</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="D67" s="2"/>
       <c r="E67" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F67" s="2" t="s">
-        <v>627</v>
+        <v>650</v>
       </c>
       <c r="G67" s="2"/>
-      <c r="H67" s="2"/>
+      <c r="H67" s="2" t="s">
+        <v>165</v>
+      </c>
       <c r="I67" s="2" t="s">
-        <v>650</v>
+        <v>479</v>
       </c>
       <c r="J67" s="2" t="s">
         <v>650</v>
       </c>
       <c r="K67" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="L67" s="2"/>
-      <c r="M67" s="2"/>
+        <v>657</v>
+      </c>
+      <c r="L67" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="M67" s="2" t="s">
+        <v>155</v>
+      </c>
       <c r="N67" s="2"/>
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.2">
@@ -19125,30 +20088,34 @@
         <v>635</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D68" s="15" t="s">
-        <v>228</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="D68" s="2"/>
       <c r="E68" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F68" s="2" t="s">
-        <v>628</v>
+        <v>650</v>
       </c>
       <c r="G68" s="2"/>
-      <c r="H68" s="2"/>
+      <c r="H68" s="2" t="s">
+        <v>165</v>
+      </c>
       <c r="I68" s="2" t="s">
-        <v>650</v>
+        <v>480</v>
       </c>
       <c r="J68" s="2" t="s">
         <v>650</v>
       </c>
       <c r="K68" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="L68" s="2"/>
-      <c r="M68" s="2"/>
+        <v>658</v>
+      </c>
+      <c r="L68" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="M68" s="2" t="s">
+        <v>155</v>
+      </c>
       <c r="N68" s="2"/>
     </row>
     <row r="69" spans="1:14" x14ac:dyDescent="0.2">
@@ -19159,30 +20126,34 @@
         <v>635</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D69" s="3" t="s">
-        <v>220</v>
-      </c>
+        <v>33</v>
+      </c>
+      <c r="D69" s="2"/>
       <c r="E69" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F69" s="2" t="s">
-        <v>465</v>
+        <v>650</v>
       </c>
       <c r="G69" s="2"/>
-      <c r="H69" s="2"/>
+      <c r="H69" s="2" t="s">
+        <v>165</v>
+      </c>
       <c r="I69" s="2" t="s">
-        <v>650</v>
+        <v>481</v>
       </c>
       <c r="J69" s="2" t="s">
         <v>650</v>
       </c>
       <c r="K69" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="L69" s="2"/>
-      <c r="M69" s="2"/>
+        <v>659</v>
+      </c>
+      <c r="L69" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="M69" s="2" t="s">
+        <v>155</v>
+      </c>
       <c r="N69" s="2"/>
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.2">
@@ -19193,30 +20164,34 @@
         <v>635</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D70" s="3" t="s">
-        <v>203</v>
-      </c>
+        <v>34</v>
+      </c>
+      <c r="D70" s="2"/>
       <c r="E70" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F70" s="2" t="s">
-        <v>466</v>
+        <v>650</v>
       </c>
       <c r="G70" s="2"/>
-      <c r="H70" s="2"/>
+      <c r="H70" s="2" t="s">
+        <v>165</v>
+      </c>
       <c r="I70" s="2" t="s">
-        <v>650</v>
+        <v>482</v>
       </c>
       <c r="J70" s="2" t="s">
         <v>650</v>
       </c>
       <c r="K70" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="L70" s="2"/>
-      <c r="M70" s="2"/>
+        <v>660</v>
+      </c>
+      <c r="L70" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="M70" s="2" t="s">
+        <v>155</v>
+      </c>
       <c r="N70" s="2"/>
     </row>
     <row r="71" spans="1:14" x14ac:dyDescent="0.2">
@@ -19227,16 +20202,14 @@
         <v>635</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D71" s="3" t="s">
-        <v>223</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="D71" s="2"/>
       <c r="E71" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F71" s="2" t="s">
-        <v>467</v>
+        <v>650</v>
       </c>
       <c r="G71" s="2"/>
       <c r="H71" s="2"/>
@@ -19244,13 +20217,17 @@
         <v>650</v>
       </c>
       <c r="J71" s="2" t="s">
-        <v>650</v>
+        <v>483</v>
       </c>
       <c r="K71" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="L71" s="2"/>
-      <c r="M71" s="2"/>
+        <v>661</v>
+      </c>
+      <c r="L71" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="M71" s="2" t="s">
+        <v>155</v>
+      </c>
       <c r="N71" s="2"/>
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.2">
@@ -19261,16 +20238,14 @@
         <v>635</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D72" s="16" t="s">
-        <v>229</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="D72" s="2"/>
       <c r="E72" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F72" s="2" t="s">
-        <v>629</v>
+        <v>650</v>
       </c>
       <c r="G72" s="2"/>
       <c r="H72" s="2"/>
@@ -19278,60 +20253,58 @@
         <v>650</v>
       </c>
       <c r="J72" s="2" t="s">
-        <v>650</v>
+        <v>484</v>
       </c>
       <c r="K72" s="2" t="s">
-        <v>650</v>
+        <v>662</v>
       </c>
       <c r="L72" s="2"/>
       <c r="M72" s="2"/>
       <c r="N72" s="2"/>
     </row>
     <row r="73" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A73" t="b">
-        <v>1</v>
-      </c>
-      <c r="B73" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="C73" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D73" s="16" t="s">
-        <v>230</v>
-      </c>
-      <c r="E73" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="F73" s="2" t="s">
-        <v>630</v>
-      </c>
+      <c r="B73" s="2"/>
+      <c r="C73" s="2"/>
+      <c r="D73" s="2"/>
+      <c r="E73" s="2"/>
+      <c r="F73" s="2"/>
       <c r="G73" s="2"/>
       <c r="H73" s="2"/>
-      <c r="I73" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="J73" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="K73" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="I73" s="2"/>
+      <c r="J73" s="2"/>
+      <c r="K73" s="2"/>
       <c r="L73" s="2"/>
       <c r="M73" s="2"/>
       <c r="N73" s="2"/>
     </row>
     <row r="74" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B74" s="2"/>
-      <c r="C74" s="2"/>
-      <c r="D74" s="16"/>
-      <c r="E74" s="2"/>
+      <c r="A74" t="b">
+        <v>1</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="C74" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D74" s="3" t="s">
+        <v>816</v>
+      </c>
+      <c r="E74" s="2" t="s">
+        <v>152</v>
+      </c>
       <c r="F74" s="2"/>
       <c r="G74" s="2"/>
       <c r="H74" s="2"/>
-      <c r="I74" s="2"/>
-      <c r="J74" s="2"/>
-      <c r="K74" s="2"/>
+      <c r="I74" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="J74" s="2" t="s">
+        <v>485</v>
+      </c>
+      <c r="K74" s="2" t="s">
+        <v>687</v>
+      </c>
       <c r="L74" s="2"/>
       <c r="M74" s="2"/>
       <c r="N74" s="2"/>
@@ -19344,34 +20317,30 @@
         <v>635</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="D75" s="2"/>
+        <v>37</v>
+      </c>
+      <c r="D75" s="3" t="s">
+        <v>250</v>
+      </c>
       <c r="E75" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F75" s="2" t="s">
-        <v>650</v>
+        <v>631</v>
       </c>
       <c r="G75" s="2"/>
-      <c r="H75" s="2" t="s">
-        <v>165</v>
-      </c>
+      <c r="H75" s="2"/>
       <c r="I75" s="2" t="s">
-        <v>479</v>
+        <v>650</v>
       </c>
       <c r="J75" s="2" t="s">
         <v>650</v>
       </c>
       <c r="K75" s="2" t="s">
-        <v>657</v>
-      </c>
-      <c r="L75" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="M75" s="2" t="s">
-        <v>155</v>
-      </c>
+        <v>650</v>
+      </c>
+      <c r="L75" s="2"/>
+      <c r="M75" s="2"/>
       <c r="N75" s="2"/>
     </row>
     <row r="76" spans="1:14" x14ac:dyDescent="0.2">
@@ -19382,34 +20351,30 @@
         <v>635</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="D76" s="2"/>
+        <v>37</v>
+      </c>
+      <c r="D76" s="3" t="s">
+        <v>238</v>
+      </c>
       <c r="E76" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F76" s="2" t="s">
-        <v>650</v>
+        <v>487</v>
       </c>
       <c r="G76" s="2"/>
-      <c r="H76" s="2" t="s">
-        <v>165</v>
-      </c>
+      <c r="H76" s="2"/>
       <c r="I76" s="2" t="s">
-        <v>480</v>
+        <v>650</v>
       </c>
       <c r="J76" s="2" t="s">
         <v>650</v>
       </c>
       <c r="K76" s="2" t="s">
-        <v>658</v>
-      </c>
-      <c r="L76" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="M76" s="2" t="s">
-        <v>155</v>
-      </c>
+        <v>650</v>
+      </c>
+      <c r="L76" s="2"/>
+      <c r="M76" s="2"/>
       <c r="N76" s="2"/>
     </row>
     <row r="77" spans="1:14" x14ac:dyDescent="0.2">
@@ -19420,34 +20385,30 @@
         <v>635</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D77" s="2"/>
+        <v>37</v>
+      </c>
+      <c r="D77" s="3" t="s">
+        <v>237</v>
+      </c>
       <c r="E77" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F77" s="2" t="s">
-        <v>650</v>
+        <v>488</v>
       </c>
       <c r="G77" s="2"/>
-      <c r="H77" s="2" t="s">
-        <v>165</v>
-      </c>
+      <c r="H77" s="2"/>
       <c r="I77" s="2" t="s">
-        <v>481</v>
+        <v>650</v>
       </c>
       <c r="J77" s="2" t="s">
         <v>650</v>
       </c>
       <c r="K77" s="2" t="s">
-        <v>659</v>
-      </c>
-      <c r="L77" s="2" t="s">
-        <v>158</v>
-      </c>
-      <c r="M77" s="2" t="s">
-        <v>155</v>
-      </c>
+        <v>650</v>
+      </c>
+      <c r="L77" s="2"/>
+      <c r="M77" s="2"/>
       <c r="N77" s="2"/>
     </row>
     <row r="78" spans="1:14" x14ac:dyDescent="0.2">
@@ -19458,34 +20419,30 @@
         <v>635</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="D78" s="2"/>
+        <v>37</v>
+      </c>
+      <c r="D78" s="3" t="s">
+        <v>240</v>
+      </c>
       <c r="E78" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F78" s="2" t="s">
-        <v>650</v>
+        <v>489</v>
       </c>
       <c r="G78" s="2"/>
-      <c r="H78" s="2" t="s">
-        <v>165</v>
-      </c>
+      <c r="H78" s="2"/>
       <c r="I78" s="2" t="s">
-        <v>482</v>
+        <v>650</v>
       </c>
       <c r="J78" s="2" t="s">
         <v>650</v>
       </c>
       <c r="K78" s="2" t="s">
-        <v>660</v>
-      </c>
-      <c r="L78" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="M78" s="2" t="s">
-        <v>155</v>
-      </c>
+        <v>650</v>
+      </c>
+      <c r="L78" s="2"/>
+      <c r="M78" s="2"/>
       <c r="N78" s="2"/>
     </row>
     <row r="79" spans="1:14" x14ac:dyDescent="0.2">
@@ -19496,14 +20453,16 @@
         <v>635</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="D79" s="2"/>
+        <v>37</v>
+      </c>
+      <c r="D79" s="3" t="s">
+        <v>239</v>
+      </c>
       <c r="E79" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F79" s="2" t="s">
-        <v>650</v>
+        <v>490</v>
       </c>
       <c r="G79" s="2"/>
       <c r="H79" s="2"/>
@@ -19511,17 +20470,13 @@
         <v>650</v>
       </c>
       <c r="J79" s="2" t="s">
-        <v>483</v>
+        <v>650</v>
       </c>
       <c r="K79" s="2" t="s">
-        <v>661</v>
-      </c>
-      <c r="L79" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="M79" s="2" t="s">
-        <v>155</v>
-      </c>
+        <v>650</v>
+      </c>
+      <c r="L79" s="2"/>
+      <c r="M79" s="2"/>
       <c r="N79" s="2"/>
     </row>
     <row r="80" spans="1:14" x14ac:dyDescent="0.2">
@@ -19532,14 +20487,16 @@
         <v>635</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D80" s="2"/>
+        <v>37</v>
+      </c>
+      <c r="D80" s="3" t="s">
+        <v>247</v>
+      </c>
       <c r="E80" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F80" s="2" t="s">
-        <v>650</v>
+        <v>491</v>
       </c>
       <c r="G80" s="2"/>
       <c r="H80" s="2"/>
@@ -19547,26 +20504,45 @@
         <v>650</v>
       </c>
       <c r="J80" s="2" t="s">
-        <v>484</v>
+        <v>650</v>
       </c>
       <c r="K80" s="2" t="s">
-        <v>662</v>
+        <v>650</v>
       </c>
       <c r="L80" s="2"/>
       <c r="M80" s="2"/>
       <c r="N80" s="2"/>
     </row>
     <row r="81" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B81" s="2"/>
-      <c r="C81" s="2"/>
-      <c r="D81" s="2"/>
-      <c r="E81" s="2"/>
-      <c r="F81" s="2"/>
+      <c r="A81" t="b">
+        <v>1</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="C81" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D81" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="E81" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F81" s="2" t="s">
+        <v>492</v>
+      </c>
       <c r="G81" s="2"/>
       <c r="H81" s="2"/>
-      <c r="I81" s="2"/>
-      <c r="J81" s="2"/>
-      <c r="K81" s="2"/>
+      <c r="I81" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="J81" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="K81" s="2" t="s">
+        <v>650</v>
+      </c>
       <c r="L81" s="2"/>
       <c r="M81" s="2"/>
       <c r="N81" s="2"/>
@@ -19582,22 +20558,24 @@
         <v>37</v>
       </c>
       <c r="D82" s="3" t="s">
-        <v>816</v>
+        <v>249</v>
       </c>
       <c r="E82" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="F82" s="2"/>
+      <c r="F82" s="2" t="s">
+        <v>493</v>
+      </c>
       <c r="G82" s="2"/>
       <c r="H82" s="2"/>
       <c r="I82" s="2" t="s">
         <v>650</v>
       </c>
       <c r="J82" s="2" t="s">
-        <v>485</v>
+        <v>650</v>
       </c>
       <c r="K82" s="2" t="s">
-        <v>687</v>
+        <v>650</v>
       </c>
       <c r="L82" s="2"/>
       <c r="M82" s="2"/>
@@ -19614,13 +20592,13 @@
         <v>37</v>
       </c>
       <c r="D83" s="3" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="E83" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F83" s="2" t="s">
-        <v>631</v>
+        <v>494</v>
       </c>
       <c r="G83" s="2"/>
       <c r="H83" s="2"/>
@@ -19648,13 +20626,13 @@
         <v>37</v>
       </c>
       <c r="D84" s="3" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="E84" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F84" s="2" t="s">
-        <v>487</v>
+        <v>495</v>
       </c>
       <c r="G84" s="2"/>
       <c r="H84" s="2"/>
@@ -19682,13 +20660,13 @@
         <v>37</v>
       </c>
       <c r="D85" s="3" t="s">
-        <v>237</v>
+        <v>248</v>
       </c>
       <c r="E85" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F85" s="2" t="s">
-        <v>488</v>
+        <v>632</v>
       </c>
       <c r="G85" s="2"/>
       <c r="H85" s="2"/>
@@ -19716,13 +20694,13 @@
         <v>37</v>
       </c>
       <c r="D86" s="3" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="E86" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F86" s="2" t="s">
-        <v>489</v>
+        <v>495</v>
       </c>
       <c r="G86" s="2"/>
       <c r="H86" s="2"/>
@@ -19750,13 +20728,13 @@
         <v>37</v>
       </c>
       <c r="D87" s="3" t="s">
-        <v>239</v>
+        <v>251</v>
       </c>
       <c r="E87" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F87" s="2" t="s">
-        <v>490</v>
+        <v>633</v>
       </c>
       <c r="G87" s="2"/>
       <c r="H87" s="2"/>
@@ -19784,13 +20762,13 @@
         <v>37</v>
       </c>
       <c r="D88" s="3" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="E88" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F88" s="2" t="s">
-        <v>491</v>
+        <v>496</v>
       </c>
       <c r="G88" s="2"/>
       <c r="H88" s="2"/>
@@ -19818,13 +20796,13 @@
         <v>37</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="E89" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F89" s="2" t="s">
-        <v>492</v>
+        <v>497</v>
       </c>
       <c r="G89" s="2"/>
       <c r="H89" s="2"/>
@@ -19842,35 +20820,16 @@
       <c r="N89" s="2"/>
     </row>
     <row r="90" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A90" t="b">
-        <v>1</v>
-      </c>
-      <c r="B90" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="C90" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D90" s="3" t="s">
-        <v>249</v>
-      </c>
-      <c r="E90" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="F90" s="2" t="s">
-        <v>493</v>
-      </c>
+      <c r="B90" s="2"/>
+      <c r="C90" s="2"/>
+      <c r="D90" s="3"/>
+      <c r="E90" s="2"/>
+      <c r="F90" s="2"/>
       <c r="G90" s="2"/>
       <c r="H90" s="2"/>
-      <c r="I90" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="J90" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="K90" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="I90" s="2"/>
+      <c r="J90" s="2"/>
+      <c r="K90" s="2"/>
       <c r="L90" s="2"/>
       <c r="M90" s="2"/>
       <c r="N90" s="2"/>
@@ -19883,27 +20842,25 @@
         <v>635</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D91" s="3" t="s">
-        <v>245</v>
+        <v>816</v>
       </c>
       <c r="E91" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="F91" s="2" t="s">
-        <v>494</v>
-      </c>
+      <c r="F91" s="2"/>
       <c r="G91" s="2"/>
       <c r="H91" s="2"/>
       <c r="I91" s="2" t="s">
         <v>650</v>
       </c>
       <c r="J91" s="2" t="s">
-        <v>650</v>
+        <v>486</v>
       </c>
       <c r="K91" s="2" t="s">
-        <v>650</v>
+        <v>688</v>
       </c>
       <c r="L91" s="2"/>
       <c r="M91" s="2"/>
@@ -19917,16 +20874,16 @@
         <v>635</v>
       </c>
       <c r="C92" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D92" s="3" t="s">
-        <v>241</v>
+        <v>254</v>
       </c>
       <c r="E92" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F92" s="2" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="G92" s="2"/>
       <c r="H92" s="2"/>
@@ -19951,16 +20908,16 @@
         <v>635</v>
       </c>
       <c r="C93" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D93" s="3" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
       <c r="E93" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F93" s="2" t="s">
-        <v>632</v>
+        <v>500</v>
       </c>
       <c r="G93" s="2"/>
       <c r="H93" s="2"/>
@@ -19985,16 +20942,16 @@
         <v>635</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D94" s="3" t="s">
-        <v>242</v>
+        <v>256</v>
       </c>
       <c r="E94" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F94" s="2" t="s">
-        <v>495</v>
+        <v>501</v>
       </c>
       <c r="G94" s="2"/>
       <c r="H94" s="2"/>
@@ -20019,16 +20976,16 @@
         <v>635</v>
       </c>
       <c r="C95" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D95" s="3" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E95" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F95" s="2" t="s">
-        <v>633</v>
+        <v>502</v>
       </c>
       <c r="G95" s="2"/>
       <c r="H95" s="2"/>
@@ -20053,16 +21010,16 @@
         <v>635</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D96" s="3" t="s">
-        <v>243</v>
+        <v>253</v>
       </c>
       <c r="E96" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F96" s="2" t="s">
-        <v>496</v>
+        <v>503</v>
       </c>
       <c r="G96" s="2"/>
       <c r="H96" s="2"/>
@@ -20087,16 +21044,16 @@
         <v>635</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D97" s="3" t="s">
-        <v>244</v>
+        <v>255</v>
       </c>
       <c r="E97" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F97" s="2" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="G97" s="2"/>
       <c r="H97" s="2"/>
@@ -20136,60 +21093,41 @@
         <v>635</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D99" s="3" t="s">
-        <v>816</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="D99" s="2"/>
       <c r="E99" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="F99" s="2"/>
+      <c r="F99" s="2" t="s">
+        <v>650</v>
+      </c>
       <c r="G99" s="2"/>
       <c r="H99" s="2"/>
       <c r="I99" s="2" t="s">
         <v>650</v>
       </c>
       <c r="J99" s="2" t="s">
-        <v>486</v>
+        <v>504</v>
       </c>
       <c r="K99" s="2" t="s">
-        <v>688</v>
+        <v>664</v>
       </c>
       <c r="L99" s="2"/>
       <c r="M99" s="2"/>
       <c r="N99" s="2"/>
     </row>
     <row r="100" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A100" t="b">
-        <v>1</v>
-      </c>
-      <c r="B100" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="C100" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D100" s="3" t="s">
-        <v>254</v>
-      </c>
-      <c r="E100" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="F100" s="2" t="s">
-        <v>498</v>
-      </c>
+      <c r="B100" s="2"/>
+      <c r="C100" s="2"/>
+      <c r="D100" s="2"/>
+      <c r="E100" s="2"/>
+      <c r="F100" s="2"/>
       <c r="G100" s="2"/>
       <c r="H100" s="2"/>
-      <c r="I100" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="J100" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="K100" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="I100" s="2"/>
+      <c r="J100" s="2"/>
+      <c r="K100" s="2"/>
       <c r="L100" s="2"/>
       <c r="M100" s="2"/>
       <c r="N100" s="2"/>
@@ -20202,16 +21140,16 @@
         <v>635</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="D101" s="3" t="s">
-        <v>257</v>
+        <v>389</v>
       </c>
       <c r="E101" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F101" s="2" t="s">
-        <v>500</v>
+        <v>389</v>
       </c>
       <c r="G101" s="2"/>
       <c r="H101" s="2"/>
@@ -20219,10 +21157,10 @@
         <v>650</v>
       </c>
       <c r="J101" s="2" t="s">
-        <v>650</v>
+        <v>468</v>
       </c>
       <c r="K101" s="2" t="s">
-        <v>650</v>
+        <v>689</v>
       </c>
       <c r="L101" s="2"/>
       <c r="M101" s="2"/>
@@ -20236,16 +21174,16 @@
         <v>635</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="D102" s="3" t="s">
-        <v>256</v>
+        <v>390</v>
       </c>
       <c r="E102" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F102" s="2" t="s">
-        <v>501</v>
+        <v>390</v>
       </c>
       <c r="G102" s="2"/>
       <c r="H102" s="2"/>
@@ -20270,16 +21208,16 @@
         <v>635</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="D103" s="3" t="s">
-        <v>252</v>
+        <v>391</v>
       </c>
       <c r="E103" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F103" s="2" t="s">
-        <v>502</v>
+        <v>472</v>
       </c>
       <c r="G103" s="2"/>
       <c r="H103" s="2"/>
@@ -20304,16 +21242,16 @@
         <v>635</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="D104" s="3" t="s">
-        <v>253</v>
+        <v>392</v>
       </c>
       <c r="E104" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F104" s="2" t="s">
-        <v>503</v>
+        <v>469</v>
       </c>
       <c r="G104" s="2"/>
       <c r="H104" s="2"/>
@@ -20338,16 +21276,16 @@
         <v>635</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="D105" s="3" t="s">
-        <v>255</v>
+        <v>393</v>
       </c>
       <c r="E105" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F105" s="2" t="s">
-        <v>499</v>
+        <v>470</v>
       </c>
       <c r="G105" s="2"/>
       <c r="H105" s="2"/>
@@ -20365,16 +21303,35 @@
       <c r="N105" s="2"/>
     </row>
     <row r="106" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B106" s="2"/>
-      <c r="C106" s="2"/>
-      <c r="D106" s="3"/>
-      <c r="E106" s="2"/>
-      <c r="F106" s="2"/>
+      <c r="A106" t="b">
+        <v>1</v>
+      </c>
+      <c r="B106" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="C106" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="D106" s="3" t="s">
+        <v>394</v>
+      </c>
+      <c r="E106" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F106" s="2" t="s">
+        <v>471</v>
+      </c>
       <c r="G106" s="2"/>
       <c r="H106" s="2"/>
-      <c r="I106" s="2"/>
-      <c r="J106" s="2"/>
-      <c r="K106" s="2"/>
+      <c r="I106" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="J106" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="K106" s="2" t="s">
+        <v>650</v>
+      </c>
       <c r="L106" s="2"/>
       <c r="M106" s="2"/>
       <c r="N106" s="2"/>
@@ -20387,79 +21344,79 @@
         <v>635</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="D107" s="2"/>
+        <v>41</v>
+      </c>
+      <c r="D107" s="3" t="s">
+        <v>395</v>
+      </c>
       <c r="E107" s="2" t="s">
-        <v>115</v>
+        <v>152</v>
       </c>
       <c r="F107" s="2" t="s">
-        <v>650</v>
+        <v>390</v>
       </c>
       <c r="G107" s="2"/>
-      <c r="H107" s="2" t="s">
-        <v>165</v>
-      </c>
+      <c r="H107" s="2"/>
       <c r="I107" s="2" t="s">
-        <v>581</v>
+        <v>650</v>
       </c>
       <c r="J107" s="2" t="s">
         <v>650</v>
       </c>
       <c r="K107" s="2" t="s">
-        <v>663</v>
-      </c>
-      <c r="L107" s="2" t="s">
-        <v>582</v>
-      </c>
-      <c r="M107" s="2" t="s">
-        <v>155</v>
-      </c>
+        <v>650</v>
+      </c>
+      <c r="L107" s="2"/>
+      <c r="M107" s="2"/>
       <c r="N107" s="2"/>
     </row>
     <row r="108" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A108" t="b">
-        <v>1</v>
-      </c>
-      <c r="B108" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="C108" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="D108" s="2"/>
-      <c r="E108" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="F108" s="2" t="s">
-        <v>650</v>
-      </c>
+      <c r="B108" s="2"/>
+      <c r="C108" s="2"/>
+      <c r="D108" s="3"/>
+      <c r="E108" s="2"/>
+      <c r="F108" s="2"/>
       <c r="G108" s="2"/>
       <c r="H108" s="2"/>
-      <c r="I108" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="J108" s="2" t="s">
-        <v>504</v>
-      </c>
-      <c r="K108" s="2" t="s">
-        <v>664</v>
-      </c>
+      <c r="I108" s="2"/>
+      <c r="J108" s="2"/>
+      <c r="K108" s="2"/>
       <c r="L108" s="2"/>
       <c r="M108" s="2"/>
       <c r="N108" s="2"/>
     </row>
     <row r="109" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B109" s="2"/>
-      <c r="C109" s="2"/>
-      <c r="D109" s="2"/>
-      <c r="E109" s="2"/>
-      <c r="F109" s="2"/>
-      <c r="G109" s="2"/>
+      <c r="A109" t="b">
+        <v>1</v>
+      </c>
+      <c r="B109" s="2" t="s">
+        <v>635</v>
+      </c>
+      <c r="C109" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D109" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="E109" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F109" s="2" t="s">
+        <v>408</v>
+      </c>
+      <c r="G109" s="2" t="s">
+        <v>823</v>
+      </c>
       <c r="H109" s="2"/>
-      <c r="I109" s="2"/>
-      <c r="J109" s="2"/>
-      <c r="K109" s="2"/>
+      <c r="I109" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="J109" s="2" t="s">
+        <v>507</v>
+      </c>
+      <c r="K109" s="2" t="s">
+        <v>690</v>
+      </c>
       <c r="L109" s="2"/>
       <c r="M109" s="2"/>
       <c r="N109" s="2"/>
@@ -20472,16 +21429,16 @@
         <v>635</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D110" s="3" t="s">
-        <v>389</v>
+        <v>409</v>
       </c>
       <c r="E110" s="2" t="s">
         <v>152</v>
       </c>
       <c r="F110" s="2" t="s">
-        <v>389</v>
+        <v>409</v>
       </c>
       <c r="G110" s="2"/>
       <c r="H110" s="2"/>
@@ -20489,10 +21446,10 @@
         <v>650</v>
       </c>
       <c r="J110" s="2" t="s">
-        <v>468</v>
+        <v>650</v>
       </c>
       <c r="K110" s="2" t="s">
-        <v>689</v>
+        <v>650</v>
       </c>
       <c r="L110" s="2"/>
       <c r="M110" s="2"/>
@@ -20505,32 +21462,30 @@
       <c r="B111" s="2" t="s">
         <v>635</v>
       </c>
-      <c r="C111" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D111" s="3" t="s">
-        <v>390</v>
-      </c>
+      <c r="C111" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D111" s="1"/>
       <c r="E111" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="F111" s="2" t="s">
-        <v>390</v>
-      </c>
-      <c r="G111" s="2"/>
-      <c r="H111" s="2"/>
-      <c r="I111" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="J111" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="K111" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="L111" s="2"/>
-      <c r="M111" s="2"/>
-      <c r="N111" s="2"/>
+      <c r="F111" s="1"/>
+      <c r="G111" s="1"/>
+      <c r="H111" s="1"/>
+      <c r="I111" s="1" t="s">
+        <v>650</v>
+      </c>
+      <c r="J111" s="1" t="s">
+        <v>650</v>
+      </c>
+      <c r="K111" s="1" t="s">
+        <v>691</v>
+      </c>
+      <c r="L111" s="1"/>
+      <c r="M111" s="1"/>
+      <c r="N111" s="18" t="s">
+        <v>478</v>
+      </c>
     </row>
     <row r="112" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A112" t="b">
@@ -20540,958 +21495,56 @@
         <v>635</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D112" s="3" t="s">
-        <v>391</v>
-      </c>
+        <v>44</v>
+      </c>
+      <c r="D112" s="2"/>
       <c r="E112" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="F112" s="2" t="s">
-        <v>472</v>
-      </c>
+      <c r="F112" s="2"/>
       <c r="G112" s="2"/>
       <c r="H112" s="2"/>
       <c r="I112" s="2" t="s">
         <v>650</v>
       </c>
       <c r="J112" s="2" t="s">
-        <v>650</v>
+        <v>583</v>
       </c>
       <c r="K112" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="L112" s="2"/>
-      <c r="M112" s="2"/>
-      <c r="N112" s="2"/>
-    </row>
-    <row r="113" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A113" t="b">
-        <v>1</v>
-      </c>
-      <c r="B113" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="C113" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D113" s="3" t="s">
-        <v>392</v>
-      </c>
-      <c r="E113" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="F113" s="2" t="s">
-        <v>469</v>
-      </c>
-      <c r="G113" s="2"/>
-      <c r="H113" s="2"/>
-      <c r="I113" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="J113" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="K113" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="L113" s="2"/>
-      <c r="M113" s="2"/>
-      <c r="N113" s="2"/>
-    </row>
-    <row r="114" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A114" t="b">
-        <v>1</v>
-      </c>
-      <c r="B114" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="C114" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D114" s="3" t="s">
-        <v>393</v>
-      </c>
-      <c r="E114" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="F114" s="2" t="s">
-        <v>470</v>
-      </c>
-      <c r="G114" s="2"/>
-      <c r="H114" s="2"/>
-      <c r="I114" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="J114" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="K114" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="L114" s="2"/>
-      <c r="M114" s="2"/>
-      <c r="N114" s="2"/>
-    </row>
-    <row r="115" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A115" t="b">
-        <v>1</v>
-      </c>
-      <c r="B115" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="C115" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D115" s="3" t="s">
-        <v>394</v>
-      </c>
-      <c r="E115" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="F115" s="2" t="s">
-        <v>471</v>
-      </c>
-      <c r="G115" s="2"/>
-      <c r="H115" s="2"/>
-      <c r="I115" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="J115" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="K115" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="L115" s="2"/>
-      <c r="M115" s="2"/>
-      <c r="N115" s="2"/>
-    </row>
-    <row r="116" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A116" t="b">
-        <v>1</v>
-      </c>
-      <c r="B116" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="C116" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D116" s="3" t="s">
-        <v>395</v>
-      </c>
-      <c r="E116" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="F116" s="2" t="s">
-        <v>390</v>
-      </c>
-      <c r="G116" s="2"/>
-      <c r="H116" s="2"/>
-      <c r="I116" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="J116" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="K116" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="L116" s="2"/>
-      <c r="M116" s="2"/>
-      <c r="N116" s="2"/>
-    </row>
-    <row r="117" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="B117" s="2"/>
-      <c r="C117" s="2"/>
-      <c r="D117" s="3"/>
-      <c r="E117" s="2"/>
-      <c r="F117" s="2"/>
-      <c r="G117" s="2"/>
-      <c r="H117" s="2"/>
-      <c r="I117" s="2"/>
-      <c r="J117" s="2"/>
-      <c r="K117" s="2"/>
-      <c r="L117" s="2"/>
-      <c r="M117" s="2"/>
-      <c r="N117" s="2"/>
-    </row>
-    <row r="118" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A118" t="b">
-        <v>1</v>
-      </c>
-      <c r="B118" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="C118" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D118" s="3" t="s">
-        <v>408</v>
-      </c>
-      <c r="E118" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="F118" s="2" t="s">
-        <v>408</v>
-      </c>
-      <c r="G118" s="2" t="s">
-        <v>823</v>
-      </c>
-      <c r="H118" s="2"/>
-      <c r="I118" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="J118" s="2" t="s">
-        <v>507</v>
-      </c>
-      <c r="K118" s="2" t="s">
-        <v>690</v>
-      </c>
-      <c r="L118" s="2"/>
-      <c r="M118" s="2"/>
-      <c r="N118" s="2"/>
-    </row>
-    <row r="119" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A119" t="b">
-        <v>1</v>
-      </c>
-      <c r="B119" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="C119" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D119" s="3" t="s">
-        <v>409</v>
-      </c>
-      <c r="E119" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="F119" s="2" t="s">
-        <v>409</v>
-      </c>
-      <c r="G119" s="2"/>
-      <c r="H119" s="2"/>
-      <c r="I119" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="J119" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="K119" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="L119" s="2"/>
-      <c r="M119" s="2"/>
-      <c r="N119" s="2"/>
-    </row>
-    <row r="120" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A120" t="b">
-        <v>1</v>
-      </c>
-      <c r="B120" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="C120" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="D120" s="1"/>
-      <c r="E120" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="F120" s="1"/>
-      <c r="G120" s="1"/>
-      <c r="H120" s="1"/>
-      <c r="I120" s="1" t="s">
-        <v>650</v>
-      </c>
-      <c r="J120" s="1" t="s">
-        <v>650</v>
-      </c>
-      <c r="K120" s="1" t="s">
-        <v>691</v>
-      </c>
-      <c r="L120" s="1"/>
-      <c r="M120" s="1"/>
-      <c r="N120" s="18" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="121" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A121" t="b">
-        <v>1</v>
-      </c>
-      <c r="B121" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="C121" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="D121" s="2"/>
-      <c r="E121" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="F121" s="2"/>
-      <c r="G121" s="2"/>
-      <c r="H121" s="2"/>
-      <c r="I121" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="J121" s="2" t="s">
-        <v>583</v>
-      </c>
-      <c r="K121" s="2" t="s">
         <v>692</v>
       </c>
-      <c r="L121" s="2" t="s">
+      <c r="L112" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="M121" s="2" t="s">
+      <c r="M112" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="N121" s="2" t="s">
+      <c r="N112" s="2" t="s">
         <v>693</v>
       </c>
     </row>
-    <row r="122" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A122" t="b">
-        <v>1</v>
-      </c>
-      <c r="B122" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="C122" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="D122" s="2"/>
-      <c r="E122" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="F122" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="G122" s="2"/>
-      <c r="H122" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="I122" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="J122" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="K122" s="2" t="s">
-        <v>665</v>
-      </c>
-      <c r="L122" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="M122" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="N122" s="2"/>
-    </row>
-    <row r="123" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A123" t="b">
-        <v>1</v>
-      </c>
-      <c r="B123" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="C123" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="D123" s="2"/>
-      <c r="E123" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="F123" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="G123" s="2"/>
-      <c r="H123" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="I123" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="J123" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="K123" s="2" t="s">
-        <v>666</v>
-      </c>
-      <c r="L123" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="M123" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="N123" s="2"/>
-    </row>
-    <row r="124" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A124" t="b">
-        <v>1</v>
-      </c>
-      <c r="B124" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="C124" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="D124" s="2"/>
-      <c r="E124" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="F124" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="G124" s="2"/>
-      <c r="H124" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="I124" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="J124" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="K124" s="2" t="s">
-        <v>667</v>
-      </c>
-      <c r="L124" s="2" t="s">
-        <v>174</v>
-      </c>
-      <c r="M124" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="N124" s="2"/>
-    </row>
-    <row r="125" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A125" t="b">
-        <v>1</v>
-      </c>
-      <c r="B125" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="C125" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D125" s="2"/>
-      <c r="E125" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="F125" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="G125" s="2"/>
-      <c r="H125" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="I125" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="J125" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="K125" s="2" t="s">
-        <v>668</v>
-      </c>
-      <c r="L125" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="M125" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="N125" s="2"/>
-    </row>
-    <row r="126" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A126" t="b">
-        <v>1</v>
-      </c>
-      <c r="B126" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="C126" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="D126" s="2"/>
-      <c r="E126" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="F126" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="G126" s="2"/>
-      <c r="H126" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="I126" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="J126" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="K126" s="2" t="s">
-        <v>669</v>
-      </c>
-      <c r="L126" s="2" t="s">
-        <v>169</v>
-      </c>
-      <c r="M126" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="N126" s="2"/>
-    </row>
-    <row r="127" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A127" t="b">
-        <v>1</v>
-      </c>
-      <c r="B127" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="C127" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="D127" s="2"/>
-      <c r="E127" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="F127" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="G127" s="2"/>
-      <c r="H127" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="I127" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="J127" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="K127" s="2" t="s">
-        <v>670</v>
-      </c>
-      <c r="L127" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="M127" s="2" t="s">
-        <v>155</v>
-      </c>
-      <c r="N127" s="2"/>
-    </row>
-    <row r="128" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A128" t="b">
-        <v>1</v>
-      </c>
-      <c r="B128" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="C128" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D128" s="2"/>
-      <c r="E128" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="F128" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="G128" s="2" t="s">
-        <v>824</v>
-      </c>
-      <c r="H128" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="I128" s="1" t="s">
-        <v>642</v>
-      </c>
-      <c r="J128" s="1" t="s">
-        <v>650</v>
-      </c>
-      <c r="K128" s="2" t="s">
-        <v>671</v>
-      </c>
-      <c r="L128" s="1" t="s">
-        <v>646</v>
-      </c>
-      <c r="M128" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="N128" s="2" t="s">
-        <v>721</v>
-      </c>
-    </row>
-    <row r="129" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A129" t="b">
-        <v>1</v>
-      </c>
-      <c r="B129" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="C129" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="D129" s="2"/>
-      <c r="E129" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="F129" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="G129" s="2" t="s">
-        <v>825</v>
-      </c>
-      <c r="H129" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="I129" s="1" t="s">
-        <v>642</v>
-      </c>
-      <c r="J129" s="1" t="s">
-        <v>650</v>
-      </c>
-      <c r="K129" s="2" t="s">
-        <v>672</v>
-      </c>
-      <c r="L129" s="1" t="s">
-        <v>646</v>
-      </c>
-      <c r="M129" s="2" t="s">
-        <v>592</v>
-      </c>
-      <c r="N129" s="1" t="s">
-        <v>593</v>
-      </c>
-    </row>
-    <row r="130" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A130" t="b">
-        <v>1</v>
-      </c>
-      <c r="B130" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="C130" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="D130" s="2"/>
-      <c r="E130" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="F130" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="G130" s="2" t="s">
-        <v>825</v>
-      </c>
-      <c r="H130" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="I130" s="1" t="s">
-        <v>642</v>
-      </c>
-      <c r="J130" s="1" t="s">
-        <v>650</v>
-      </c>
-      <c r="K130" s="2" t="s">
-        <v>673</v>
-      </c>
-      <c r="L130" s="1" t="s">
-        <v>646</v>
-      </c>
-      <c r="M130" s="2" t="s">
-        <v>594</v>
-      </c>
-      <c r="N130" s="1" t="s">
-        <v>593</v>
-      </c>
-    </row>
-    <row r="131" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A131" t="b">
-        <v>1</v>
-      </c>
-      <c r="B131" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="C131" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="D131" s="2"/>
-      <c r="E131" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="F131" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="G131" s="2" t="s">
-        <v>825</v>
-      </c>
-      <c r="H131" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="I131" s="1" t="s">
-        <v>642</v>
-      </c>
-      <c r="J131" s="1" t="s">
-        <v>650</v>
-      </c>
-      <c r="K131" s="2" t="s">
-        <v>674</v>
-      </c>
-      <c r="L131" s="1" t="s">
-        <v>646</v>
-      </c>
-      <c r="M131" s="2" t="s">
-        <v>595</v>
-      </c>
-      <c r="N131" s="1" t="s">
-        <v>593</v>
-      </c>
-    </row>
-    <row r="132" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A132" t="b">
-        <v>1</v>
-      </c>
-      <c r="B132" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="C132" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D132" s="2"/>
-      <c r="E132" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="F132" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="G132" s="2" t="s">
-        <v>826</v>
-      </c>
-      <c r="H132" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="I132" s="2" t="s">
-        <v>599</v>
-      </c>
-      <c r="J132" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="K132" s="2" t="s">
-        <v>675</v>
-      </c>
-      <c r="L132" s="2" t="s">
-        <v>646</v>
-      </c>
-      <c r="M132" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="N132" s="1" t="s">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="133" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A133" t="b">
-        <v>1</v>
-      </c>
-      <c r="B133" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="C133" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="D133" s="2"/>
-      <c r="E133" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="F133" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="G133" s="2"/>
-      <c r="H133" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="I133" s="2" t="s">
-        <v>601</v>
-      </c>
-      <c r="J133" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="K133" s="2" t="s">
-        <v>676</v>
-      </c>
-      <c r="L133" s="2" t="s">
-        <v>164</v>
-      </c>
-      <c r="M133" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="N133" s="1" t="s">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="134" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A134" t="b">
-        <v>1</v>
-      </c>
-      <c r="B134" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="C134" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="D134" s="2"/>
-      <c r="E134" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="F134" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="G134" s="2" t="s">
-        <v>827</v>
-      </c>
-      <c r="H134" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="I134" s="1" t="s">
-        <v>643</v>
-      </c>
-      <c r="J134" s="1" t="s">
-        <v>650</v>
-      </c>
-      <c r="K134" s="2" t="s">
-        <v>677</v>
-      </c>
-      <c r="L134" s="1" t="s">
-        <v>647</v>
-      </c>
-      <c r="M134" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="N134" s="2"/>
-    </row>
-    <row r="135" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A135" t="b">
-        <v>1</v>
-      </c>
-      <c r="B135" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="C135" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="D135" s="2"/>
-      <c r="E135" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="F135" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="G135" s="2" t="s">
-        <v>828</v>
-      </c>
-      <c r="H135" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="I135" s="1" t="s">
-        <v>644</v>
-      </c>
-      <c r="J135" s="1" t="s">
-        <v>650</v>
-      </c>
-      <c r="K135" s="2" t="s">
-        <v>678</v>
-      </c>
-      <c r="L135" s="1" t="s">
-        <v>648</v>
-      </c>
-      <c r="M135" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="N135" s="2"/>
-    </row>
-    <row r="136" spans="1:14" x14ac:dyDescent="0.2">
-      <c r="A136" t="b">
-        <v>1</v>
-      </c>
-      <c r="B136" s="2" t="s">
-        <v>635</v>
-      </c>
-      <c r="C136" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="D136" s="2"/>
-      <c r="E136" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="F136" s="2" t="s">
-        <v>650</v>
-      </c>
-      <c r="G136" s="2" t="s">
-        <v>829</v>
-      </c>
-      <c r="H136" s="2" t="s">
-        <v>165</v>
-      </c>
-      <c r="I136" s="1" t="s">
-        <v>645</v>
-      </c>
-      <c r="J136" s="1" t="s">
-        <v>650</v>
-      </c>
-      <c r="K136" s="2" t="s">
-        <v>679</v>
-      </c>
-      <c r="L136" s="1" t="s">
-        <v>649</v>
-      </c>
-      <c r="M136" s="2" t="s">
-        <v>159</v>
-      </c>
-      <c r="N136" s="2"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:N136" xr:uid="{B39AC7DD-3F73-2C47-925D-21E5B4EBE6FC}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="D99:D105">
-    <sortCondition ref="D99:D105"/>
-  </sortState>
-  <conditionalFormatting sqref="I99:J99">
-    <cfRule type="duplicateValues" dxfId="8" priority="11"/>
+  <conditionalFormatting sqref="I91:J91">
+    <cfRule type="duplicateValues" dxfId="4" priority="4"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K94">
-    <cfRule type="duplicateValues" dxfId="7" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="6" priority="2"/>
+  <conditionalFormatting sqref="K86">
+    <cfRule type="duplicateValues" dxfId="3" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K121:M121">
-    <cfRule type="duplicateValues" dxfId="5" priority="7"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L122 I122:J122 L127:L128">
-    <cfRule type="duplicateValues" dxfId="4" priority="8"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L134">
-    <cfRule type="duplicateValues" dxfId="3" priority="5"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L135">
-    <cfRule type="duplicateValues" dxfId="2" priority="4"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L136">
-    <cfRule type="duplicateValues" dxfId="1" priority="3"/>
+  <conditionalFormatting sqref="K112:M112">
+    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B4CA3B6-4765-0A43-8534-6DA7BF8A336D}">
   <dimension ref="A1:K17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="18.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17" customWidth="1"/>
     <col min="6" max="6" width="12.1640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.83203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="23" customWidth="1"/>
@@ -21711,7 +21764,7 @@
         <v>598</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="19" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:11" ht="17" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" t="b">
         <v>1</v>
       </c>
@@ -21805,7 +21858,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BC10C3F-0C27-5546-8767-E60C7CACEA9D}">
   <dimension ref="A1:J185"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -25552,7 +25605,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{077DB476-AE11-E742-9E3D-7ABA37A90AEF}">
   <dimension ref="A1:G88"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -26432,7 +26485,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6FF6C9F4-4010-9243-98AE-74EEEFFCAC53}">
   <dimension ref="A1:L87"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
Remove cast to string for inhibition_detect and inhibition_adjust in expr code (casting not needed)
</commit_message>
<xml_diff>
--- a/data/mapping_config_files/NWSS-to-ODM-dictionary.xlsx
+++ b/data/mapping_config_files/NWSS-to-ODM-dictionary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martinwellman/Documents/Health/Wastewater/PHES-ODM-MapGenerator/PHES-ODM-MapGenerator/data/mapping_config_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99F92C19-512E-3C41-ACA8-AE862A9ABD13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1F379BF-1E55-BE48-A1A6-2C0B94893D9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1980" yWindow="500" windowWidth="38940" windowHeight="20880" activeTab="2" xr2:uid="{77810E24-F86B-BC44-A0D5-8790E6EC60B4}"/>
   </bookViews>
@@ -2725,13 +2725,6 @@
   </si>
   <si>
     <t>case(
-    ((str(inhibition_detect) == "yes") * (str(inhibition_adjust) == "yes"), "flagFI"),
-    ((str(inhibition_detect) == "yes") * (str(inhibition_adjust) == "no"), "flagAI"),
-    (True, "&lt;ignore&gt;")
-)</t>
-  </si>
-  <si>
-    <t>case(
     (sample_location == "wwtp",
         case((stormwater_input == "yes", "wwtpMuC"),
             (stormwater_input == "no", "wwtpMuS"),
@@ -2747,6 +2740,13 @@
         )
     ),
     (True, "")
+)</t>
+  </si>
+  <si>
+    <t>case(
+    ((inhibition_detect == "yes") * (inhibition_adjust == "yes"), "flagFI"),
+    ((inhibition_detect == "yes") * (inhibition_adjust == "no"), "flagAI"),
+    (True, "&lt;ignore&gt;")
 )</t>
   </si>
 </sst>
@@ -15526,7 +15526,7 @@
       </c>
       <c r="G57" s="27"/>
       <c r="H57" s="50" t="s">
-        <v>882</v>
+        <v>881</v>
       </c>
       <c r="I57" s="27"/>
       <c r="J57" s="27"/>
@@ -17036,7 +17036,7 @@
         <v>799</v>
       </c>
       <c r="K2" s="42" t="s">
-        <v>881</v>
+        <v>882</v>
       </c>
       <c r="L2" s="42" t="s">
         <v>866</v>

</xml_diff>